<commit_message>
graph à partir des data papers recensés
</commit_message>
<xml_diff>
--- a/Data/FairCarboN_Datas_Contacts.xlsx
+++ b/Data/FairCarboN_Datas_Contacts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dutroncj\Documents\Outils\FairCarboN_datas\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCCD8027-95E0-44E7-8AAE-52EB49F89DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D87CDB89-D825-4788-8395-EB9D8789BBAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6316,6 +6316,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:V719"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -6409,7 +6410,7 @@
         <v>1761</v>
       </c>
     </row>
-    <row r="2" spans="1:22" s="2" customFormat="1" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" s="2" customFormat="1" ht="188.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -6463,7 +6464,7 @@
       <c r="U2" s="1"/>
       <c r="V2" s="1"/>
     </row>
-    <row r="3" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -6517,7 +6518,7 @@
       <c r="U3" s="1"/>
       <c r="V3" s="1"/>
     </row>
-    <row r="4" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -6571,7 +6572,7 @@
       <c r="U4" s="1"/>
       <c r="V4" s="1"/>
     </row>
-    <row r="5" spans="1:22" s="2" customFormat="1" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" s="2" customFormat="1" ht="188.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -6625,7 +6626,7 @@
       <c r="U5" s="1"/>
       <c r="V5" s="1"/>
     </row>
-    <row r="6" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -6681,7 +6682,7 @@
       <c r="U6" s="1"/>
       <c r="V6" s="1"/>
     </row>
-    <row r="7" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
@@ -6737,7 +6738,7 @@
       <c r="U7" s="1"/>
       <c r="V7" s="1"/>
     </row>
-    <row r="8" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -6791,7 +6792,7 @@
       <c r="U8" s="1"/>
       <c r="V8" s="1"/>
     </row>
-    <row r="9" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
@@ -6845,7 +6846,7 @@
       <c r="U9" s="1"/>
       <c r="V9" s="1"/>
     </row>
-    <row r="10" spans="1:22" s="2" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" s="2" customFormat="1" ht="159.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
@@ -6899,7 +6900,7 @@
       <c r="U10" s="1"/>
       <c r="V10" s="1"/>
     </row>
-    <row r="11" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>6</v>
       </c>
@@ -6953,7 +6954,7 @@
       <c r="U11" s="1"/>
       <c r="V11" s="1"/>
     </row>
-    <row r="12" spans="1:22" s="2" customFormat="1" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" s="2" customFormat="1" ht="188.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>6</v>
       </c>
@@ -7007,7 +7008,7 @@
       <c r="U12" s="1"/>
       <c r="V12" s="1"/>
     </row>
-    <row r="13" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>6</v>
       </c>
@@ -7061,7 +7062,7 @@
       <c r="U13" s="1"/>
       <c r="V13" s="1"/>
     </row>
-    <row r="14" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>6</v>
       </c>
@@ -7115,7 +7116,7 @@
       <c r="U14" s="1"/>
       <c r="V14" s="1"/>
     </row>
-    <row r="15" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>6</v>
       </c>
@@ -7171,7 +7172,7 @@
       <c r="U15" s="1"/>
       <c r="V15" s="1"/>
     </row>
-    <row r="16" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>6</v>
       </c>
@@ -7225,7 +7226,7 @@
       <c r="U16" s="1"/>
       <c r="V16" s="1"/>
     </row>
-    <row r="17" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>6</v>
       </c>
@@ -7281,7 +7282,7 @@
       <c r="U17" s="1"/>
       <c r="V17" s="1"/>
     </row>
-    <row r="18" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>6</v>
       </c>
@@ -7335,7 +7336,7 @@
       <c r="U18" s="1"/>
       <c r="V18" s="1"/>
     </row>
-    <row r="19" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>6</v>
       </c>
@@ -7389,7 +7390,7 @@
       <c r="U19" s="1"/>
       <c r="V19" s="1"/>
     </row>
-    <row r="20" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>6</v>
       </c>
@@ -7443,7 +7444,7 @@
       <c r="U20" s="1"/>
       <c r="V20" s="1"/>
     </row>
-    <row r="21" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>6</v>
       </c>
@@ -7497,7 +7498,7 @@
       <c r="U21" s="1"/>
       <c r="V21" s="1"/>
     </row>
-    <row r="22" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>6</v>
       </c>
@@ -7551,7 +7552,7 @@
       <c r="U22" s="1"/>
       <c r="V22" s="1"/>
     </row>
-    <row r="23" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>6</v>
       </c>
@@ -7605,7 +7606,7 @@
       <c r="U23" s="1"/>
       <c r="V23" s="1"/>
     </row>
-    <row r="24" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>6</v>
       </c>
@@ -7659,7 +7660,7 @@
       <c r="U24" s="1"/>
       <c r="V24" s="1"/>
     </row>
-    <row r="25" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>6</v>
       </c>
@@ -7715,7 +7716,7 @@
       <c r="U25" s="1"/>
       <c r="V25" s="1"/>
     </row>
-    <row r="26" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>6</v>
       </c>
@@ -7769,7 +7770,7 @@
       <c r="U26" s="1"/>
       <c r="V26" s="1"/>
     </row>
-    <row r="27" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>6</v>
       </c>
@@ -7823,7 +7824,7 @@
       <c r="U27" s="1"/>
       <c r="V27" s="1"/>
     </row>
-    <row r="28" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>6</v>
       </c>
@@ -7877,7 +7878,7 @@
       <c r="U28" s="1"/>
       <c r="V28" s="1"/>
     </row>
-    <row r="29" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>6</v>
       </c>
@@ -7931,7 +7932,7 @@
       <c r="U29" s="1"/>
       <c r="V29" s="1"/>
     </row>
-    <row r="30" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>6</v>
       </c>
@@ -7985,7 +7986,7 @@
       <c r="U30" s="1"/>
       <c r="V30" s="1"/>
     </row>
-    <row r="31" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>6</v>
       </c>
@@ -8039,7 +8040,7 @@
       <c r="U31" s="1"/>
       <c r="V31" s="1"/>
     </row>
-    <row r="32" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>6</v>
       </c>
@@ -8095,7 +8096,7 @@
       <c r="U32" s="1"/>
       <c r="V32" s="1"/>
     </row>
-    <row r="33" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>6</v>
       </c>
@@ -8149,7 +8150,7 @@
       <c r="U33" s="1"/>
       <c r="V33" s="1"/>
     </row>
-    <row r="34" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>6</v>
       </c>
@@ -8203,7 +8204,7 @@
       <c r="U34" s="1"/>
       <c r="V34" s="1"/>
     </row>
-    <row r="35" spans="1:22" s="2" customFormat="1" ht="232" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:22" s="2" customFormat="1" ht="232" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>6</v>
       </c>
@@ -8259,7 +8260,7 @@
       <c r="U35" s="1"/>
       <c r="V35" s="1"/>
     </row>
-    <row r="36" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>6</v>
       </c>
@@ -8313,7 +8314,7 @@
       <c r="U36" s="1"/>
       <c r="V36" s="1"/>
     </row>
-    <row r="37" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>6</v>
       </c>
@@ -8367,7 +8368,7 @@
       <c r="U37" s="1"/>
       <c r="V37" s="1"/>
     </row>
-    <row r="38" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>6</v>
       </c>
@@ -8421,7 +8422,7 @@
       <c r="U38" s="1"/>
       <c r="V38" s="1"/>
     </row>
-    <row r="39" spans="1:22" s="2" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:22" s="2" customFormat="1" ht="159.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>6</v>
       </c>
@@ -8475,7 +8476,7 @@
       <c r="U39" s="1"/>
       <c r="V39" s="1"/>
     </row>
-    <row r="40" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>6</v>
       </c>
@@ -8529,7 +8530,7 @@
       <c r="U40" s="1"/>
       <c r="V40" s="1"/>
     </row>
-    <row r="41" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>6</v>
       </c>
@@ -8583,7 +8584,7 @@
       <c r="U41" s="1"/>
       <c r="V41" s="1"/>
     </row>
-    <row r="42" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>6</v>
       </c>
@@ -8637,7 +8638,7 @@
       <c r="U42" s="1"/>
       <c r="V42" s="1"/>
     </row>
-    <row r="43" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>6</v>
       </c>
@@ -8691,7 +8692,7 @@
       <c r="U43" s="1"/>
       <c r="V43" s="1"/>
     </row>
-    <row r="44" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>6</v>
       </c>
@@ -8745,7 +8746,7 @@
       <c r="U44" s="1"/>
       <c r="V44" s="1"/>
     </row>
-    <row r="45" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>6</v>
       </c>
@@ -8799,7 +8800,7 @@
       <c r="U45" s="1"/>
       <c r="V45" s="1"/>
     </row>
-    <row r="46" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>6</v>
       </c>
@@ -8853,7 +8854,7 @@
       <c r="U46" s="1"/>
       <c r="V46" s="1"/>
     </row>
-    <row r="47" spans="1:22" s="2" customFormat="1" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:22" s="2" customFormat="1" ht="275.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>6</v>
       </c>
@@ -8911,7 +8912,7 @@
       <c r="U47" s="1"/>
       <c r="V47" s="1"/>
     </row>
-    <row r="48" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>6</v>
       </c>
@@ -8965,7 +8966,7 @@
       <c r="U48" s="1"/>
       <c r="V48" s="1"/>
     </row>
-    <row r="49" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>6</v>
       </c>
@@ -9021,7 +9022,7 @@
       <c r="U49" s="1"/>
       <c r="V49" s="1"/>
     </row>
-    <row r="50" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>6</v>
       </c>
@@ -9075,7 +9076,7 @@
       <c r="U50" s="1"/>
       <c r="V50" s="1"/>
     </row>
-    <row r="51" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>6</v>
       </c>
@@ -9129,7 +9130,7 @@
       <c r="U51" s="1"/>
       <c r="V51" s="1"/>
     </row>
-    <row r="52" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>6</v>
       </c>
@@ -9183,7 +9184,7 @@
       <c r="U52" s="1"/>
       <c r="V52" s="1"/>
     </row>
-    <row r="53" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>6</v>
       </c>
@@ -9237,7 +9238,7 @@
       <c r="U53" s="1"/>
       <c r="V53" s="1"/>
     </row>
-    <row r="54" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>6</v>
       </c>
@@ -9291,7 +9292,7 @@
       <c r="U54" s="1"/>
       <c r="V54" s="1"/>
     </row>
-    <row r="55" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>6</v>
       </c>
@@ -9345,7 +9346,7 @@
       <c r="U55" s="1"/>
       <c r="V55" s="1"/>
     </row>
-    <row r="56" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>6</v>
       </c>
@@ -9399,7 +9400,7 @@
       <c r="U56" s="1"/>
       <c r="V56" s="1"/>
     </row>
-    <row r="57" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>6</v>
       </c>
@@ -9453,7 +9454,7 @@
       <c r="U57" s="1"/>
       <c r="V57" s="1"/>
     </row>
-    <row r="58" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>6</v>
       </c>
@@ -9507,7 +9508,7 @@
       <c r="U58" s="1"/>
       <c r="V58" s="1"/>
     </row>
-    <row r="59" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>6</v>
       </c>
@@ -9563,7 +9564,7 @@
       <c r="U59" s="1"/>
       <c r="V59" s="1"/>
     </row>
-    <row r="60" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>6</v>
       </c>
@@ -9619,7 +9620,7 @@
       <c r="U60" s="1"/>
       <c r="V60" s="1"/>
     </row>
-    <row r="61" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>6</v>
       </c>
@@ -9675,7 +9676,7 @@
       <c r="U61" s="1"/>
       <c r="V61" s="1"/>
     </row>
-    <row r="62" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>6</v>
       </c>
@@ -9731,7 +9732,7 @@
       <c r="U62" s="1"/>
       <c r="V62" s="1"/>
     </row>
-    <row r="63" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>6</v>
       </c>
@@ -9785,7 +9786,7 @@
       <c r="U63" s="1"/>
       <c r="V63" s="1"/>
     </row>
-    <row r="64" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>6</v>
       </c>
@@ -9841,7 +9842,7 @@
       <c r="U64" s="1"/>
       <c r="V64" s="1"/>
     </row>
-    <row r="65" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>6</v>
       </c>
@@ -9939,7 +9940,7 @@
         <v>1</v>
       </c>
       <c r="O66" s="52">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="P66" s="1" t="s">
         <v>1800</v>
@@ -9953,7 +9954,7 @@
       <c r="U66" s="1"/>
       <c r="V66" s="1"/>
     </row>
-    <row r="67" spans="1:22" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:22" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>6</v>
       </c>
@@ -10007,7 +10008,7 @@
       <c r="U67" s="1"/>
       <c r="V67" s="1"/>
     </row>
-    <row r="68" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>6</v>
       </c>
@@ -10063,7 +10064,7 @@
       <c r="U68" s="1"/>
       <c r="V68" s="1"/>
     </row>
-    <row r="69" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>6</v>
       </c>
@@ -10117,7 +10118,7 @@
       <c r="U69" s="1"/>
       <c r="V69" s="1"/>
     </row>
-    <row r="70" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>6</v>
       </c>
@@ -10171,7 +10172,7 @@
       <c r="U70" s="1"/>
       <c r="V70" s="1"/>
     </row>
-    <row r="71" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>6</v>
       </c>
@@ -10225,7 +10226,7 @@
       <c r="U71" s="1"/>
       <c r="V71" s="1"/>
     </row>
-    <row r="72" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>6</v>
       </c>
@@ -10279,7 +10280,7 @@
       <c r="U72" s="1"/>
       <c r="V72" s="1"/>
     </row>
-    <row r="73" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>6</v>
       </c>
@@ -10333,7 +10334,7 @@
       <c r="U73" s="1"/>
       <c r="V73" s="1"/>
     </row>
-    <row r="74" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>6</v>
       </c>
@@ -10387,7 +10388,7 @@
       <c r="U74" s="1"/>
       <c r="V74" s="1"/>
     </row>
-    <row r="75" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>6</v>
       </c>
@@ -10441,7 +10442,7 @@
       <c r="U75" s="1"/>
       <c r="V75" s="1"/>
     </row>
-    <row r="76" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>6</v>
       </c>
@@ -10495,7 +10496,7 @@
       <c r="U76" s="1"/>
       <c r="V76" s="1"/>
     </row>
-    <row r="77" spans="1:22" s="2" customFormat="1" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:22" s="2" customFormat="1" ht="27.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>6</v>
       </c>
@@ -10551,7 +10552,7 @@
       <c r="U77" s="1"/>
       <c r="V77" s="1"/>
     </row>
-    <row r="78" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>6</v>
       </c>
@@ -10605,7 +10606,7 @@
       <c r="U78" s="1"/>
       <c r="V78" s="1"/>
     </row>
-    <row r="79" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>6</v>
       </c>
@@ -10659,7 +10660,7 @@
       <c r="U79" s="1"/>
       <c r="V79" s="1"/>
     </row>
-    <row r="80" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>6</v>
       </c>
@@ -10713,7 +10714,7 @@
       <c r="U80" s="1"/>
       <c r="V80" s="1"/>
     </row>
-    <row r="81" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>6</v>
       </c>
@@ -10769,7 +10770,7 @@
       <c r="U81" s="1"/>
       <c r="V81" s="1"/>
     </row>
-    <row r="82" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>6</v>
       </c>
@@ -10823,7 +10824,7 @@
       <c r="U82" s="1"/>
       <c r="V82" s="1"/>
     </row>
-    <row r="83" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>6</v>
       </c>
@@ -10879,7 +10880,7 @@
       <c r="U83" s="1"/>
       <c r="V83" s="1"/>
     </row>
-    <row r="84" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>6</v>
       </c>
@@ -10933,7 +10934,7 @@
       <c r="U84" s="1"/>
       <c r="V84" s="1"/>
     </row>
-    <row r="85" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>6</v>
       </c>
@@ -10989,7 +10990,7 @@
       <c r="U85" s="1"/>
       <c r="V85" s="1"/>
     </row>
-    <row r="86" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>6</v>
       </c>
@@ -11045,7 +11046,7 @@
       <c r="U86" s="1"/>
       <c r="V86" s="1"/>
     </row>
-    <row r="87" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>6</v>
       </c>
@@ -11099,7 +11100,7 @@
       <c r="U87" s="1"/>
       <c r="V87" s="1"/>
     </row>
-    <row r="88" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>6</v>
       </c>
@@ -11153,7 +11154,7 @@
       <c r="U88" s="1"/>
       <c r="V88" s="1"/>
     </row>
-    <row r="89" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>6</v>
       </c>
@@ -11205,7 +11206,7 @@
       <c r="U89" s="1"/>
       <c r="V89" s="1"/>
     </row>
-    <row r="90" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>6</v>
       </c>
@@ -11261,7 +11262,7 @@
       <c r="U90" s="1"/>
       <c r="V90" s="1"/>
     </row>
-    <row r="91" spans="1:22" s="2" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:22" s="2" customFormat="1" ht="159.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>6</v>
       </c>
@@ -11315,7 +11316,7 @@
       <c r="U91" s="1"/>
       <c r="V91" s="1"/>
     </row>
-    <row r="92" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>6</v>
       </c>
@@ -11369,7 +11370,7 @@
       <c r="U92" s="1"/>
       <c r="V92" s="1"/>
     </row>
-    <row r="93" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
         <v>6</v>
       </c>
@@ -11423,7 +11424,7 @@
       <c r="U93" s="1"/>
       <c r="V93" s="1"/>
     </row>
-    <row r="94" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
         <v>6</v>
       </c>
@@ -11477,7 +11478,7 @@
       <c r="U94" s="1"/>
       <c r="V94" s="1"/>
     </row>
-    <row r="95" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
         <v>6</v>
       </c>
@@ -11531,7 +11532,7 @@
       <c r="U95" s="1"/>
       <c r="V95" s="1"/>
     </row>
-    <row r="96" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>6</v>
       </c>
@@ -11585,7 +11586,7 @@
       <c r="U96" s="1"/>
       <c r="V96" s="1"/>
     </row>
-    <row r="97" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>6</v>
       </c>
@@ -11639,7 +11640,7 @@
       <c r="U97" s="1"/>
       <c r="V97" s="1"/>
     </row>
-    <row r="98" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>6</v>
       </c>
@@ -11693,7 +11694,7 @@
       <c r="U98" s="1"/>
       <c r="V98" s="1"/>
     </row>
-    <row r="99" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>6</v>
       </c>
@@ -11747,7 +11748,7 @@
       <c r="U99" s="1"/>
       <c r="V99" s="1"/>
     </row>
-    <row r="100" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
         <v>6</v>
       </c>
@@ -11801,7 +11802,7 @@
       <c r="U100" s="1"/>
       <c r="V100" s="1"/>
     </row>
-    <row r="101" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>6</v>
       </c>
@@ -11853,7 +11854,7 @@
       <c r="U101" s="1"/>
       <c r="V101" s="1"/>
     </row>
-    <row r="102" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
         <v>6</v>
       </c>
@@ -11909,7 +11910,7 @@
       <c r="U102" s="1"/>
       <c r="V102" s="1"/>
     </row>
-    <row r="103" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>6</v>
       </c>
@@ -11963,7 +11964,7 @@
       <c r="U103" s="1"/>
       <c r="V103" s="1"/>
     </row>
-    <row r="104" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
         <v>6</v>
       </c>
@@ -12015,7 +12016,7 @@
       <c r="U104" s="1"/>
       <c r="V104" s="1"/>
     </row>
-    <row r="105" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>6</v>
       </c>
@@ -12071,7 +12072,7 @@
       <c r="U105" s="1"/>
       <c r="V105" s="1"/>
     </row>
-    <row r="106" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>6</v>
       </c>
@@ -12125,7 +12126,7 @@
       <c r="U106" s="1"/>
       <c r="V106" s="1"/>
     </row>
-    <row r="107" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
         <v>6</v>
       </c>
@@ -12179,7 +12180,7 @@
       <c r="U107" s="1"/>
       <c r="V107" s="1"/>
     </row>
-    <row r="108" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
         <v>6</v>
       </c>
@@ -12233,7 +12234,7 @@
       <c r="U108" s="1"/>
       <c r="V108" s="1"/>
     </row>
-    <row r="109" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
         <v>6</v>
       </c>
@@ -12285,7 +12286,7 @@
       <c r="U109" s="1"/>
       <c r="V109" s="1"/>
     </row>
-    <row r="110" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
         <v>6</v>
       </c>
@@ -12339,7 +12340,7 @@
       <c r="U110" s="1"/>
       <c r="V110" s="1"/>
     </row>
-    <row r="111" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>6</v>
       </c>
@@ -12395,7 +12396,7 @@
       <c r="U111" s="1"/>
       <c r="V111" s="1"/>
     </row>
-    <row r="112" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>6</v>
       </c>
@@ -12449,7 +12450,7 @@
       <c r="U112" s="1"/>
       <c r="V112" s="1"/>
     </row>
-    <row r="113" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
         <v>6</v>
       </c>
@@ -12503,7 +12504,7 @@
       <c r="U113" s="1"/>
       <c r="V113" s="1"/>
     </row>
-    <row r="114" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
         <v>6</v>
       </c>
@@ -12557,7 +12558,7 @@
       <c r="U114" s="1"/>
       <c r="V114" s="1"/>
     </row>
-    <row r="115" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" s="1" t="s">
         <v>6</v>
       </c>
@@ -12611,7 +12612,7 @@
       <c r="U115" s="1"/>
       <c r="V115" s="1"/>
     </row>
-    <row r="116" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
         <v>6</v>
       </c>
@@ -12665,7 +12666,7 @@
       <c r="U116" s="1"/>
       <c r="V116" s="1"/>
     </row>
-    <row r="117" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
         <v>6</v>
       </c>
@@ -12719,7 +12720,7 @@
       <c r="U117" s="1"/>
       <c r="V117" s="1"/>
     </row>
-    <row r="118" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
         <v>6</v>
       </c>
@@ -12773,7 +12774,7 @@
       <c r="U118" s="1"/>
       <c r="V118" s="1"/>
     </row>
-    <row r="119" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
         <v>6</v>
       </c>
@@ -12827,7 +12828,7 @@
       <c r="U119" s="1"/>
       <c r="V119" s="1"/>
     </row>
-    <row r="120" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
         <v>6</v>
       </c>
@@ -12881,7 +12882,7 @@
       <c r="U120" s="1"/>
       <c r="V120" s="1"/>
     </row>
-    <row r="121" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
         <v>6</v>
       </c>
@@ -12937,7 +12938,7 @@
       <c r="U121" s="1"/>
       <c r="V121" s="1"/>
     </row>
-    <row r="122" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" s="1" t="s">
         <v>6</v>
       </c>
@@ -12991,7 +12992,7 @@
       <c r="U122" s="1"/>
       <c r="V122" s="1"/>
     </row>
-    <row r="123" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
         <v>6</v>
       </c>
@@ -13045,7 +13046,7 @@
       <c r="U123" s="1"/>
       <c r="V123" s="1"/>
     </row>
-    <row r="124" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
         <v>6</v>
       </c>
@@ -13099,7 +13100,7 @@
       <c r="U124" s="1"/>
       <c r="V124" s="1"/>
     </row>
-    <row r="125" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
         <v>6</v>
       </c>
@@ -13153,7 +13154,7 @@
       <c r="U125" s="1"/>
       <c r="V125" s="1"/>
     </row>
-    <row r="126" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
         <v>6</v>
       </c>
@@ -13207,7 +13208,7 @@
       <c r="U126" s="1"/>
       <c r="V126" s="1"/>
     </row>
-    <row r="127" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
         <v>6</v>
       </c>
@@ -13261,7 +13262,7 @@
       <c r="U127" s="1"/>
       <c r="V127" s="1"/>
     </row>
-    <row r="128" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" s="1" t="s">
         <v>6</v>
       </c>
@@ -13315,7 +13316,7 @@
       <c r="U128" s="1"/>
       <c r="V128" s="1"/>
     </row>
-    <row r="129" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" s="1" t="s">
         <v>6</v>
       </c>
@@ -13369,7 +13370,7 @@
       <c r="U129" s="1"/>
       <c r="V129" s="1"/>
     </row>
-    <row r="130" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130" s="1" t="s">
         <v>6</v>
       </c>
@@ -13423,7 +13424,7 @@
       <c r="U130" s="1"/>
       <c r="V130" s="1"/>
     </row>
-    <row r="131" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" s="1" t="s">
         <v>6</v>
       </c>
@@ -13477,7 +13478,7 @@
       <c r="U131" s="1"/>
       <c r="V131" s="1"/>
     </row>
-    <row r="132" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132" s="1" t="s">
         <v>6</v>
       </c>
@@ -13531,7 +13532,7 @@
       <c r="U132" s="1"/>
       <c r="V132" s="1"/>
     </row>
-    <row r="133" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" s="1" t="s">
         <v>6</v>
       </c>
@@ -13585,7 +13586,7 @@
       <c r="U133" s="1"/>
       <c r="V133" s="1"/>
     </row>
-    <row r="134" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A134" s="1" t="s">
         <v>6</v>
       </c>
@@ -13639,7 +13640,7 @@
       <c r="U134" s="1"/>
       <c r="V134" s="1"/>
     </row>
-    <row r="135" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
         <v>6</v>
       </c>
@@ -13693,7 +13694,7 @@
       <c r="U135" s="1"/>
       <c r="V135" s="1"/>
     </row>
-    <row r="136" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" s="1" t="s">
         <v>6</v>
       </c>
@@ -13747,7 +13748,7 @@
       <c r="U136" s="1"/>
       <c r="V136" s="1"/>
     </row>
-    <row r="137" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
         <v>6</v>
       </c>
@@ -13801,7 +13802,7 @@
       <c r="U137" s="1"/>
       <c r="V137" s="1"/>
     </row>
-    <row r="138" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
         <v>6</v>
       </c>
@@ -13855,7 +13856,7 @@
       <c r="U138" s="1"/>
       <c r="V138" s="1"/>
     </row>
-    <row r="139" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A139" s="1" t="s">
         <v>6</v>
       </c>
@@ -13909,7 +13910,7 @@
       <c r="U139" s="1"/>
       <c r="V139" s="1"/>
     </row>
-    <row r="140" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140" s="1" t="s">
         <v>6</v>
       </c>
@@ -13965,7 +13966,7 @@
       <c r="U140" s="1"/>
       <c r="V140" s="1"/>
     </row>
-    <row r="141" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141" s="1" t="s">
         <v>6</v>
       </c>
@@ -14019,7 +14020,7 @@
       <c r="U141" s="1"/>
       <c r="V141" s="1"/>
     </row>
-    <row r="142" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A142" s="1" t="s">
         <v>6</v>
       </c>
@@ -14073,7 +14074,7 @@
       <c r="U142" s="1"/>
       <c r="V142" s="1"/>
     </row>
-    <row r="143" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143" s="1" t="s">
         <v>6</v>
       </c>
@@ -14127,7 +14128,7 @@
       <c r="U143" s="1"/>
       <c r="V143" s="1"/>
     </row>
-    <row r="144" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144" s="1" t="s">
         <v>6</v>
       </c>
@@ -14183,7 +14184,7 @@
       <c r="U144" s="1"/>
       <c r="V144" s="1"/>
     </row>
-    <row r="145" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
         <v>6</v>
       </c>
@@ -14237,7 +14238,7 @@
       <c r="U145" s="1"/>
       <c r="V145" s="1"/>
     </row>
-    <row r="146" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" s="1" t="s">
         <v>6</v>
       </c>
@@ -14291,7 +14292,7 @@
       <c r="U146" s="1"/>
       <c r="V146" s="1"/>
     </row>
-    <row r="147" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
       <c r="A147" s="1" t="s">
         <v>6</v>
       </c>
@@ -14347,7 +14348,7 @@
       <c r="U147" s="1"/>
       <c r="V147" s="1"/>
     </row>
-    <row r="148" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A148" s="1" t="s">
         <v>6</v>
       </c>
@@ -14401,7 +14402,7 @@
       <c r="U148" s="1"/>
       <c r="V148" s="1"/>
     </row>
-    <row r="149" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149" s="1" t="s">
         <v>6</v>
       </c>
@@ -14455,7 +14456,7 @@
       <c r="U149" s="1"/>
       <c r="V149" s="1"/>
     </row>
-    <row r="150" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A150" s="1" t="s">
         <v>6</v>
       </c>
@@ -14509,7 +14510,7 @@
       <c r="U150" s="1"/>
       <c r="V150" s="1"/>
     </row>
-    <row r="151" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A151" s="1" t="s">
         <v>6</v>
       </c>
@@ -14563,7 +14564,7 @@
       <c r="U151" s="1"/>
       <c r="V151" s="1"/>
     </row>
-    <row r="152" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A152" s="1" t="s">
         <v>6</v>
       </c>
@@ -14617,7 +14618,7 @@
       <c r="U152" s="1"/>
       <c r="V152" s="1"/>
     </row>
-    <row r="153" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A153" s="1" t="s">
         <v>6</v>
       </c>
@@ -14671,7 +14672,7 @@
       <c r="U153" s="1"/>
       <c r="V153" s="1"/>
     </row>
-    <row r="154" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A154" s="1" t="s">
         <v>6</v>
       </c>
@@ -14725,7 +14726,7 @@
       <c r="U154" s="1"/>
       <c r="V154" s="1"/>
     </row>
-    <row r="155" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A155" s="1" t="s">
         <v>6</v>
       </c>
@@ -14779,7 +14780,7 @@
       <c r="U155" s="1"/>
       <c r="V155" s="1"/>
     </row>
-    <row r="156" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A156" s="1" t="s">
         <v>6</v>
       </c>
@@ -14833,7 +14834,7 @@
       <c r="U156" s="1"/>
       <c r="V156" s="1"/>
     </row>
-    <row r="157" spans="1:22" s="2" customFormat="1" ht="65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:22" s="2" customFormat="1" ht="65" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A157" s="1" t="s">
         <v>6</v>
       </c>
@@ -14897,7 +14898,7 @@
         <v>1764</v>
       </c>
     </row>
-    <row r="158" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A158" s="1" t="s">
         <v>6</v>
       </c>
@@ -14953,7 +14954,7 @@
       <c r="U158" s="1"/>
       <c r="V158" s="1"/>
     </row>
-    <row r="159" spans="1:22" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:22" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A159" s="1" t="s">
         <v>6</v>
       </c>
@@ -15009,7 +15010,7 @@
       <c r="U159" s="1"/>
       <c r="V159" s="1"/>
     </row>
-    <row r="160" spans="1:22" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:22" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A160" s="1" t="s">
         <v>6</v>
       </c>
@@ -15065,7 +15066,7 @@
       <c r="U160" s="1"/>
       <c r="V160" s="1"/>
     </row>
-    <row r="161" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
       <c r="A161" s="1" t="s">
         <v>6</v>
       </c>
@@ -15121,7 +15122,7 @@
       <c r="U161" s="1"/>
       <c r="V161" s="1"/>
     </row>
-    <row r="162" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
       <c r="A162" s="1" t="s">
         <v>6</v>
       </c>
@@ -15179,7 +15180,7 @@
       <c r="U162" s="1"/>
       <c r="V162" s="1"/>
     </row>
-    <row r="163" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A163" s="1" t="s">
         <v>6</v>
       </c>
@@ -15235,7 +15236,7 @@
       <c r="U163" s="1"/>
       <c r="V163" s="1"/>
     </row>
-    <row r="164" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A164" s="1" t="s">
         <v>6</v>
       </c>
@@ -15291,7 +15292,7 @@
       <c r="U164" s="1"/>
       <c r="V164" s="1"/>
     </row>
-    <row r="165" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A165" s="1" t="s">
         <v>6</v>
       </c>
@@ -15347,7 +15348,7 @@
       <c r="U165" s="1"/>
       <c r="V165" s="1"/>
     </row>
-    <row r="166" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A166" s="1" t="s">
         <v>6</v>
       </c>
@@ -15403,7 +15404,7 @@
       <c r="U166" s="1"/>
       <c r="V166" s="1"/>
     </row>
-    <row r="167" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
       <c r="A167" s="1" t="s">
         <v>6</v>
       </c>
@@ -15461,7 +15462,7 @@
       <c r="U167" s="1"/>
       <c r="V167" s="1"/>
     </row>
-    <row r="168" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
       <c r="A168" s="1" t="s">
         <v>6</v>
       </c>
@@ -15521,7 +15522,7 @@
       <c r="U168" s="1"/>
       <c r="V168" s="1"/>
     </row>
-    <row r="169" spans="1:22" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:22" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A169" s="1" t="s">
         <v>6</v>
       </c>
@@ -15577,7 +15578,7 @@
       <c r="U169" s="1"/>
       <c r="V169" s="1"/>
     </row>
-    <row r="170" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A170" s="1" t="s">
         <v>6</v>
       </c>
@@ -15633,7 +15634,7 @@
       <c r="U170" s="1"/>
       <c r="V170" s="1"/>
     </row>
-    <row r="171" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
       <c r="A171" s="1" t="s">
         <v>6</v>
       </c>
@@ -15689,7 +15690,7 @@
       <c r="U171" s="1"/>
       <c r="V171" s="1"/>
     </row>
-    <row r="172" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A172" s="1" t="s">
         <v>6</v>
       </c>
@@ -15745,7 +15746,7 @@
       <c r="U172" s="1"/>
       <c r="V172" s="1"/>
     </row>
-    <row r="173" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A173" s="1" t="s">
         <v>6</v>
       </c>
@@ -15799,7 +15800,7 @@
       <c r="U173" s="1"/>
       <c r="V173" s="1"/>
     </row>
-    <row r="174" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A174" s="1" t="s">
         <v>6</v>
       </c>
@@ -15853,7 +15854,7 @@
       <c r="U174" s="1"/>
       <c r="V174" s="1"/>
     </row>
-    <row r="175" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A175" s="1" t="s">
         <v>6</v>
       </c>
@@ -15907,7 +15908,7 @@
       <c r="U175" s="1"/>
       <c r="V175" s="1"/>
     </row>
-    <row r="176" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A176" s="1" t="s">
         <v>6</v>
       </c>
@@ -15961,7 +15962,7 @@
       <c r="U176" s="1"/>
       <c r="V176" s="1"/>
     </row>
-    <row r="177" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A177" s="1" t="s">
         <v>6</v>
       </c>
@@ -16015,7 +16016,7 @@
       <c r="U177" s="1"/>
       <c r="V177" s="1"/>
     </row>
-    <row r="178" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
       <c r="A178" s="1" t="s">
         <v>6</v>
       </c>
@@ -16069,7 +16070,7 @@
       <c r="U178" s="1"/>
       <c r="V178" s="1"/>
     </row>
-    <row r="179" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
       <c r="A179" s="1" t="s">
         <v>6</v>
       </c>
@@ -16123,7 +16124,7 @@
       <c r="U179" s="1"/>
       <c r="V179" s="1"/>
     </row>
-    <row r="180" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A180" s="1" t="s">
         <v>6</v>
       </c>
@@ -16177,7 +16178,7 @@
       <c r="U180" s="1"/>
       <c r="V180" s="1"/>
     </row>
-    <row r="181" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
       <c r="A181" s="1" t="s">
         <v>6</v>
       </c>
@@ -16233,7 +16234,7 @@
       <c r="U181" s="1"/>
       <c r="V181" s="1"/>
     </row>
-    <row r="182" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A182" s="1" t="s">
         <v>6</v>
       </c>
@@ -16287,7 +16288,7 @@
       <c r="U182" s="1"/>
       <c r="V182" s="1"/>
     </row>
-    <row r="183" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A183" s="1" t="s">
         <v>6</v>
       </c>
@@ -16341,7 +16342,7 @@
       <c r="U183" s="1"/>
       <c r="V183" s="1"/>
     </row>
-    <row r="184" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A184" s="1" t="s">
         <v>6</v>
       </c>
@@ -16395,7 +16396,7 @@
       <c r="U184" s="1"/>
       <c r="V184" s="1"/>
     </row>
-    <row r="185" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A185" s="1" t="s">
         <v>6</v>
       </c>
@@ -16449,7 +16450,7 @@
       <c r="U185" s="1"/>
       <c r="V185" s="1"/>
     </row>
-    <row r="186" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A186" s="1" t="s">
         <v>6</v>
       </c>
@@ -16505,7 +16506,7 @@
       <c r="U186" s="1"/>
       <c r="V186" s="1"/>
     </row>
-    <row r="187" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A187" s="1" t="s">
         <v>6</v>
       </c>
@@ -16559,7 +16560,7 @@
       <c r="U187" s="1"/>
       <c r="V187" s="1"/>
     </row>
-    <row r="188" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A188" s="1" t="s">
         <v>6</v>
       </c>
@@ -16613,7 +16614,7 @@
       <c r="U188" s="1"/>
       <c r="V188" s="1"/>
     </row>
-    <row r="189" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A189" s="1" t="s">
         <v>6</v>
       </c>
@@ -16667,7 +16668,7 @@
       <c r="U189" s="1"/>
       <c r="V189" s="1"/>
     </row>
-    <row r="190" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A190" s="1" t="s">
         <v>6</v>
       </c>
@@ -16721,7 +16722,7 @@
       <c r="U190" s="1"/>
       <c r="V190" s="1"/>
     </row>
-    <row r="191" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A191" s="1" t="s">
         <v>6</v>
       </c>
@@ -16775,7 +16776,7 @@
       <c r="U191" s="1"/>
       <c r="V191" s="1"/>
     </row>
-    <row r="192" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A192" s="1" t="s">
         <v>6</v>
       </c>
@@ -16829,7 +16830,7 @@
       <c r="U192" s="1"/>
       <c r="V192" s="1"/>
     </row>
-    <row r="193" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A193" s="1" t="s">
         <v>6</v>
       </c>
@@ -16883,7 +16884,7 @@
       <c r="U193" s="1"/>
       <c r="V193" s="1"/>
     </row>
-    <row r="194" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A194" s="1" t="s">
         <v>6</v>
       </c>
@@ -16937,7 +16938,7 @@
       <c r="U194" s="1"/>
       <c r="V194" s="1"/>
     </row>
-    <row r="195" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A195" s="1" t="s">
         <v>6</v>
       </c>
@@ -16991,7 +16992,7 @@
       <c r="U195" s="1"/>
       <c r="V195" s="1"/>
     </row>
-    <row r="196" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A196" s="1" t="s">
         <v>6</v>
       </c>
@@ -17045,7 +17046,7 @@
       <c r="U196" s="1"/>
       <c r="V196" s="1"/>
     </row>
-    <row r="197" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A197" s="1" t="s">
         <v>6</v>
       </c>
@@ -17099,7 +17100,7 @@
       <c r="U197" s="1"/>
       <c r="V197" s="1"/>
     </row>
-    <row r="198" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A198" s="1" t="s">
         <v>6</v>
       </c>
@@ -17153,7 +17154,7 @@
       <c r="U198" s="1"/>
       <c r="V198" s="1"/>
     </row>
-    <row r="199" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A199" s="1" t="s">
         <v>6</v>
       </c>
@@ -17207,7 +17208,7 @@
       <c r="U199" s="1"/>
       <c r="V199" s="1"/>
     </row>
-    <row r="200" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A200" s="1" t="s">
         <v>6</v>
       </c>
@@ -17261,7 +17262,7 @@
       <c r="U200" s="1"/>
       <c r="V200" s="1"/>
     </row>
-    <row r="201" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A201" s="1" t="s">
         <v>6</v>
       </c>
@@ -17315,7 +17316,7 @@
       <c r="U201" s="1"/>
       <c r="V201" s="1"/>
     </row>
-    <row r="202" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A202" s="1" t="s">
         <v>6</v>
       </c>
@@ -17369,7 +17370,7 @@
       <c r="U202" s="1"/>
       <c r="V202" s="1"/>
     </row>
-    <row r="203" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A203" s="1" t="s">
         <v>6</v>
       </c>
@@ -17423,7 +17424,7 @@
       <c r="U203" s="1"/>
       <c r="V203" s="1"/>
     </row>
-    <row r="204" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A204" s="1" t="s">
         <v>6</v>
       </c>
@@ -17477,7 +17478,7 @@
       <c r="U204" s="1"/>
       <c r="V204" s="1"/>
     </row>
-    <row r="205" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A205" s="1" t="s">
         <v>6</v>
       </c>
@@ -17531,7 +17532,7 @@
       <c r="U205" s="1"/>
       <c r="V205" s="1"/>
     </row>
-    <row r="206" spans="1:22" ht="87" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:22" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A206" s="1" t="s">
         <v>6</v>
       </c>
@@ -17585,7 +17586,7 @@
       <c r="U206" s="1"/>
       <c r="V206" s="1"/>
     </row>
-    <row r="207" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A207" s="1" t="s">
         <v>6</v>
       </c>
@@ -17639,7 +17640,7 @@
       <c r="U207" s="1"/>
       <c r="V207" s="1"/>
     </row>
-    <row r="208" spans="1:22" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:22" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A208" s="1" t="s">
         <v>6</v>
       </c>
@@ -17693,7 +17694,7 @@
       <c r="U208" s="1"/>
       <c r="V208" s="1"/>
     </row>
-    <row r="209" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A209" s="1" t="s">
         <v>6</v>
       </c>
@@ -17747,7 +17748,7 @@
       <c r="U209" s="1"/>
       <c r="V209" s="1"/>
     </row>
-    <row r="210" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A210" s="1" t="s">
         <v>6</v>
       </c>
@@ -17801,7 +17802,7 @@
       <c r="U210" s="1"/>
       <c r="V210" s="1"/>
     </row>
-    <row r="211" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A211" s="1" t="s">
         <v>6</v>
       </c>
@@ -17853,7 +17854,7 @@
       <c r="U211" s="1"/>
       <c r="V211" s="1"/>
     </row>
-    <row r="212" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A212" s="1" t="s">
         <v>6</v>
       </c>
@@ -17905,7 +17906,7 @@
       <c r="U212" s="1"/>
       <c r="V212" s="1"/>
     </row>
-    <row r="213" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
       <c r="A213" s="1" t="s">
         <v>6</v>
       </c>
@@ -17959,7 +17960,7 @@
       <c r="U213" s="1"/>
       <c r="V213" s="1"/>
     </row>
-    <row r="214" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A214" s="1" t="s">
         <v>6</v>
       </c>
@@ -18011,7 +18012,7 @@
       <c r="U214" s="1"/>
       <c r="V214" s="1"/>
     </row>
-    <row r="215" spans="1:22" s="2" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:22" s="2" customFormat="1" ht="159.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A215" s="1" t="s">
         <v>6</v>
       </c>
@@ -18063,7 +18064,7 @@
       <c r="U215" s="1"/>
       <c r="V215" s="1"/>
     </row>
-    <row r="216" spans="1:22" s="2" customFormat="1" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:22" s="2" customFormat="1" ht="188.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A216" s="1" t="s">
         <v>6</v>
       </c>
@@ -18115,7 +18116,7 @@
       <c r="U216" s="1"/>
       <c r="V216" s="1"/>
     </row>
-    <row r="217" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A217" s="1" t="s">
         <v>6</v>
       </c>
@@ -18167,7 +18168,7 @@
       <c r="U217" s="1"/>
       <c r="V217" s="1"/>
     </row>
-    <row r="218" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A218" s="1" t="s">
         <v>6</v>
       </c>
@@ -18221,7 +18222,7 @@
       <c r="U218" s="1"/>
       <c r="V218" s="1"/>
     </row>
-    <row r="219" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A219" s="1" t="s">
         <v>6</v>
       </c>
@@ -18275,7 +18276,7 @@
       <c r="U219" s="1"/>
       <c r="V219" s="1"/>
     </row>
-    <row r="220" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A220" s="1" t="s">
         <v>6</v>
       </c>
@@ -18331,7 +18332,7 @@
       <c r="U220" s="1"/>
       <c r="V220" s="1"/>
     </row>
-    <row r="221" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A221" s="1" t="s">
         <v>6</v>
       </c>
@@ -18385,7 +18386,7 @@
       <c r="U221" s="1"/>
       <c r="V221" s="1"/>
     </row>
-    <row r="222" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A222" s="1" t="s">
         <v>6</v>
       </c>
@@ -18437,7 +18438,7 @@
       <c r="U222" s="1"/>
       <c r="V222" s="1"/>
     </row>
-    <row r="223" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A223" s="1" t="s">
         <v>6</v>
       </c>
@@ -18491,7 +18492,7 @@
       <c r="U223" s="1"/>
       <c r="V223" s="1"/>
     </row>
-    <row r="224" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A224" s="1" t="s">
         <v>6</v>
       </c>
@@ -18547,7 +18548,7 @@
       <c r="U224" s="1"/>
       <c r="V224" s="1"/>
     </row>
-    <row r="225" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A225" s="1" t="s">
         <v>6</v>
       </c>
@@ -18603,7 +18604,7 @@
       <c r="U225" s="1"/>
       <c r="V225" s="1"/>
     </row>
-    <row r="226" spans="1:22" s="2" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:22" s="2" customFormat="1" ht="159.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A226" s="1" t="s">
         <v>6</v>
       </c>
@@ -18657,7 +18658,7 @@
       <c r="U226" s="1"/>
       <c r="V226" s="1"/>
     </row>
-    <row r="227" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A227" s="1" t="s">
         <v>6</v>
       </c>
@@ -18709,7 +18710,7 @@
       <c r="U227" s="1"/>
       <c r="V227" s="1"/>
     </row>
-    <row r="228" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A228" s="1" t="s">
         <v>6</v>
       </c>
@@ -18761,7 +18762,7 @@
       <c r="U228" s="1"/>
       <c r="V228" s="1"/>
     </row>
-    <row r="229" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A229" s="1" t="s">
         <v>6</v>
       </c>
@@ -18817,7 +18818,7 @@
       <c r="U229" s="1"/>
       <c r="V229" s="1"/>
     </row>
-    <row r="230" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A230" s="1" t="s">
         <v>6</v>
       </c>
@@ -18871,7 +18872,7 @@
       <c r="U230" s="1"/>
       <c r="V230" s="1"/>
     </row>
-    <row r="231" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A231" s="1" t="s">
         <v>6</v>
       </c>
@@ -18923,7 +18924,7 @@
       <c r="U231" s="1"/>
       <c r="V231" s="1"/>
     </row>
-    <row r="232" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A232" s="1" t="s">
         <v>6</v>
       </c>
@@ -18975,7 +18976,7 @@
       <c r="U232" s="1"/>
       <c r="V232" s="1"/>
     </row>
-    <row r="233" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A233" s="1" t="s">
         <v>6</v>
       </c>
@@ -19027,7 +19028,7 @@
       <c r="U233" s="1"/>
       <c r="V233" s="1"/>
     </row>
-    <row r="234" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A234" s="1" t="s">
         <v>6</v>
       </c>
@@ -19079,7 +19080,7 @@
       <c r="U234" s="1"/>
       <c r="V234" s="1"/>
     </row>
-    <row r="235" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A235" s="1" t="s">
         <v>6</v>
       </c>
@@ -19131,7 +19132,7 @@
       <c r="U235" s="1"/>
       <c r="V235" s="1"/>
     </row>
-    <row r="236" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A236" s="1" t="s">
         <v>6</v>
       </c>
@@ -19183,7 +19184,7 @@
       <c r="U236" s="1"/>
       <c r="V236" s="1"/>
     </row>
-    <row r="237" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A237" s="1" t="s">
         <v>6</v>
       </c>
@@ -19235,7 +19236,7 @@
       <c r="U237" s="1"/>
       <c r="V237" s="1"/>
     </row>
-    <row r="238" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A238" s="1" t="s">
         <v>6</v>
       </c>
@@ -19289,7 +19290,7 @@
       <c r="U238" s="1"/>
       <c r="V238" s="1"/>
     </row>
-    <row r="239" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A239" s="1" t="s">
         <v>6</v>
       </c>
@@ -19341,7 +19342,7 @@
       <c r="U239" s="1"/>
       <c r="V239" s="1"/>
     </row>
-    <row r="240" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A240" s="1" t="s">
         <v>6</v>
       </c>
@@ -19393,7 +19394,7 @@
       <c r="U240" s="1"/>
       <c r="V240" s="1"/>
     </row>
-    <row r="241" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A241" s="1" t="s">
         <v>6</v>
       </c>
@@ -19445,7 +19446,7 @@
       <c r="U241" s="1"/>
       <c r="V241" s="1"/>
     </row>
-    <row r="242" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A242" s="1" t="s">
         <v>6</v>
       </c>
@@ -19497,7 +19498,7 @@
       <c r="U242" s="1"/>
       <c r="V242" s="1"/>
     </row>
-    <row r="243" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A243" s="1" t="s">
         <v>6</v>
       </c>
@@ -19549,7 +19550,7 @@
       <c r="U243" s="1"/>
       <c r="V243" s="1"/>
     </row>
-    <row r="244" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A244" s="1" t="s">
         <v>6</v>
       </c>
@@ -19601,7 +19602,7 @@
       <c r="U244" s="1"/>
       <c r="V244" s="1"/>
     </row>
-    <row r="245" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A245" s="1" t="s">
         <v>6</v>
       </c>
@@ -19655,7 +19656,7 @@
       <c r="U245" s="1"/>
       <c r="V245" s="1"/>
     </row>
-    <row r="246" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A246" s="1" t="s">
         <v>6</v>
       </c>
@@ -19709,7 +19710,7 @@
       <c r="U246" s="1"/>
       <c r="V246" s="1"/>
     </row>
-    <row r="247" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A247" s="1" t="s">
         <v>6</v>
       </c>
@@ -19761,7 +19762,7 @@
       <c r="U247" s="1"/>
       <c r="V247" s="1"/>
     </row>
-    <row r="248" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A248" s="1" t="s">
         <v>6</v>
       </c>
@@ -19813,7 +19814,7 @@
       <c r="U248" s="1"/>
       <c r="V248" s="1"/>
     </row>
-    <row r="249" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A249" s="1" t="s">
         <v>6</v>
       </c>
@@ -19865,7 +19866,7 @@
       <c r="U249" s="1"/>
       <c r="V249" s="1"/>
     </row>
-    <row r="250" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
       <c r="A250" s="1" t="s">
         <v>6</v>
       </c>
@@ -19917,7 +19918,7 @@
       <c r="U250" s="1"/>
       <c r="V250" s="1"/>
     </row>
-    <row r="251" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
       <c r="A251" s="1" t="s">
         <v>6</v>
       </c>
@@ -19969,7 +19970,7 @@
       <c r="U251" s="1"/>
       <c r="V251" s="1"/>
     </row>
-    <row r="252" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
       <c r="A252" s="1" t="s">
         <v>6</v>
       </c>
@@ -20021,7 +20022,7 @@
       <c r="U252" s="1"/>
       <c r="V252" s="1"/>
     </row>
-    <row r="253" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A253" s="1" t="s">
         <v>6</v>
       </c>
@@ -20077,7 +20078,7 @@
       <c r="U253" s="1"/>
       <c r="V253" s="1"/>
     </row>
-    <row r="254" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A254" s="1" t="s">
         <v>6</v>
       </c>
@@ -20131,7 +20132,7 @@
       <c r="U254" s="1"/>
       <c r="V254" s="1"/>
     </row>
-    <row r="255" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A255" s="1" t="s">
         <v>6</v>
       </c>
@@ -20185,7 +20186,7 @@
       <c r="U255" s="1"/>
       <c r="V255" s="1"/>
     </row>
-    <row r="256" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A256" s="1" t="s">
         <v>6</v>
       </c>
@@ -20237,7 +20238,7 @@
       <c r="U256" s="1"/>
       <c r="V256" s="1"/>
     </row>
-    <row r="257" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A257" s="1" t="s">
         <v>6</v>
       </c>
@@ -20289,7 +20290,7 @@
       <c r="U257" s="1"/>
       <c r="V257" s="1"/>
     </row>
-    <row r="258" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
       <c r="A258" s="1" t="s">
         <v>6</v>
       </c>
@@ -20341,7 +20342,7 @@
       <c r="U258" s="1"/>
       <c r="V258" s="1"/>
     </row>
-    <row r="259" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A259" s="1" t="s">
         <v>6</v>
       </c>
@@ -20393,7 +20394,7 @@
       <c r="U259" s="1"/>
       <c r="V259" s="1"/>
     </row>
-    <row r="260" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A260" s="1" t="s">
         <v>6</v>
       </c>
@@ -20445,7 +20446,7 @@
       <c r="U260" s="1"/>
       <c r="V260" s="1"/>
     </row>
-    <row r="261" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A261" s="1" t="s">
         <v>6</v>
       </c>
@@ -20499,7 +20500,7 @@
       <c r="U261" s="1"/>
       <c r="V261" s="1"/>
     </row>
-    <row r="262" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A262" s="1" t="s">
         <v>6</v>
       </c>
@@ -20551,7 +20552,7 @@
       <c r="U262" s="1"/>
       <c r="V262" s="1"/>
     </row>
-    <row r="263" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A263" s="1" t="s">
         <v>6</v>
       </c>
@@ -20603,7 +20604,7 @@
       <c r="U263" s="1"/>
       <c r="V263" s="1"/>
     </row>
-    <row r="264" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A264" s="1" t="s">
         <v>6</v>
       </c>
@@ -20655,7 +20656,7 @@
       <c r="U264" s="1"/>
       <c r="V264" s="1"/>
     </row>
-    <row r="265" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A265" s="1" t="s">
         <v>6</v>
       </c>
@@ -20707,7 +20708,7 @@
       <c r="U265" s="1"/>
       <c r="V265" s="1"/>
     </row>
-    <row r="266" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A266" s="1" t="s">
         <v>6</v>
       </c>
@@ -20759,7 +20760,7 @@
       <c r="U266" s="1"/>
       <c r="V266" s="1"/>
     </row>
-    <row r="267" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A267" s="1" t="s">
         <v>6</v>
       </c>
@@ -20811,7 +20812,7 @@
       <c r="U267" s="1"/>
       <c r="V267" s="1"/>
     </row>
-    <row r="268" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A268" s="1" t="s">
         <v>6</v>
       </c>
@@ -20865,7 +20866,7 @@
       <c r="U268" s="1"/>
       <c r="V268" s="1"/>
     </row>
-    <row r="269" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
       <c r="A269" s="1" t="s">
         <v>6</v>
       </c>
@@ -20917,7 +20918,7 @@
       <c r="U269" s="1"/>
       <c r="V269" s="1"/>
     </row>
-    <row r="270" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A270" s="1" t="s">
         <v>6</v>
       </c>
@@ -20969,7 +20970,7 @@
       <c r="U270" s="1"/>
       <c r="V270" s="1"/>
     </row>
-    <row r="271" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A271" s="1" t="s">
         <v>6</v>
       </c>
@@ -21021,7 +21022,7 @@
       <c r="U271" s="1"/>
       <c r="V271" s="1"/>
     </row>
-    <row r="272" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A272" s="1" t="s">
         <v>6</v>
       </c>
@@ -21075,7 +21076,7 @@
       <c r="U272" s="1"/>
       <c r="V272" s="1"/>
     </row>
-    <row r="273" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A273" s="1" t="s">
         <v>6</v>
       </c>
@@ -21129,7 +21130,7 @@
       <c r="U273" s="1"/>
       <c r="V273" s="1"/>
     </row>
-    <row r="274" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A274" s="1" t="s">
         <v>6</v>
       </c>
@@ -21183,7 +21184,7 @@
       <c r="U274" s="1"/>
       <c r="V274" s="1"/>
     </row>
-    <row r="275" spans="1:22" s="2" customFormat="1" ht="377" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:22" s="2" customFormat="1" ht="377" hidden="1" x14ac:dyDescent="0.35">
       <c r="A275" s="1" t="s">
         <v>6</v>
       </c>
@@ -21239,7 +21240,7 @@
       <c r="U275" s="1"/>
       <c r="V275" s="1"/>
     </row>
-    <row r="276" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A276" s="1" t="s">
         <v>6</v>
       </c>
@@ -21293,7 +21294,7 @@
       <c r="U276" s="1"/>
       <c r="V276" s="1"/>
     </row>
-    <row r="277" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A277" s="1" t="s">
         <v>6</v>
       </c>
@@ -21347,7 +21348,7 @@
       <c r="U277" s="1"/>
       <c r="V277" s="1"/>
     </row>
-    <row r="278" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A278" s="1" t="s">
         <v>6</v>
       </c>
@@ -21401,7 +21402,7 @@
       <c r="U278" s="1"/>
       <c r="V278" s="1"/>
     </row>
-    <row r="279" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A279" s="1" t="s">
         <v>6</v>
       </c>
@@ -21455,7 +21456,7 @@
       <c r="U279" s="1"/>
       <c r="V279" s="1"/>
     </row>
-    <row r="280" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A280" s="1" t="s">
         <v>6</v>
       </c>
@@ -21511,7 +21512,7 @@
       <c r="U280" s="1"/>
       <c r="V280" s="1"/>
     </row>
-    <row r="281" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A281" s="1" t="s">
         <v>6</v>
       </c>
@@ -21565,7 +21566,7 @@
       <c r="U281" s="1"/>
       <c r="V281" s="1"/>
     </row>
-    <row r="282" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
       <c r="A282" s="1" t="s">
         <v>6</v>
       </c>
@@ -21619,7 +21620,7 @@
       <c r="U282" s="1"/>
       <c r="V282" s="1"/>
     </row>
-    <row r="283" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A283" s="1" t="s">
         <v>6</v>
       </c>
@@ -21673,7 +21674,7 @@
       <c r="U283" s="1"/>
       <c r="V283" s="1"/>
     </row>
-    <row r="284" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
       <c r="A284" s="1" t="s">
         <v>6</v>
       </c>
@@ -21727,7 +21728,7 @@
       <c r="U284" s="1"/>
       <c r="V284" s="1"/>
     </row>
-    <row r="285" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A285" s="1" t="s">
         <v>6</v>
       </c>
@@ -21779,7 +21780,7 @@
       <c r="U285" s="1"/>
       <c r="V285" s="1"/>
     </row>
-    <row r="286" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A286" s="1" t="s">
         <v>6</v>
       </c>
@@ -21831,7 +21832,7 @@
       <c r="U286" s="1"/>
       <c r="V286" s="1"/>
     </row>
-    <row r="287" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A287" s="1" t="s">
         <v>6</v>
       </c>
@@ -21883,7 +21884,7 @@
       <c r="U287" s="1"/>
       <c r="V287" s="1"/>
     </row>
-    <row r="288" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A288" s="1" t="s">
         <v>6</v>
       </c>
@@ -21935,7 +21936,7 @@
       <c r="U288" s="1"/>
       <c r="V288" s="1"/>
     </row>
-    <row r="289" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A289" s="1" t="s">
         <v>6</v>
       </c>
@@ -21987,7 +21988,7 @@
       <c r="U289" s="1"/>
       <c r="V289" s="1"/>
     </row>
-    <row r="290" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
       <c r="A290" s="1" t="s">
         <v>6</v>
       </c>
@@ -22039,7 +22040,7 @@
       <c r="U290" s="1"/>
       <c r="V290" s="1"/>
     </row>
-    <row r="291" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
       <c r="A291" s="1" t="s">
         <v>6</v>
       </c>
@@ -22091,7 +22092,7 @@
       <c r="U291" s="1"/>
       <c r="V291" s="1"/>
     </row>
-    <row r="292" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
       <c r="A292" s="1" t="s">
         <v>6</v>
       </c>
@@ -22143,7 +22144,7 @@
       <c r="U292" s="1"/>
       <c r="V292" s="1"/>
     </row>
-    <row r="293" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A293" s="1" t="s">
         <v>6</v>
       </c>
@@ -22195,7 +22196,7 @@
       <c r="U293" s="1"/>
       <c r="V293" s="1"/>
     </row>
-    <row r="294" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A294" s="1" t="s">
         <v>6</v>
       </c>
@@ -22247,7 +22248,7 @@
       <c r="U294" s="1"/>
       <c r="V294" s="1"/>
     </row>
-    <row r="295" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A295" s="1" t="s">
         <v>6</v>
       </c>
@@ -22299,7 +22300,7 @@
       <c r="U295" s="1"/>
       <c r="V295" s="1"/>
     </row>
-    <row r="296" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A296" s="1" t="s">
         <v>6</v>
       </c>
@@ -22351,7 +22352,7 @@
       <c r="U296" s="1"/>
       <c r="V296" s="1"/>
     </row>
-    <row r="297" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A297" s="1" t="s">
         <v>6</v>
       </c>
@@ -22403,7 +22404,7 @@
       <c r="U297" s="1"/>
       <c r="V297" s="1"/>
     </row>
-    <row r="298" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A298" s="1" t="s">
         <v>6</v>
       </c>
@@ -22455,7 +22456,7 @@
       <c r="U298" s="1"/>
       <c r="V298" s="1"/>
     </row>
-    <row r="299" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A299" s="1" t="s">
         <v>6</v>
       </c>
@@ -22507,7 +22508,7 @@
       <c r="U299" s="1"/>
       <c r="V299" s="1"/>
     </row>
-    <row r="300" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A300" s="1" t="s">
         <v>6</v>
       </c>
@@ -22559,7 +22560,7 @@
       <c r="U300" s="1"/>
       <c r="V300" s="1"/>
     </row>
-    <row r="301" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A301" s="1" t="s">
         <v>6</v>
       </c>
@@ -22611,7 +22612,7 @@
       <c r="U301" s="1"/>
       <c r="V301" s="1"/>
     </row>
-    <row r="302" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A302" s="1" t="s">
         <v>6</v>
       </c>
@@ -22663,7 +22664,7 @@
       <c r="U302" s="1"/>
       <c r="V302" s="1"/>
     </row>
-    <row r="303" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A303" s="1" t="s">
         <v>6</v>
       </c>
@@ -22717,7 +22718,7 @@
       <c r="U303" s="1"/>
       <c r="V303" s="1"/>
     </row>
-    <row r="304" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A304" s="1" t="s">
         <v>6</v>
       </c>
@@ -22769,7 +22770,7 @@
       <c r="U304" s="1"/>
       <c r="V304" s="1"/>
     </row>
-    <row r="305" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A305" s="1" t="s">
         <v>6</v>
       </c>
@@ -22821,7 +22822,7 @@
       <c r="U305" s="1"/>
       <c r="V305" s="1"/>
     </row>
-    <row r="306" spans="1:22" s="2" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:22" s="2" customFormat="1" ht="76.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A306" s="1" t="s">
         <v>6</v>
       </c>
@@ -22873,7 +22874,7 @@
       <c r="U306" s="1"/>
       <c r="V306" s="1"/>
     </row>
-    <row r="307" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
       <c r="A307" s="1" t="s">
         <v>6</v>
       </c>
@@ -22925,7 +22926,7 @@
       <c r="U307" s="1"/>
       <c r="V307" s="1"/>
     </row>
-    <row r="308" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A308" s="1" t="s">
         <v>6</v>
       </c>
@@ -22977,7 +22978,7 @@
       <c r="U308" s="1"/>
       <c r="V308" s="1"/>
     </row>
-    <row r="309" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A309" s="1" t="s">
         <v>6</v>
       </c>
@@ -23029,7 +23030,7 @@
       <c r="U309" s="1"/>
       <c r="V309" s="1"/>
     </row>
-    <row r="310" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A310" s="1" t="s">
         <v>6</v>
       </c>
@@ -23081,7 +23082,7 @@
       <c r="U310" s="1"/>
       <c r="V310" s="1"/>
     </row>
-    <row r="311" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A311" s="1" t="s">
         <v>6</v>
       </c>
@@ -23133,7 +23134,7 @@
       <c r="U311" s="1"/>
       <c r="V311" s="1"/>
     </row>
-    <row r="312" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A312" s="1" t="s">
         <v>6</v>
       </c>
@@ -23185,7 +23186,7 @@
       <c r="U312" s="1"/>
       <c r="V312" s="1"/>
     </row>
-    <row r="313" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A313" s="1" t="s">
         <v>6</v>
       </c>
@@ -23237,7 +23238,7 @@
       <c r="U313" s="1"/>
       <c r="V313" s="1"/>
     </row>
-    <row r="314" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A314" s="1" t="s">
         <v>6</v>
       </c>
@@ -23293,7 +23294,7 @@
       <c r="U314" s="1"/>
       <c r="V314" s="1"/>
     </row>
-    <row r="315" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A315" s="1" t="s">
         <v>6</v>
       </c>
@@ -23351,7 +23352,7 @@
       <c r="U315" s="1"/>
       <c r="V315" s="1"/>
     </row>
-    <row r="316" spans="1:22" ht="87" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:22" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A316" s="1" t="s">
         <v>6</v>
       </c>
@@ -23407,7 +23408,7 @@
       <c r="U316" s="1"/>
       <c r="V316" s="1"/>
     </row>
-    <row r="317" spans="1:22" ht="87" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:22" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A317" s="1" t="s">
         <v>6</v>
       </c>
@@ -23461,7 +23462,7 @@
       <c r="U317" s="1"/>
       <c r="V317" s="1"/>
     </row>
-    <row r="318" spans="1:22" ht="87" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:22" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A318" s="1" t="s">
         <v>6</v>
       </c>
@@ -23511,7 +23512,7 @@
       <c r="U318" s="1"/>
       <c r="V318" s="1"/>
     </row>
-    <row r="319" spans="1:22" ht="87" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:22" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A319" s="1" t="s">
         <v>6</v>
       </c>
@@ -23567,7 +23568,7 @@
       <c r="U319" s="1"/>
       <c r="V319" s="1"/>
     </row>
-    <row r="320" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A320" s="1" t="s">
         <v>6</v>
       </c>
@@ -23619,7 +23620,7 @@
       <c r="U320" s="1"/>
       <c r="V320" s="1"/>
     </row>
-    <row r="321" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A321" s="1" t="s">
         <v>6</v>
       </c>
@@ -23673,7 +23674,7 @@
       <c r="U321" s="1"/>
       <c r="V321" s="1"/>
     </row>
-    <row r="322" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A322" s="1" t="s">
         <v>6</v>
       </c>
@@ -23725,7 +23726,7 @@
       <c r="U322" s="1"/>
       <c r="V322" s="1"/>
     </row>
-    <row r="323" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A323" s="1" t="s">
         <v>6</v>
       </c>
@@ -23781,7 +23782,7 @@
       <c r="U323" s="1"/>
       <c r="V323" s="1"/>
     </row>
-    <row r="324" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A324" s="1" t="s">
         <v>6</v>
       </c>
@@ -23833,7 +23834,7 @@
       <c r="U324" s="1"/>
       <c r="V324" s="1"/>
     </row>
-    <row r="325" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A325" s="1" t="s">
         <v>6</v>
       </c>
@@ -23885,7 +23886,7 @@
       <c r="U325" s="1"/>
       <c r="V325" s="1"/>
     </row>
-    <row r="326" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A326" s="1" t="s">
         <v>6</v>
       </c>
@@ -23937,7 +23938,7 @@
       <c r="U326" s="1"/>
       <c r="V326" s="1"/>
     </row>
-    <row r="327" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A327" s="1" t="s">
         <v>6</v>
       </c>
@@ -23989,7 +23990,7 @@
       <c r="U327" s="1"/>
       <c r="V327" s="1"/>
     </row>
-    <row r="328" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A328" s="1" t="s">
         <v>6</v>
       </c>
@@ -24041,7 +24042,7 @@
       <c r="U328" s="1"/>
       <c r="V328" s="1"/>
     </row>
-    <row r="329" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A329" s="1" t="s">
         <v>6</v>
       </c>
@@ -24093,7 +24094,7 @@
       <c r="U329" s="1"/>
       <c r="V329" s="1"/>
     </row>
-    <row r="330" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A330" s="1" t="s">
         <v>6</v>
       </c>
@@ -24145,7 +24146,7 @@
       <c r="U330" s="1"/>
       <c r="V330" s="1"/>
     </row>
-    <row r="331" spans="1:22" ht="58" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:22" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A331" s="1" t="s">
         <v>6</v>
       </c>
@@ -24197,7 +24198,7 @@
       <c r="U331" s="1"/>
       <c r="V331" s="1"/>
     </row>
-    <row r="332" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A332" s="1" t="s">
         <v>6</v>
       </c>
@@ -24251,7 +24252,7 @@
       <c r="U332" s="1"/>
       <c r="V332" s="1"/>
     </row>
-    <row r="333" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
       <c r="A333" s="1" t="s">
         <v>6</v>
       </c>
@@ -24305,7 +24306,7 @@
       <c r="U333" s="1"/>
       <c r="V333" s="1"/>
     </row>
-    <row r="334" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
       <c r="A334" s="1" t="s">
         <v>6</v>
       </c>
@@ -24359,7 +24360,7 @@
       <c r="U334" s="1"/>
       <c r="V334" s="1"/>
     </row>
-    <row r="335" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
       <c r="A335" s="1" t="s">
         <v>6</v>
       </c>
@@ -24411,7 +24412,7 @@
       <c r="U335" s="1"/>
       <c r="V335" s="1"/>
     </row>
-    <row r="336" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A336" s="1" t="s">
         <v>6</v>
       </c>
@@ -24463,7 +24464,7 @@
       <c r="U336" s="1"/>
       <c r="V336" s="1"/>
     </row>
-    <row r="337" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A337" s="1" t="s">
         <v>6</v>
       </c>
@@ -24515,7 +24516,7 @@
       <c r="U337" s="1"/>
       <c r="V337" s="1"/>
     </row>
-    <row r="338" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A338" s="1" t="s">
         <v>6</v>
       </c>
@@ -24569,7 +24570,7 @@
       <c r="U338" s="1"/>
       <c r="V338" s="1"/>
     </row>
-    <row r="339" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A339" s="1" t="s">
         <v>6</v>
       </c>
@@ -24621,7 +24622,7 @@
       <c r="U339" s="1"/>
       <c r="V339" s="1"/>
     </row>
-    <row r="340" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A340" s="1" t="s">
         <v>6</v>
       </c>
@@ -24673,7 +24674,7 @@
       <c r="U340" s="1"/>
       <c r="V340" s="1"/>
     </row>
-    <row r="341" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A341" s="1" t="s">
         <v>6</v>
       </c>
@@ -24725,7 +24726,7 @@
       <c r="U341" s="1"/>
       <c r="V341" s="1"/>
     </row>
-    <row r="342" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A342" s="1" t="s">
         <v>6</v>
       </c>
@@ -24779,7 +24780,7 @@
       <c r="U342" s="1"/>
       <c r="V342" s="1"/>
     </row>
-    <row r="343" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A343" s="1" t="s">
         <v>6</v>
       </c>
@@ -24833,7 +24834,7 @@
       <c r="U343" s="1"/>
       <c r="V343" s="1"/>
     </row>
-    <row r="344" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A344" s="1" t="s">
         <v>6</v>
       </c>
@@ -24885,7 +24886,7 @@
       <c r="U344" s="1"/>
       <c r="V344" s="1"/>
     </row>
-    <row r="345" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A345" s="1" t="s">
         <v>6</v>
       </c>
@@ -24937,7 +24938,7 @@
       <c r="U345" s="1"/>
       <c r="V345" s="1"/>
     </row>
-    <row r="346" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A346" s="1" t="s">
         <v>6</v>
       </c>
@@ -24989,7 +24990,7 @@
       <c r="U346" s="1"/>
       <c r="V346" s="1"/>
     </row>
-    <row r="347" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A347" s="1" t="s">
         <v>6</v>
       </c>
@@ -25043,7 +25044,7 @@
       <c r="U347" s="1"/>
       <c r="V347" s="1"/>
     </row>
-    <row r="348" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A348" s="1" t="s">
         <v>6</v>
       </c>
@@ -25095,7 +25096,7 @@
       <c r="U348" s="1"/>
       <c r="V348" s="1"/>
     </row>
-    <row r="349" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A349" s="1" t="s">
         <v>6</v>
       </c>
@@ -25149,7 +25150,7 @@
       <c r="U349" s="1"/>
       <c r="V349" s="1"/>
     </row>
-    <row r="350" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A350" s="1" t="s">
         <v>6</v>
       </c>
@@ -25201,7 +25202,7 @@
       <c r="U350" s="1"/>
       <c r="V350" s="1"/>
     </row>
-    <row r="351" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A351" s="1" t="s">
         <v>6</v>
       </c>
@@ -25253,7 +25254,7 @@
       <c r="U351" s="1"/>
       <c r="V351" s="1"/>
     </row>
-    <row r="352" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A352" s="1" t="s">
         <v>6</v>
       </c>
@@ -25307,7 +25308,7 @@
       <c r="U352" s="1"/>
       <c r="V352" s="1"/>
     </row>
-    <row r="353" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A353" s="1" t="s">
         <v>6</v>
       </c>
@@ -25357,7 +25358,7 @@
       <c r="U353" s="1"/>
       <c r="V353" s="1"/>
     </row>
-    <row r="354" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A354" s="1" t="s">
         <v>6</v>
       </c>
@@ -25407,7 +25408,7 @@
       <c r="U354" s="1"/>
       <c r="V354" s="1"/>
     </row>
-    <row r="355" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A355" s="1" t="s">
         <v>6</v>
       </c>
@@ -25459,7 +25460,7 @@
       <c r="U355" s="1"/>
       <c r="V355" s="1"/>
     </row>
-    <row r="356" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A356" s="1" t="s">
         <v>6</v>
       </c>
@@ -25511,7 +25512,7 @@
       <c r="U356" s="1"/>
       <c r="V356" s="1"/>
     </row>
-    <row r="357" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A357" s="1" t="s">
         <v>6</v>
       </c>
@@ -25563,7 +25564,7 @@
       <c r="U357" s="1"/>
       <c r="V357" s="1"/>
     </row>
-    <row r="358" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A358" s="1" t="s">
         <v>6</v>
       </c>
@@ -25615,7 +25616,7 @@
       <c r="U358" s="1"/>
       <c r="V358" s="1"/>
     </row>
-    <row r="359" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A359" s="1" t="s">
         <v>6</v>
       </c>
@@ -25669,7 +25670,7 @@
       <c r="U359" s="1"/>
       <c r="V359" s="1"/>
     </row>
-    <row r="360" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A360" s="1" t="s">
         <v>6</v>
       </c>
@@ -25721,7 +25722,7 @@
       <c r="U360" s="1"/>
       <c r="V360" s="1"/>
     </row>
-    <row r="361" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A361" s="1" t="s">
         <v>6</v>
       </c>
@@ -25773,7 +25774,7 @@
       <c r="U361" s="1"/>
       <c r="V361" s="1"/>
     </row>
-    <row r="362" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A362" s="1" t="s">
         <v>6</v>
       </c>
@@ -25825,7 +25826,7 @@
       <c r="U362" s="1"/>
       <c r="V362" s="1"/>
     </row>
-    <row r="363" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A363" s="1" t="s">
         <v>6</v>
       </c>
@@ -25879,7 +25880,7 @@
       <c r="U363" s="1"/>
       <c r="V363" s="1"/>
     </row>
-    <row r="364" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A364" s="1" t="s">
         <v>6</v>
       </c>
@@ -25931,7 +25932,7 @@
       <c r="U364" s="1"/>
       <c r="V364" s="1"/>
     </row>
-    <row r="365" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A365" s="1" t="s">
         <v>6</v>
       </c>
@@ -25983,7 +25984,7 @@
       <c r="U365" s="1"/>
       <c r="V365" s="1"/>
     </row>
-    <row r="366" spans="1:22" s="2" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:22" s="2" customFormat="1" ht="159.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A366" s="1" t="s">
         <v>6</v>
       </c>
@@ -26035,7 +26036,7 @@
       <c r="U366" s="1"/>
       <c r="V366" s="1"/>
     </row>
-    <row r="367" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A367" s="1" t="s">
         <v>6</v>
       </c>
@@ -26087,7 +26088,7 @@
       <c r="U367" s="1"/>
       <c r="V367" s="1"/>
     </row>
-    <row r="368" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A368" s="1" t="s">
         <v>6</v>
       </c>
@@ -26139,7 +26140,7 @@
       <c r="U368" s="1"/>
       <c r="V368" s="1"/>
     </row>
-    <row r="369" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A369" s="1" t="s">
         <v>6</v>
       </c>
@@ -26191,7 +26192,7 @@
       <c r="U369" s="1"/>
       <c r="V369" s="1"/>
     </row>
-    <row r="370" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A370" s="1" t="s">
         <v>6</v>
       </c>
@@ -26245,7 +26246,7 @@
       <c r="U370" s="1"/>
       <c r="V370" s="1"/>
     </row>
-    <row r="371" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A371" s="1" t="s">
         <v>6</v>
       </c>
@@ -26297,7 +26298,7 @@
       <c r="U371" s="1"/>
       <c r="V371" s="1"/>
     </row>
-    <row r="372" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A372" s="1" t="s">
         <v>6</v>
       </c>
@@ -26349,7 +26350,7 @@
       <c r="U372" s="1"/>
       <c r="V372" s="1"/>
     </row>
-    <row r="373" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A373" s="1" t="s">
         <v>6</v>
       </c>
@@ -26401,7 +26402,7 @@
       <c r="U373" s="1"/>
       <c r="V373" s="1"/>
     </row>
-    <row r="374" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A374" s="1" t="s">
         <v>6</v>
       </c>
@@ -26455,7 +26456,7 @@
       <c r="U374" s="1"/>
       <c r="V374" s="1"/>
     </row>
-    <row r="375" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A375" s="1" t="s">
         <v>6</v>
       </c>
@@ -26509,7 +26510,7 @@
       <c r="U375" s="1"/>
       <c r="V375" s="1"/>
     </row>
-    <row r="376" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A376" s="1" t="s">
         <v>6</v>
       </c>
@@ -26565,7 +26566,7 @@
       <c r="U376" s="1"/>
       <c r="V376" s="1"/>
     </row>
-    <row r="377" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A377" s="1" t="s">
         <v>6</v>
       </c>
@@ -26619,7 +26620,7 @@
       <c r="U377" s="1"/>
       <c r="V377" s="1"/>
     </row>
-    <row r="378" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A378" s="1" t="s">
         <v>6</v>
       </c>
@@ -26673,7 +26674,7 @@
       <c r="U378" s="1"/>
       <c r="V378" s="1"/>
     </row>
-    <row r="379" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A379" s="1" t="s">
         <v>6</v>
       </c>
@@ -26729,7 +26730,7 @@
       <c r="U379" s="1"/>
       <c r="V379" s="1"/>
     </row>
-    <row r="380" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A380" s="1" t="s">
         <v>6</v>
       </c>
@@ -26785,7 +26786,7 @@
       <c r="U380" s="1"/>
       <c r="V380" s="1"/>
     </row>
-    <row r="381" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A381" s="1" t="s">
         <v>6</v>
       </c>
@@ -26839,7 +26840,7 @@
       <c r="U381" s="1"/>
       <c r="V381" s="1"/>
     </row>
-    <row r="382" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A382" s="1" t="s">
         <v>6</v>
       </c>
@@ -26895,7 +26896,7 @@
       <c r="U382" s="1"/>
       <c r="V382" s="1"/>
     </row>
-    <row r="383" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="383" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A383" s="1" t="s">
         <v>6</v>
       </c>
@@ -26949,7 +26950,7 @@
       <c r="U383" s="1"/>
       <c r="V383" s="1"/>
     </row>
-    <row r="384" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="384" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A384" s="1" t="s">
         <v>6</v>
       </c>
@@ -27001,7 +27002,7 @@
       <c r="U384" s="1"/>
       <c r="V384" s="1"/>
     </row>
-    <row r="385" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="385" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A385" s="1" t="s">
         <v>6</v>
       </c>
@@ -27055,7 +27056,7 @@
       <c r="U385" s="1"/>
       <c r="V385" s="1"/>
     </row>
-    <row r="386" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="386" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A386" s="1" t="s">
         <v>6</v>
       </c>
@@ -27111,7 +27112,7 @@
       <c r="U386" s="1"/>
       <c r="V386" s="1"/>
     </row>
-    <row r="387" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="387" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A387" s="1" t="s">
         <v>6</v>
       </c>
@@ -27165,7 +27166,7 @@
       <c r="U387" s="1"/>
       <c r="V387" s="1"/>
     </row>
-    <row r="388" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="388" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A388" s="1" t="s">
         <v>6</v>
       </c>
@@ -27219,7 +27220,7 @@
       <c r="U388" s="1"/>
       <c r="V388" s="1"/>
     </row>
-    <row r="389" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="389" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A389" s="1" t="s">
         <v>6</v>
       </c>
@@ -27273,7 +27274,7 @@
       <c r="U389" s="1"/>
       <c r="V389" s="1"/>
     </row>
-    <row r="390" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="390" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A390" s="1" t="s">
         <v>6</v>
       </c>
@@ -27327,7 +27328,7 @@
       <c r="U390" s="1"/>
       <c r="V390" s="1"/>
     </row>
-    <row r="391" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="391" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
       <c r="A391" s="1" t="s">
         <v>6</v>
       </c>
@@ -27383,7 +27384,7 @@
       <c r="U391" s="1"/>
       <c r="V391" s="1"/>
     </row>
-    <row r="392" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="392" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A392" s="1" t="s">
         <v>6</v>
       </c>
@@ -27437,7 +27438,7 @@
       <c r="U392" s="1"/>
       <c r="V392" s="1"/>
     </row>
-    <row r="393" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="393" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A393" s="1" t="s">
         <v>6</v>
       </c>
@@ -27491,7 +27492,7 @@
       <c r="U393" s="1"/>
       <c r="V393" s="1"/>
     </row>
-    <row r="394" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="394" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A394" s="1" t="s">
         <v>6</v>
       </c>
@@ -27545,7 +27546,7 @@
       <c r="U394" s="1"/>
       <c r="V394" s="1"/>
     </row>
-    <row r="395" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="395" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A395" s="1" t="s">
         <v>6</v>
       </c>
@@ -27599,7 +27600,7 @@
       <c r="U395" s="1"/>
       <c r="V395" s="1"/>
     </row>
-    <row r="396" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="396" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A396" s="1" t="s">
         <v>6</v>
       </c>
@@ -27655,7 +27656,7 @@
       <c r="U396" s="1"/>
       <c r="V396" s="1"/>
     </row>
-    <row r="397" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="397" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A397" s="1" t="s">
         <v>6</v>
       </c>
@@ -27711,7 +27712,7 @@
       <c r="U397" s="1"/>
       <c r="V397" s="1"/>
     </row>
-    <row r="398" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="398" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A398" s="1" t="s">
         <v>6</v>
       </c>
@@ -27765,7 +27766,7 @@
       <c r="U398" s="1"/>
       <c r="V398" s="1"/>
     </row>
-    <row r="399" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="399" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A399" s="1" t="s">
         <v>6</v>
       </c>
@@ -27819,7 +27820,7 @@
       <c r="U399" s="1"/>
       <c r="V399" s="1"/>
     </row>
-    <row r="400" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="400" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A400" s="1" t="s">
         <v>6</v>
       </c>
@@ -27875,7 +27876,7 @@
       <c r="U400" s="1"/>
       <c r="V400" s="1"/>
     </row>
-    <row r="401" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="401" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A401" s="1" t="s">
         <v>6</v>
       </c>
@@ -27929,7 +27930,7 @@
       <c r="U401" s="1"/>
       <c r="V401" s="1"/>
     </row>
-    <row r="402" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="402" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A402" s="1" t="s">
         <v>6</v>
       </c>
@@ -27983,7 +27984,7 @@
       <c r="U402" s="1"/>
       <c r="V402" s="1"/>
     </row>
-    <row r="403" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="403" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A403" s="1" t="s">
         <v>6</v>
       </c>
@@ -28037,7 +28038,7 @@
       <c r="U403" s="1"/>
       <c r="V403" s="1"/>
     </row>
-    <row r="404" spans="1:22" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="404" spans="1:22" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A404" s="1" t="s">
         <v>6</v>
       </c>
@@ -28091,7 +28092,7 @@
       <c r="U404" s="1"/>
       <c r="V404" s="1"/>
     </row>
-    <row r="405" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="405" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A405" s="1" t="s">
         <v>6</v>
       </c>
@@ -28145,7 +28146,7 @@
       <c r="U405" s="1"/>
       <c r="V405" s="1"/>
     </row>
-    <row r="406" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="406" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A406" s="1" t="s">
         <v>6</v>
       </c>
@@ -28199,7 +28200,7 @@
       <c r="U406" s="1"/>
       <c r="V406" s="1"/>
     </row>
-    <row r="407" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="407" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A407" s="1" t="s">
         <v>6</v>
       </c>
@@ -28253,7 +28254,7 @@
       <c r="U407" s="1"/>
       <c r="V407" s="1"/>
     </row>
-    <row r="408" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="408" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A408" s="1" t="s">
         <v>6</v>
       </c>
@@ -28307,7 +28308,7 @@
       <c r="U408" s="1"/>
       <c r="V408" s="1"/>
     </row>
-    <row r="409" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="409" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A409" s="1" t="s">
         <v>6</v>
       </c>
@@ -28361,7 +28362,7 @@
       <c r="U409" s="1"/>
       <c r="V409" s="1"/>
     </row>
-    <row r="410" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="410" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A410" s="1" t="s">
         <v>6</v>
       </c>
@@ -28415,7 +28416,7 @@
       <c r="U410" s="1"/>
       <c r="V410" s="1"/>
     </row>
-    <row r="411" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="411" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A411" s="1" t="s">
         <v>6</v>
       </c>
@@ -28469,7 +28470,7 @@
       <c r="U411" s="1"/>
       <c r="V411" s="1"/>
     </row>
-    <row r="412" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="412" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A412" s="1" t="s">
         <v>6</v>
       </c>
@@ -28523,7 +28524,7 @@
       <c r="U412" s="1"/>
       <c r="V412" s="1"/>
     </row>
-    <row r="413" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="413" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A413" s="1" t="s">
         <v>6</v>
       </c>
@@ -28575,7 +28576,7 @@
       <c r="U413" s="1"/>
       <c r="V413" s="1"/>
     </row>
-    <row r="414" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="414" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A414" s="1" t="s">
         <v>6</v>
       </c>
@@ -28627,7 +28628,7 @@
       <c r="U414" s="1"/>
       <c r="V414" s="1"/>
     </row>
-    <row r="415" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="415" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A415" s="1" t="s">
         <v>6</v>
       </c>
@@ -28679,7 +28680,7 @@
       <c r="U415" s="1"/>
       <c r="V415" s="1"/>
     </row>
-    <row r="416" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="416" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A416" s="1" t="s">
         <v>6</v>
       </c>
@@ -28731,7 +28732,7 @@
       <c r="U416" s="1"/>
       <c r="V416" s="1"/>
     </row>
-    <row r="417" spans="1:22" ht="58" x14ac:dyDescent="0.35">
+    <row r="417" spans="1:22" ht="58" hidden="1" x14ac:dyDescent="0.35">
       <c r="A417" s="1" t="s">
         <v>6</v>
       </c>
@@ -28785,7 +28786,7 @@
       <c r="U417" s="1"/>
       <c r="V417" s="1"/>
     </row>
-    <row r="418" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="418" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A418" s="1" t="s">
         <v>6</v>
       </c>
@@ -28839,7 +28840,7 @@
       <c r="U418" s="1"/>
       <c r="V418" s="1"/>
     </row>
-    <row r="419" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="419" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A419" s="1" t="s">
         <v>6</v>
       </c>
@@ -29039,7 +29040,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V419" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <autoFilter ref="A1:V419" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Philippe Ciais"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L229">
     <sortCondition ref="C2:C424"/>
   </sortState>

</xml_diff>

<commit_message>
ajout premier auteur des publis HAL
</commit_message>
<xml_diff>
--- a/Data/FairCarboN_Datas_Contacts.xlsx
+++ b/Data/FairCarboN_Datas_Contacts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dutroncj\Documents\Outils\FairCarboN_datas\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D87CDB89-D825-4788-8395-EB9D8789BBAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FCEAADA-B3E8-4D79-92A3-240B48ACC832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6316,22 +6316,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:V719"/>
+  <dimension ref="A1:V419"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.54296875" style="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.453125" style="35" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32.453125" style="35" customWidth="1"/>
-    <col min="4" max="4" width="46.81640625" style="27" hidden="1" customWidth="1"/>
-    <col min="5" max="6" width="16.7265625" style="35" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="16.7265625" style="7" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="27.1796875" style="7" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="27.81640625" style="35" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="12" style="7" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="12.26953125" style="7" hidden="1" customWidth="1"/>
-    <col min="12" max="13" width="22.90625" style="7" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="22.90625" style="7" customWidth="1"/>
+    <col min="4" max="4" width="46.81640625" style="27" customWidth="1"/>
+    <col min="5" max="6" width="16.7265625" style="35" customWidth="1"/>
+    <col min="7" max="7" width="16.7265625" style="7" customWidth="1"/>
+    <col min="8" max="8" width="27.1796875" style="7" customWidth="1"/>
+    <col min="9" max="9" width="27.81640625" style="35" customWidth="1"/>
+    <col min="10" max="10" width="12" style="7" customWidth="1"/>
+    <col min="11" max="11" width="12.26953125" style="7" customWidth="1"/>
+    <col min="12" max="14" width="22.90625" style="7" customWidth="1"/>
     <col min="15" max="15" width="22.90625" style="54" customWidth="1"/>
     <col min="16" max="17" width="48.7265625" style="7" customWidth="1"/>
     <col min="18" max="18" width="17.36328125" style="7" customWidth="1"/>
@@ -6410,7 +6408,7 @@
         <v>1761</v>
       </c>
     </row>
-    <row r="2" spans="1:22" s="2" customFormat="1" ht="188.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" s="2" customFormat="1" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -6464,7 +6462,7 @@
       <c r="U2" s="1"/>
       <c r="V2" s="1"/>
     </row>
-    <row r="3" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -6518,7 +6516,7 @@
       <c r="U3" s="1"/>
       <c r="V3" s="1"/>
     </row>
-    <row r="4" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -6572,7 +6570,7 @@
       <c r="U4" s="1"/>
       <c r="V4" s="1"/>
     </row>
-    <row r="5" spans="1:22" s="2" customFormat="1" ht="188.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" s="2" customFormat="1" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -6626,7 +6624,7 @@
       <c r="U5" s="1"/>
       <c r="V5" s="1"/>
     </row>
-    <row r="6" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -6682,7 +6680,7 @@
       <c r="U6" s="1"/>
       <c r="V6" s="1"/>
     </row>
-    <row r="7" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
@@ -6738,7 +6736,7 @@
       <c r="U7" s="1"/>
       <c r="V7" s="1"/>
     </row>
-    <row r="8" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -6792,7 +6790,7 @@
       <c r="U8" s="1"/>
       <c r="V8" s="1"/>
     </row>
-    <row r="9" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
@@ -6846,7 +6844,7 @@
       <c r="U9" s="1"/>
       <c r="V9" s="1"/>
     </row>
-    <row r="10" spans="1:22" s="2" customFormat="1" ht="159.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" s="2" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
@@ -6900,7 +6898,7 @@
       <c r="U10" s="1"/>
       <c r="V10" s="1"/>
     </row>
-    <row r="11" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>6</v>
       </c>
@@ -6954,7 +6952,7 @@
       <c r="U11" s="1"/>
       <c r="V11" s="1"/>
     </row>
-    <row r="12" spans="1:22" s="2" customFormat="1" ht="188.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" s="2" customFormat="1" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>6</v>
       </c>
@@ -7008,7 +7006,7 @@
       <c r="U12" s="1"/>
       <c r="V12" s="1"/>
     </row>
-    <row r="13" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>6</v>
       </c>
@@ -7062,7 +7060,7 @@
       <c r="U13" s="1"/>
       <c r="V13" s="1"/>
     </row>
-    <row r="14" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>6</v>
       </c>
@@ -7116,7 +7114,7 @@
       <c r="U14" s="1"/>
       <c r="V14" s="1"/>
     </row>
-    <row r="15" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>6</v>
       </c>
@@ -7172,7 +7170,7 @@
       <c r="U15" s="1"/>
       <c r="V15" s="1"/>
     </row>
-    <row r="16" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>6</v>
       </c>
@@ -7226,7 +7224,7 @@
       <c r="U16" s="1"/>
       <c r="V16" s="1"/>
     </row>
-    <row r="17" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>6</v>
       </c>
@@ -7282,7 +7280,7 @@
       <c r="U17" s="1"/>
       <c r="V17" s="1"/>
     </row>
-    <row r="18" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>6</v>
       </c>
@@ -7336,7 +7334,7 @@
       <c r="U18" s="1"/>
       <c r="V18" s="1"/>
     </row>
-    <row r="19" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>6</v>
       </c>
@@ -7390,7 +7388,7 @@
       <c r="U19" s="1"/>
       <c r="V19" s="1"/>
     </row>
-    <row r="20" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>6</v>
       </c>
@@ -7444,7 +7442,7 @@
       <c r="U20" s="1"/>
       <c r="V20" s="1"/>
     </row>
-    <row r="21" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>6</v>
       </c>
@@ -7498,7 +7496,7 @@
       <c r="U21" s="1"/>
       <c r="V21" s="1"/>
     </row>
-    <row r="22" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>6</v>
       </c>
@@ -7552,7 +7550,7 @@
       <c r="U22" s="1"/>
       <c r="V22" s="1"/>
     </row>
-    <row r="23" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>6</v>
       </c>
@@ -7606,7 +7604,7 @@
       <c r="U23" s="1"/>
       <c r="V23" s="1"/>
     </row>
-    <row r="24" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>6</v>
       </c>
@@ -7660,7 +7658,7 @@
       <c r="U24" s="1"/>
       <c r="V24" s="1"/>
     </row>
-    <row r="25" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>6</v>
       </c>
@@ -7716,7 +7714,7 @@
       <c r="U25" s="1"/>
       <c r="V25" s="1"/>
     </row>
-    <row r="26" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>6</v>
       </c>
@@ -7770,7 +7768,7 @@
       <c r="U26" s="1"/>
       <c r="V26" s="1"/>
     </row>
-    <row r="27" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>6</v>
       </c>
@@ -7824,7 +7822,7 @@
       <c r="U27" s="1"/>
       <c r="V27" s="1"/>
     </row>
-    <row r="28" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>6</v>
       </c>
@@ -7878,7 +7876,7 @@
       <c r="U28" s="1"/>
       <c r="V28" s="1"/>
     </row>
-    <row r="29" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>6</v>
       </c>
@@ -7932,7 +7930,7 @@
       <c r="U29" s="1"/>
       <c r="V29" s="1"/>
     </row>
-    <row r="30" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>6</v>
       </c>
@@ -7986,7 +7984,7 @@
       <c r="U30" s="1"/>
       <c r="V30" s="1"/>
     </row>
-    <row r="31" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>6</v>
       </c>
@@ -8040,7 +8038,7 @@
       <c r="U31" s="1"/>
       <c r="V31" s="1"/>
     </row>
-    <row r="32" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>6</v>
       </c>
@@ -8096,7 +8094,7 @@
       <c r="U32" s="1"/>
       <c r="V32" s="1"/>
     </row>
-    <row r="33" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>6</v>
       </c>
@@ -8150,7 +8148,7 @@
       <c r="U33" s="1"/>
       <c r="V33" s="1"/>
     </row>
-    <row r="34" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>6</v>
       </c>
@@ -8204,7 +8202,7 @@
       <c r="U34" s="1"/>
       <c r="V34" s="1"/>
     </row>
-    <row r="35" spans="1:22" s="2" customFormat="1" ht="232" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:22" s="2" customFormat="1" ht="232" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>6</v>
       </c>
@@ -8260,7 +8258,7 @@
       <c r="U35" s="1"/>
       <c r="V35" s="1"/>
     </row>
-    <row r="36" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>6</v>
       </c>
@@ -8314,7 +8312,7 @@
       <c r="U36" s="1"/>
       <c r="V36" s="1"/>
     </row>
-    <row r="37" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>6</v>
       </c>
@@ -8368,7 +8366,7 @@
       <c r="U37" s="1"/>
       <c r="V37" s="1"/>
     </row>
-    <row r="38" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>6</v>
       </c>
@@ -8422,7 +8420,7 @@
       <c r="U38" s="1"/>
       <c r="V38" s="1"/>
     </row>
-    <row r="39" spans="1:22" s="2" customFormat="1" ht="159.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:22" s="2" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>6</v>
       </c>
@@ -8476,7 +8474,7 @@
       <c r="U39" s="1"/>
       <c r="V39" s="1"/>
     </row>
-    <row r="40" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>6</v>
       </c>
@@ -8530,7 +8528,7 @@
       <c r="U40" s="1"/>
       <c r="V40" s="1"/>
     </row>
-    <row r="41" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>6</v>
       </c>
@@ -8584,7 +8582,7 @@
       <c r="U41" s="1"/>
       <c r="V41" s="1"/>
     </row>
-    <row r="42" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>6</v>
       </c>
@@ -8638,7 +8636,7 @@
       <c r="U42" s="1"/>
       <c r="V42" s="1"/>
     </row>
-    <row r="43" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>6</v>
       </c>
@@ -8692,7 +8690,7 @@
       <c r="U43" s="1"/>
       <c r="V43" s="1"/>
     </row>
-    <row r="44" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>6</v>
       </c>
@@ -8746,7 +8744,7 @@
       <c r="U44" s="1"/>
       <c r="V44" s="1"/>
     </row>
-    <row r="45" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>6</v>
       </c>
@@ -8800,7 +8798,7 @@
       <c r="U45" s="1"/>
       <c r="V45" s="1"/>
     </row>
-    <row r="46" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>6</v>
       </c>
@@ -8854,7 +8852,7 @@
       <c r="U46" s="1"/>
       <c r="V46" s="1"/>
     </row>
-    <row r="47" spans="1:22" s="2" customFormat="1" ht="275.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:22" s="2" customFormat="1" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>6</v>
       </c>
@@ -8912,7 +8910,7 @@
       <c r="U47" s="1"/>
       <c r="V47" s="1"/>
     </row>
-    <row r="48" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>6</v>
       </c>
@@ -8966,7 +8964,7 @@
       <c r="U48" s="1"/>
       <c r="V48" s="1"/>
     </row>
-    <row r="49" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>6</v>
       </c>
@@ -9022,7 +9020,7 @@
       <c r="U49" s="1"/>
       <c r="V49" s="1"/>
     </row>
-    <row r="50" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>6</v>
       </c>
@@ -9076,7 +9074,7 @@
       <c r="U50" s="1"/>
       <c r="V50" s="1"/>
     </row>
-    <row r="51" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>6</v>
       </c>
@@ -9130,7 +9128,7 @@
       <c r="U51" s="1"/>
       <c r="V51" s="1"/>
     </row>
-    <row r="52" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>6</v>
       </c>
@@ -9184,7 +9182,7 @@
       <c r="U52" s="1"/>
       <c r="V52" s="1"/>
     </row>
-    <row r="53" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>6</v>
       </c>
@@ -9238,7 +9236,7 @@
       <c r="U53" s="1"/>
       <c r="V53" s="1"/>
     </row>
-    <row r="54" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>6</v>
       </c>
@@ -9292,7 +9290,7 @@
       <c r="U54" s="1"/>
       <c r="V54" s="1"/>
     </row>
-    <row r="55" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>6</v>
       </c>
@@ -9346,7 +9344,7 @@
       <c r="U55" s="1"/>
       <c r="V55" s="1"/>
     </row>
-    <row r="56" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>6</v>
       </c>
@@ -9400,7 +9398,7 @@
       <c r="U56" s="1"/>
       <c r="V56" s="1"/>
     </row>
-    <row r="57" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>6</v>
       </c>
@@ -9454,7 +9452,7 @@
       <c r="U57" s="1"/>
       <c r="V57" s="1"/>
     </row>
-    <row r="58" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>6</v>
       </c>
@@ -9508,7 +9506,7 @@
       <c r="U58" s="1"/>
       <c r="V58" s="1"/>
     </row>
-    <row r="59" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>6</v>
       </c>
@@ -9564,7 +9562,7 @@
       <c r="U59" s="1"/>
       <c r="V59" s="1"/>
     </row>
-    <row r="60" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>6</v>
       </c>
@@ -9620,7 +9618,7 @@
       <c r="U60" s="1"/>
       <c r="V60" s="1"/>
     </row>
-    <row r="61" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>6</v>
       </c>
@@ -9676,7 +9674,7 @@
       <c r="U61" s="1"/>
       <c r="V61" s="1"/>
     </row>
-    <row r="62" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>6</v>
       </c>
@@ -9732,7 +9730,7 @@
       <c r="U62" s="1"/>
       <c r="V62" s="1"/>
     </row>
-    <row r="63" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>6</v>
       </c>
@@ -9786,7 +9784,7 @@
       <c r="U63" s="1"/>
       <c r="V63" s="1"/>
     </row>
-    <row r="64" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>6</v>
       </c>
@@ -9842,7 +9840,7 @@
       <c r="U64" s="1"/>
       <c r="V64" s="1"/>
     </row>
-    <row r="65" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>6</v>
       </c>
@@ -9954,7 +9952,7 @@
       <c r="U66" s="1"/>
       <c r="V66" s="1"/>
     </row>
-    <row r="67" spans="1:22" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:22" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>6</v>
       </c>
@@ -10008,7 +10006,7 @@
       <c r="U67" s="1"/>
       <c r="V67" s="1"/>
     </row>
-    <row r="68" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>6</v>
       </c>
@@ -10064,7 +10062,7 @@
       <c r="U68" s="1"/>
       <c r="V68" s="1"/>
     </row>
-    <row r="69" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>6</v>
       </c>
@@ -10118,7 +10116,7 @@
       <c r="U69" s="1"/>
       <c r="V69" s="1"/>
     </row>
-    <row r="70" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>6</v>
       </c>
@@ -10172,7 +10170,7 @@
       <c r="U70" s="1"/>
       <c r="V70" s="1"/>
     </row>
-    <row r="71" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>6</v>
       </c>
@@ -10226,7 +10224,7 @@
       <c r="U71" s="1"/>
       <c r="V71" s="1"/>
     </row>
-    <row r="72" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>6</v>
       </c>
@@ -10280,7 +10278,7 @@
       <c r="U72" s="1"/>
       <c r="V72" s="1"/>
     </row>
-    <row r="73" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>6</v>
       </c>
@@ -10334,7 +10332,7 @@
       <c r="U73" s="1"/>
       <c r="V73" s="1"/>
     </row>
-    <row r="74" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>6</v>
       </c>
@@ -10388,7 +10386,7 @@
       <c r="U74" s="1"/>
       <c r="V74" s="1"/>
     </row>
-    <row r="75" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>6</v>
       </c>
@@ -10442,7 +10440,7 @@
       <c r="U75" s="1"/>
       <c r="V75" s="1"/>
     </row>
-    <row r="76" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>6</v>
       </c>
@@ -10496,7 +10494,7 @@
       <c r="U76" s="1"/>
       <c r="V76" s="1"/>
     </row>
-    <row r="77" spans="1:22" s="2" customFormat="1" ht="27.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:22" s="2" customFormat="1" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>6</v>
       </c>
@@ -10552,7 +10550,7 @@
       <c r="U77" s="1"/>
       <c r="V77" s="1"/>
     </row>
-    <row r="78" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>6</v>
       </c>
@@ -10606,7 +10604,7 @@
       <c r="U78" s="1"/>
       <c r="V78" s="1"/>
     </row>
-    <row r="79" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>6</v>
       </c>
@@ -10660,7 +10658,7 @@
       <c r="U79" s="1"/>
       <c r="V79" s="1"/>
     </row>
-    <row r="80" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>6</v>
       </c>
@@ -10714,7 +10712,7 @@
       <c r="U80" s="1"/>
       <c r="V80" s="1"/>
     </row>
-    <row r="81" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>6</v>
       </c>
@@ -10770,7 +10768,7 @@
       <c r="U81" s="1"/>
       <c r="V81" s="1"/>
     </row>
-    <row r="82" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>6</v>
       </c>
@@ -10824,7 +10822,7 @@
       <c r="U82" s="1"/>
       <c r="V82" s="1"/>
     </row>
-    <row r="83" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>6</v>
       </c>
@@ -10880,7 +10878,7 @@
       <c r="U83" s="1"/>
       <c r="V83" s="1"/>
     </row>
-    <row r="84" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>6</v>
       </c>
@@ -10934,7 +10932,7 @@
       <c r="U84" s="1"/>
       <c r="V84" s="1"/>
     </row>
-    <row r="85" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>6</v>
       </c>
@@ -10990,7 +10988,7 @@
       <c r="U85" s="1"/>
       <c r="V85" s="1"/>
     </row>
-    <row r="86" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>6</v>
       </c>
@@ -11046,7 +11044,7 @@
       <c r="U86" s="1"/>
       <c r="V86" s="1"/>
     </row>
-    <row r="87" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>6</v>
       </c>
@@ -11100,7 +11098,7 @@
       <c r="U87" s="1"/>
       <c r="V87" s="1"/>
     </row>
-    <row r="88" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>6</v>
       </c>
@@ -11154,7 +11152,7 @@
       <c r="U88" s="1"/>
       <c r="V88" s="1"/>
     </row>
-    <row r="89" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>6</v>
       </c>
@@ -11206,7 +11204,7 @@
       <c r="U89" s="1"/>
       <c r="V89" s="1"/>
     </row>
-    <row r="90" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>6</v>
       </c>
@@ -11262,7 +11260,7 @@
       <c r="U90" s="1"/>
       <c r="V90" s="1"/>
     </row>
-    <row r="91" spans="1:22" s="2" customFormat="1" ht="159.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:22" s="2" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>6</v>
       </c>
@@ -11316,7 +11314,7 @@
       <c r="U91" s="1"/>
       <c r="V91" s="1"/>
     </row>
-    <row r="92" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>6</v>
       </c>
@@ -11370,7 +11368,7 @@
       <c r="U92" s="1"/>
       <c r="V92" s="1"/>
     </row>
-    <row r="93" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
         <v>6</v>
       </c>
@@ -11424,7 +11422,7 @@
       <c r="U93" s="1"/>
       <c r="V93" s="1"/>
     </row>
-    <row r="94" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
         <v>6</v>
       </c>
@@ -11478,7 +11476,7 @@
       <c r="U94" s="1"/>
       <c r="V94" s="1"/>
     </row>
-    <row r="95" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
         <v>6</v>
       </c>
@@ -11532,7 +11530,7 @@
       <c r="U95" s="1"/>
       <c r="V95" s="1"/>
     </row>
-    <row r="96" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>6</v>
       </c>
@@ -11586,7 +11584,7 @@
       <c r="U96" s="1"/>
       <c r="V96" s="1"/>
     </row>
-    <row r="97" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>6</v>
       </c>
@@ -11640,7 +11638,7 @@
       <c r="U97" s="1"/>
       <c r="V97" s="1"/>
     </row>
-    <row r="98" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>6</v>
       </c>
@@ -11694,7 +11692,7 @@
       <c r="U98" s="1"/>
       <c r="V98" s="1"/>
     </row>
-    <row r="99" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>6</v>
       </c>
@@ -11748,7 +11746,7 @@
       <c r="U99" s="1"/>
       <c r="V99" s="1"/>
     </row>
-    <row r="100" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
         <v>6</v>
       </c>
@@ -11802,7 +11800,7 @@
       <c r="U100" s="1"/>
       <c r="V100" s="1"/>
     </row>
-    <row r="101" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>6</v>
       </c>
@@ -11854,7 +11852,7 @@
       <c r="U101" s="1"/>
       <c r="V101" s="1"/>
     </row>
-    <row r="102" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
         <v>6</v>
       </c>
@@ -11910,7 +11908,7 @@
       <c r="U102" s="1"/>
       <c r="V102" s="1"/>
     </row>
-    <row r="103" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>6</v>
       </c>
@@ -11964,7 +11962,7 @@
       <c r="U103" s="1"/>
       <c r="V103" s="1"/>
     </row>
-    <row r="104" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
         <v>6</v>
       </c>
@@ -12016,7 +12014,7 @@
       <c r="U104" s="1"/>
       <c r="V104" s="1"/>
     </row>
-    <row r="105" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>6</v>
       </c>
@@ -12072,7 +12070,7 @@
       <c r="U105" s="1"/>
       <c r="V105" s="1"/>
     </row>
-    <row r="106" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>6</v>
       </c>
@@ -12126,7 +12124,7 @@
       <c r="U106" s="1"/>
       <c r="V106" s="1"/>
     </row>
-    <row r="107" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
         <v>6</v>
       </c>
@@ -12180,7 +12178,7 @@
       <c r="U107" s="1"/>
       <c r="V107" s="1"/>
     </row>
-    <row r="108" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
         <v>6</v>
       </c>
@@ -12234,7 +12232,7 @@
       <c r="U108" s="1"/>
       <c r="V108" s="1"/>
     </row>
-    <row r="109" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
         <v>6</v>
       </c>
@@ -12286,7 +12284,7 @@
       <c r="U109" s="1"/>
       <c r="V109" s="1"/>
     </row>
-    <row r="110" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
         <v>6</v>
       </c>
@@ -12340,7 +12338,7 @@
       <c r="U110" s="1"/>
       <c r="V110" s="1"/>
     </row>
-    <row r="111" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>6</v>
       </c>
@@ -12396,7 +12394,7 @@
       <c r="U111" s="1"/>
       <c r="V111" s="1"/>
     </row>
-    <row r="112" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>6</v>
       </c>
@@ -12450,7 +12448,7 @@
       <c r="U112" s="1"/>
       <c r="V112" s="1"/>
     </row>
-    <row r="113" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
         <v>6</v>
       </c>
@@ -12504,7 +12502,7 @@
       <c r="U113" s="1"/>
       <c r="V113" s="1"/>
     </row>
-    <row r="114" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
         <v>6</v>
       </c>
@@ -12558,7 +12556,7 @@
       <c r="U114" s="1"/>
       <c r="V114" s="1"/>
     </row>
-    <row r="115" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A115" s="1" t="s">
         <v>6</v>
       </c>
@@ -12612,7 +12610,7 @@
       <c r="U115" s="1"/>
       <c r="V115" s="1"/>
     </row>
-    <row r="116" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
         <v>6</v>
       </c>
@@ -12666,7 +12664,7 @@
       <c r="U116" s="1"/>
       <c r="V116" s="1"/>
     </row>
-    <row r="117" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
         <v>6</v>
       </c>
@@ -12720,7 +12718,7 @@
       <c r="U117" s="1"/>
       <c r="V117" s="1"/>
     </row>
-    <row r="118" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
         <v>6</v>
       </c>
@@ -12774,7 +12772,7 @@
       <c r="U118" s="1"/>
       <c r="V118" s="1"/>
     </row>
-    <row r="119" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
         <v>6</v>
       </c>
@@ -12828,7 +12826,7 @@
       <c r="U119" s="1"/>
       <c r="V119" s="1"/>
     </row>
-    <row r="120" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
         <v>6</v>
       </c>
@@ -12882,7 +12880,7 @@
       <c r="U120" s="1"/>
       <c r="V120" s="1"/>
     </row>
-    <row r="121" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
         <v>6</v>
       </c>
@@ -12938,7 +12936,7 @@
       <c r="U121" s="1"/>
       <c r="V121" s="1"/>
     </row>
-    <row r="122" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A122" s="1" t="s">
         <v>6</v>
       </c>
@@ -12992,7 +12990,7 @@
       <c r="U122" s="1"/>
       <c r="V122" s="1"/>
     </row>
-    <row r="123" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
         <v>6</v>
       </c>
@@ -13046,7 +13044,7 @@
       <c r="U123" s="1"/>
       <c r="V123" s="1"/>
     </row>
-    <row r="124" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
         <v>6</v>
       </c>
@@ -13100,7 +13098,7 @@
       <c r="U124" s="1"/>
       <c r="V124" s="1"/>
     </row>
-    <row r="125" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
         <v>6</v>
       </c>
@@ -13154,7 +13152,7 @@
       <c r="U125" s="1"/>
       <c r="V125" s="1"/>
     </row>
-    <row r="126" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
         <v>6</v>
       </c>
@@ -13208,7 +13206,7 @@
       <c r="U126" s="1"/>
       <c r="V126" s="1"/>
     </row>
-    <row r="127" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
         <v>6</v>
       </c>
@@ -13262,7 +13260,7 @@
       <c r="U127" s="1"/>
       <c r="V127" s="1"/>
     </row>
-    <row r="128" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A128" s="1" t="s">
         <v>6</v>
       </c>
@@ -13316,7 +13314,7 @@
       <c r="U128" s="1"/>
       <c r="V128" s="1"/>
     </row>
-    <row r="129" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A129" s="1" t="s">
         <v>6</v>
       </c>
@@ -13370,7 +13368,7 @@
       <c r="U129" s="1"/>
       <c r="V129" s="1"/>
     </row>
-    <row r="130" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A130" s="1" t="s">
         <v>6</v>
       </c>
@@ -13424,7 +13422,7 @@
       <c r="U130" s="1"/>
       <c r="V130" s="1"/>
     </row>
-    <row r="131" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A131" s="1" t="s">
         <v>6</v>
       </c>
@@ -13478,7 +13476,7 @@
       <c r="U131" s="1"/>
       <c r="V131" s="1"/>
     </row>
-    <row r="132" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A132" s="1" t="s">
         <v>6</v>
       </c>
@@ -13532,7 +13530,7 @@
       <c r="U132" s="1"/>
       <c r="V132" s="1"/>
     </row>
-    <row r="133" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A133" s="1" t="s">
         <v>6</v>
       </c>
@@ -13586,7 +13584,7 @@
       <c r="U133" s="1"/>
       <c r="V133" s="1"/>
     </row>
-    <row r="134" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A134" s="1" t="s">
         <v>6</v>
       </c>
@@ -13640,7 +13638,7 @@
       <c r="U134" s="1"/>
       <c r="V134" s="1"/>
     </row>
-    <row r="135" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
         <v>6</v>
       </c>
@@ -13694,7 +13692,7 @@
       <c r="U135" s="1"/>
       <c r="V135" s="1"/>
     </row>
-    <row r="136" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A136" s="1" t="s">
         <v>6</v>
       </c>
@@ -13748,7 +13746,7 @@
       <c r="U136" s="1"/>
       <c r="V136" s="1"/>
     </row>
-    <row r="137" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
         <v>6</v>
       </c>
@@ -13802,7 +13800,7 @@
       <c r="U137" s="1"/>
       <c r="V137" s="1"/>
     </row>
-    <row r="138" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
         <v>6</v>
       </c>
@@ -13856,7 +13854,7 @@
       <c r="U138" s="1"/>
       <c r="V138" s="1"/>
     </row>
-    <row r="139" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A139" s="1" t="s">
         <v>6</v>
       </c>
@@ -13910,7 +13908,7 @@
       <c r="U139" s="1"/>
       <c r="V139" s="1"/>
     </row>
-    <row r="140" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A140" s="1" t="s">
         <v>6</v>
       </c>
@@ -13966,7 +13964,7 @@
       <c r="U140" s="1"/>
       <c r="V140" s="1"/>
     </row>
-    <row r="141" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A141" s="1" t="s">
         <v>6</v>
       </c>
@@ -14020,7 +14018,7 @@
       <c r="U141" s="1"/>
       <c r="V141" s="1"/>
     </row>
-    <row r="142" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A142" s="1" t="s">
         <v>6</v>
       </c>
@@ -14074,7 +14072,7 @@
       <c r="U142" s="1"/>
       <c r="V142" s="1"/>
     </row>
-    <row r="143" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A143" s="1" t="s">
         <v>6</v>
       </c>
@@ -14128,7 +14126,7 @@
       <c r="U143" s="1"/>
       <c r="V143" s="1"/>
     </row>
-    <row r="144" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A144" s="1" t="s">
         <v>6</v>
       </c>
@@ -14184,7 +14182,7 @@
       <c r="U144" s="1"/>
       <c r="V144" s="1"/>
     </row>
-    <row r="145" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
         <v>6</v>
       </c>
@@ -14238,7 +14236,7 @@
       <c r="U145" s="1"/>
       <c r="V145" s="1"/>
     </row>
-    <row r="146" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A146" s="1" t="s">
         <v>6</v>
       </c>
@@ -14292,7 +14290,7 @@
       <c r="U146" s="1"/>
       <c r="V146" s="1"/>
     </row>
-    <row r="147" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A147" s="1" t="s">
         <v>6</v>
       </c>
@@ -14348,7 +14346,7 @@
       <c r="U147" s="1"/>
       <c r="V147" s="1"/>
     </row>
-    <row r="148" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A148" s="1" t="s">
         <v>6</v>
       </c>
@@ -14402,7 +14400,7 @@
       <c r="U148" s="1"/>
       <c r="V148" s="1"/>
     </row>
-    <row r="149" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A149" s="1" t="s">
         <v>6</v>
       </c>
@@ -14456,7 +14454,7 @@
       <c r="U149" s="1"/>
       <c r="V149" s="1"/>
     </row>
-    <row r="150" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A150" s="1" t="s">
         <v>6</v>
       </c>
@@ -14510,7 +14508,7 @@
       <c r="U150" s="1"/>
       <c r="V150" s="1"/>
     </row>
-    <row r="151" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A151" s="1" t="s">
         <v>6</v>
       </c>
@@ -14564,7 +14562,7 @@
       <c r="U151" s="1"/>
       <c r="V151" s="1"/>
     </row>
-    <row r="152" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A152" s="1" t="s">
         <v>6</v>
       </c>
@@ -14618,7 +14616,7 @@
       <c r="U152" s="1"/>
       <c r="V152" s="1"/>
     </row>
-    <row r="153" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A153" s="1" t="s">
         <v>6</v>
       </c>
@@ -14672,7 +14670,7 @@
       <c r="U153" s="1"/>
       <c r="V153" s="1"/>
     </row>
-    <row r="154" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A154" s="1" t="s">
         <v>6</v>
       </c>
@@ -14726,7 +14724,7 @@
       <c r="U154" s="1"/>
       <c r="V154" s="1"/>
     </row>
-    <row r="155" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A155" s="1" t="s">
         <v>6</v>
       </c>
@@ -14780,7 +14778,7 @@
       <c r="U155" s="1"/>
       <c r="V155" s="1"/>
     </row>
-    <row r="156" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A156" s="1" t="s">
         <v>6</v>
       </c>
@@ -14834,7 +14832,7 @@
       <c r="U156" s="1"/>
       <c r="V156" s="1"/>
     </row>
-    <row r="157" spans="1:22" s="2" customFormat="1" ht="65" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:22" s="2" customFormat="1" ht="65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A157" s="1" t="s">
         <v>6</v>
       </c>
@@ -14898,7 +14896,7 @@
         <v>1764</v>
       </c>
     </row>
-    <row r="158" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A158" s="1" t="s">
         <v>6</v>
       </c>
@@ -14954,7 +14952,7 @@
       <c r="U158" s="1"/>
       <c r="V158" s="1"/>
     </row>
-    <row r="159" spans="1:22" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:22" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A159" s="1" t="s">
         <v>6</v>
       </c>
@@ -15010,7 +15008,7 @@
       <c r="U159" s="1"/>
       <c r="V159" s="1"/>
     </row>
-    <row r="160" spans="1:22" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:22" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A160" s="1" t="s">
         <v>6</v>
       </c>
@@ -15066,7 +15064,7 @@
       <c r="U160" s="1"/>
       <c r="V160" s="1"/>
     </row>
-    <row r="161" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
       <c r="A161" s="1" t="s">
         <v>6</v>
       </c>
@@ -15122,7 +15120,7 @@
       <c r="U161" s="1"/>
       <c r="V161" s="1"/>
     </row>
-    <row r="162" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
       <c r="A162" s="1" t="s">
         <v>6</v>
       </c>
@@ -15180,7 +15178,7 @@
       <c r="U162" s="1"/>
       <c r="V162" s="1"/>
     </row>
-    <row r="163" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A163" s="1" t="s">
         <v>6</v>
       </c>
@@ -15236,7 +15234,7 @@
       <c r="U163" s="1"/>
       <c r="V163" s="1"/>
     </row>
-    <row r="164" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A164" s="1" t="s">
         <v>6</v>
       </c>
@@ -15292,7 +15290,7 @@
       <c r="U164" s="1"/>
       <c r="V164" s="1"/>
     </row>
-    <row r="165" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A165" s="1" t="s">
         <v>6</v>
       </c>
@@ -15348,7 +15346,7 @@
       <c r="U165" s="1"/>
       <c r="V165" s="1"/>
     </row>
-    <row r="166" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A166" s="1" t="s">
         <v>6</v>
       </c>
@@ -15404,7 +15402,7 @@
       <c r="U166" s="1"/>
       <c r="V166" s="1"/>
     </row>
-    <row r="167" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
       <c r="A167" s="1" t="s">
         <v>6</v>
       </c>
@@ -15462,7 +15460,7 @@
       <c r="U167" s="1"/>
       <c r="V167" s="1"/>
     </row>
-    <row r="168" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
       <c r="A168" s="1" t="s">
         <v>6</v>
       </c>
@@ -15522,7 +15520,7 @@
       <c r="U168" s="1"/>
       <c r="V168" s="1"/>
     </row>
-    <row r="169" spans="1:22" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:22" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A169" s="1" t="s">
         <v>6</v>
       </c>
@@ -15578,7 +15576,7 @@
       <c r="U169" s="1"/>
       <c r="V169" s="1"/>
     </row>
-    <row r="170" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A170" s="1" t="s">
         <v>6</v>
       </c>
@@ -15634,7 +15632,7 @@
       <c r="U170" s="1"/>
       <c r="V170" s="1"/>
     </row>
-    <row r="171" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
       <c r="A171" s="1" t="s">
         <v>6</v>
       </c>
@@ -15690,7 +15688,7 @@
       <c r="U171" s="1"/>
       <c r="V171" s="1"/>
     </row>
-    <row r="172" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A172" s="1" t="s">
         <v>6</v>
       </c>
@@ -15746,7 +15744,7 @@
       <c r="U172" s="1"/>
       <c r="V172" s="1"/>
     </row>
-    <row r="173" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A173" s="1" t="s">
         <v>6</v>
       </c>
@@ -15800,7 +15798,7 @@
       <c r="U173" s="1"/>
       <c r="V173" s="1"/>
     </row>
-    <row r="174" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A174" s="1" t="s">
         <v>6</v>
       </c>
@@ -15854,7 +15852,7 @@
       <c r="U174" s="1"/>
       <c r="V174" s="1"/>
     </row>
-    <row r="175" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A175" s="1" t="s">
         <v>6</v>
       </c>
@@ -15908,7 +15906,7 @@
       <c r="U175" s="1"/>
       <c r="V175" s="1"/>
     </row>
-    <row r="176" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A176" s="1" t="s">
         <v>6</v>
       </c>
@@ -15962,7 +15960,7 @@
       <c r="U176" s="1"/>
       <c r="V176" s="1"/>
     </row>
-    <row r="177" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A177" s="1" t="s">
         <v>6</v>
       </c>
@@ -16016,7 +16014,7 @@
       <c r="U177" s="1"/>
       <c r="V177" s="1"/>
     </row>
-    <row r="178" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
       <c r="A178" s="1" t="s">
         <v>6</v>
       </c>
@@ -16070,7 +16068,7 @@
       <c r="U178" s="1"/>
       <c r="V178" s="1"/>
     </row>
-    <row r="179" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
       <c r="A179" s="1" t="s">
         <v>6</v>
       </c>
@@ -16124,7 +16122,7 @@
       <c r="U179" s="1"/>
       <c r="V179" s="1"/>
     </row>
-    <row r="180" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A180" s="1" t="s">
         <v>6</v>
       </c>
@@ -16178,7 +16176,7 @@
       <c r="U180" s="1"/>
       <c r="V180" s="1"/>
     </row>
-    <row r="181" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
       <c r="A181" s="1" t="s">
         <v>6</v>
       </c>
@@ -16234,7 +16232,7 @@
       <c r="U181" s="1"/>
       <c r="V181" s="1"/>
     </row>
-    <row r="182" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A182" s="1" t="s">
         <v>6</v>
       </c>
@@ -16288,7 +16286,7 @@
       <c r="U182" s="1"/>
       <c r="V182" s="1"/>
     </row>
-    <row r="183" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A183" s="1" t="s">
         <v>6</v>
       </c>
@@ -16342,7 +16340,7 @@
       <c r="U183" s="1"/>
       <c r="V183" s="1"/>
     </row>
-    <row r="184" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A184" s="1" t="s">
         <v>6</v>
       </c>
@@ -16396,7 +16394,7 @@
       <c r="U184" s="1"/>
       <c r="V184" s="1"/>
     </row>
-    <row r="185" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A185" s="1" t="s">
         <v>6</v>
       </c>
@@ -16450,7 +16448,7 @@
       <c r="U185" s="1"/>
       <c r="V185" s="1"/>
     </row>
-    <row r="186" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A186" s="1" t="s">
         <v>6</v>
       </c>
@@ -16506,7 +16504,7 @@
       <c r="U186" s="1"/>
       <c r="V186" s="1"/>
     </row>
-    <row r="187" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A187" s="1" t="s">
         <v>6</v>
       </c>
@@ -16560,7 +16558,7 @@
       <c r="U187" s="1"/>
       <c r="V187" s="1"/>
     </row>
-    <row r="188" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A188" s="1" t="s">
         <v>6</v>
       </c>
@@ -16614,7 +16612,7 @@
       <c r="U188" s="1"/>
       <c r="V188" s="1"/>
     </row>
-    <row r="189" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A189" s="1" t="s">
         <v>6</v>
       </c>
@@ -16668,7 +16666,7 @@
       <c r="U189" s="1"/>
       <c r="V189" s="1"/>
     </row>
-    <row r="190" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A190" s="1" t="s">
         <v>6</v>
       </c>
@@ -16722,7 +16720,7 @@
       <c r="U190" s="1"/>
       <c r="V190" s="1"/>
     </row>
-    <row r="191" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A191" s="1" t="s">
         <v>6</v>
       </c>
@@ -16776,7 +16774,7 @@
       <c r="U191" s="1"/>
       <c r="V191" s="1"/>
     </row>
-    <row r="192" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A192" s="1" t="s">
         <v>6</v>
       </c>
@@ -16830,7 +16828,7 @@
       <c r="U192" s="1"/>
       <c r="V192" s="1"/>
     </row>
-    <row r="193" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A193" s="1" t="s">
         <v>6</v>
       </c>
@@ -16884,7 +16882,7 @@
       <c r="U193" s="1"/>
       <c r="V193" s="1"/>
     </row>
-    <row r="194" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A194" s="1" t="s">
         <v>6</v>
       </c>
@@ -16938,7 +16936,7 @@
       <c r="U194" s="1"/>
       <c r="V194" s="1"/>
     </row>
-    <row r="195" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A195" s="1" t="s">
         <v>6</v>
       </c>
@@ -16992,7 +16990,7 @@
       <c r="U195" s="1"/>
       <c r="V195" s="1"/>
     </row>
-    <row r="196" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A196" s="1" t="s">
         <v>6</v>
       </c>
@@ -17046,7 +17044,7 @@
       <c r="U196" s="1"/>
       <c r="V196" s="1"/>
     </row>
-    <row r="197" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A197" s="1" t="s">
         <v>6</v>
       </c>
@@ -17100,7 +17098,7 @@
       <c r="U197" s="1"/>
       <c r="V197" s="1"/>
     </row>
-    <row r="198" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A198" s="1" t="s">
         <v>6</v>
       </c>
@@ -17154,7 +17152,7 @@
       <c r="U198" s="1"/>
       <c r="V198" s="1"/>
     </row>
-    <row r="199" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A199" s="1" t="s">
         <v>6</v>
       </c>
@@ -17208,7 +17206,7 @@
       <c r="U199" s="1"/>
       <c r="V199" s="1"/>
     </row>
-    <row r="200" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A200" s="1" t="s">
         <v>6</v>
       </c>
@@ -17262,7 +17260,7 @@
       <c r="U200" s="1"/>
       <c r="V200" s="1"/>
     </row>
-    <row r="201" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A201" s="1" t="s">
         <v>6</v>
       </c>
@@ -17316,7 +17314,7 @@
       <c r="U201" s="1"/>
       <c r="V201" s="1"/>
     </row>
-    <row r="202" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A202" s="1" t="s">
         <v>6</v>
       </c>
@@ -17370,7 +17368,7 @@
       <c r="U202" s="1"/>
       <c r="V202" s="1"/>
     </row>
-    <row r="203" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A203" s="1" t="s">
         <v>6</v>
       </c>
@@ -17424,7 +17422,7 @@
       <c r="U203" s="1"/>
       <c r="V203" s="1"/>
     </row>
-    <row r="204" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A204" s="1" t="s">
         <v>6</v>
       </c>
@@ -17478,7 +17476,7 @@
       <c r="U204" s="1"/>
       <c r="V204" s="1"/>
     </row>
-    <row r="205" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A205" s="1" t="s">
         <v>6</v>
       </c>
@@ -17532,7 +17530,7 @@
       <c r="U205" s="1"/>
       <c r="V205" s="1"/>
     </row>
-    <row r="206" spans="1:22" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:22" ht="87" x14ac:dyDescent="0.35">
       <c r="A206" s="1" t="s">
         <v>6</v>
       </c>
@@ -17586,7 +17584,7 @@
       <c r="U206" s="1"/>
       <c r="V206" s="1"/>
     </row>
-    <row r="207" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A207" s="1" t="s">
         <v>6</v>
       </c>
@@ -17640,7 +17638,7 @@
       <c r="U207" s="1"/>
       <c r="V207" s="1"/>
     </row>
-    <row r="208" spans="1:22" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:22" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A208" s="1" t="s">
         <v>6</v>
       </c>
@@ -17694,7 +17692,7 @@
       <c r="U208" s="1"/>
       <c r="V208" s="1"/>
     </row>
-    <row r="209" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A209" s="1" t="s">
         <v>6</v>
       </c>
@@ -17748,7 +17746,7 @@
       <c r="U209" s="1"/>
       <c r="V209" s="1"/>
     </row>
-    <row r="210" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A210" s="1" t="s">
         <v>6</v>
       </c>
@@ -17802,7 +17800,7 @@
       <c r="U210" s="1"/>
       <c r="V210" s="1"/>
     </row>
-    <row r="211" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A211" s="1" t="s">
         <v>6</v>
       </c>
@@ -17854,7 +17852,7 @@
       <c r="U211" s="1"/>
       <c r="V211" s="1"/>
     </row>
-    <row r="212" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A212" s="1" t="s">
         <v>6</v>
       </c>
@@ -17906,7 +17904,7 @@
       <c r="U212" s="1"/>
       <c r="V212" s="1"/>
     </row>
-    <row r="213" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A213" s="1" t="s">
         <v>6</v>
       </c>
@@ -17960,7 +17958,7 @@
       <c r="U213" s="1"/>
       <c r="V213" s="1"/>
     </row>
-    <row r="214" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A214" s="1" t="s">
         <v>6</v>
       </c>
@@ -18012,7 +18010,7 @@
       <c r="U214" s="1"/>
       <c r="V214" s="1"/>
     </row>
-    <row r="215" spans="1:22" s="2" customFormat="1" ht="159.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:22" s="2" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A215" s="1" t="s">
         <v>6</v>
       </c>
@@ -18064,7 +18062,7 @@
       <c r="U215" s="1"/>
       <c r="V215" s="1"/>
     </row>
-    <row r="216" spans="1:22" s="2" customFormat="1" ht="188.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:22" s="2" customFormat="1" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A216" s="1" t="s">
         <v>6</v>
       </c>
@@ -18116,7 +18114,7 @@
       <c r="U216" s="1"/>
       <c r="V216" s="1"/>
     </row>
-    <row r="217" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A217" s="1" t="s">
         <v>6</v>
       </c>
@@ -18168,7 +18166,7 @@
       <c r="U217" s="1"/>
       <c r="V217" s="1"/>
     </row>
-    <row r="218" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A218" s="1" t="s">
         <v>6</v>
       </c>
@@ -18222,7 +18220,7 @@
       <c r="U218" s="1"/>
       <c r="V218" s="1"/>
     </row>
-    <row r="219" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A219" s="1" t="s">
         <v>6</v>
       </c>
@@ -18276,7 +18274,7 @@
       <c r="U219" s="1"/>
       <c r="V219" s="1"/>
     </row>
-    <row r="220" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A220" s="1" t="s">
         <v>6</v>
       </c>
@@ -18332,7 +18330,7 @@
       <c r="U220" s="1"/>
       <c r="V220" s="1"/>
     </row>
-    <row r="221" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A221" s="1" t="s">
         <v>6</v>
       </c>
@@ -18386,7 +18384,7 @@
       <c r="U221" s="1"/>
       <c r="V221" s="1"/>
     </row>
-    <row r="222" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A222" s="1" t="s">
         <v>6</v>
       </c>
@@ -18438,7 +18436,7 @@
       <c r="U222" s="1"/>
       <c r="V222" s="1"/>
     </row>
-    <row r="223" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A223" s="1" t="s">
         <v>6</v>
       </c>
@@ -18492,7 +18490,7 @@
       <c r="U223" s="1"/>
       <c r="V223" s="1"/>
     </row>
-    <row r="224" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A224" s="1" t="s">
         <v>6</v>
       </c>
@@ -18548,7 +18546,7 @@
       <c r="U224" s="1"/>
       <c r="V224" s="1"/>
     </row>
-    <row r="225" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A225" s="1" t="s">
         <v>6</v>
       </c>
@@ -18604,7 +18602,7 @@
       <c r="U225" s="1"/>
       <c r="V225" s="1"/>
     </row>
-    <row r="226" spans="1:22" s="2" customFormat="1" ht="159.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:22" s="2" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A226" s="1" t="s">
         <v>6</v>
       </c>
@@ -18658,7 +18656,7 @@
       <c r="U226" s="1"/>
       <c r="V226" s="1"/>
     </row>
-    <row r="227" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A227" s="1" t="s">
         <v>6</v>
       </c>
@@ -18710,7 +18708,7 @@
       <c r="U227" s="1"/>
       <c r="V227" s="1"/>
     </row>
-    <row r="228" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A228" s="1" t="s">
         <v>6</v>
       </c>
@@ -18762,7 +18760,7 @@
       <c r="U228" s="1"/>
       <c r="V228" s="1"/>
     </row>
-    <row r="229" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A229" s="1" t="s">
         <v>6</v>
       </c>
@@ -18818,7 +18816,7 @@
       <c r="U229" s="1"/>
       <c r="V229" s="1"/>
     </row>
-    <row r="230" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A230" s="1" t="s">
         <v>6</v>
       </c>
@@ -18872,7 +18870,7 @@
       <c r="U230" s="1"/>
       <c r="V230" s="1"/>
     </row>
-    <row r="231" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A231" s="1" t="s">
         <v>6</v>
       </c>
@@ -18924,7 +18922,7 @@
       <c r="U231" s="1"/>
       <c r="V231" s="1"/>
     </row>
-    <row r="232" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A232" s="1" t="s">
         <v>6</v>
       </c>
@@ -18976,7 +18974,7 @@
       <c r="U232" s="1"/>
       <c r="V232" s="1"/>
     </row>
-    <row r="233" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A233" s="1" t="s">
         <v>6</v>
       </c>
@@ -19028,7 +19026,7 @@
       <c r="U233" s="1"/>
       <c r="V233" s="1"/>
     </row>
-    <row r="234" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A234" s="1" t="s">
         <v>6</v>
       </c>
@@ -19080,7 +19078,7 @@
       <c r="U234" s="1"/>
       <c r="V234" s="1"/>
     </row>
-    <row r="235" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A235" s="1" t="s">
         <v>6</v>
       </c>
@@ -19132,7 +19130,7 @@
       <c r="U235" s="1"/>
       <c r="V235" s="1"/>
     </row>
-    <row r="236" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A236" s="1" t="s">
         <v>6</v>
       </c>
@@ -19184,7 +19182,7 @@
       <c r="U236" s="1"/>
       <c r="V236" s="1"/>
     </row>
-    <row r="237" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A237" s="1" t="s">
         <v>6</v>
       </c>
@@ -19236,7 +19234,7 @@
       <c r="U237" s="1"/>
       <c r="V237" s="1"/>
     </row>
-    <row r="238" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A238" s="1" t="s">
         <v>6</v>
       </c>
@@ -19290,7 +19288,7 @@
       <c r="U238" s="1"/>
       <c r="V238" s="1"/>
     </row>
-    <row r="239" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A239" s="1" t="s">
         <v>6</v>
       </c>
@@ -19342,7 +19340,7 @@
       <c r="U239" s="1"/>
       <c r="V239" s="1"/>
     </row>
-    <row r="240" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A240" s="1" t="s">
         <v>6</v>
       </c>
@@ -19394,7 +19392,7 @@
       <c r="U240" s="1"/>
       <c r="V240" s="1"/>
     </row>
-    <row r="241" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A241" s="1" t="s">
         <v>6</v>
       </c>
@@ -19446,7 +19444,7 @@
       <c r="U241" s="1"/>
       <c r="V241" s="1"/>
     </row>
-    <row r="242" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A242" s="1" t="s">
         <v>6</v>
       </c>
@@ -19498,7 +19496,7 @@
       <c r="U242" s="1"/>
       <c r="V242" s="1"/>
     </row>
-    <row r="243" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A243" s="1" t="s">
         <v>6</v>
       </c>
@@ -19550,7 +19548,7 @@
       <c r="U243" s="1"/>
       <c r="V243" s="1"/>
     </row>
-    <row r="244" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A244" s="1" t="s">
         <v>6</v>
       </c>
@@ -19602,7 +19600,7 @@
       <c r="U244" s="1"/>
       <c r="V244" s="1"/>
     </row>
-    <row r="245" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A245" s="1" t="s">
         <v>6</v>
       </c>
@@ -19656,7 +19654,7 @@
       <c r="U245" s="1"/>
       <c r="V245" s="1"/>
     </row>
-    <row r="246" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A246" s="1" t="s">
         <v>6</v>
       </c>
@@ -19710,7 +19708,7 @@
       <c r="U246" s="1"/>
       <c r="V246" s="1"/>
     </row>
-    <row r="247" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A247" s="1" t="s">
         <v>6</v>
       </c>
@@ -19762,7 +19760,7 @@
       <c r="U247" s="1"/>
       <c r="V247" s="1"/>
     </row>
-    <row r="248" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A248" s="1" t="s">
         <v>6</v>
       </c>
@@ -19814,7 +19812,7 @@
       <c r="U248" s="1"/>
       <c r="V248" s="1"/>
     </row>
-    <row r="249" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A249" s="1" t="s">
         <v>6</v>
       </c>
@@ -19866,7 +19864,7 @@
       <c r="U249" s="1"/>
       <c r="V249" s="1"/>
     </row>
-    <row r="250" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A250" s="1" t="s">
         <v>6</v>
       </c>
@@ -19918,7 +19916,7 @@
       <c r="U250" s="1"/>
       <c r="V250" s="1"/>
     </row>
-    <row r="251" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A251" s="1" t="s">
         <v>6</v>
       </c>
@@ -19970,7 +19968,7 @@
       <c r="U251" s="1"/>
       <c r="V251" s="1"/>
     </row>
-    <row r="252" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A252" s="1" t="s">
         <v>6</v>
       </c>
@@ -20022,7 +20020,7 @@
       <c r="U252" s="1"/>
       <c r="V252" s="1"/>
     </row>
-    <row r="253" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A253" s="1" t="s">
         <v>6</v>
       </c>
@@ -20078,7 +20076,7 @@
       <c r="U253" s="1"/>
       <c r="V253" s="1"/>
     </row>
-    <row r="254" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A254" s="1" t="s">
         <v>6</v>
       </c>
@@ -20132,7 +20130,7 @@
       <c r="U254" s="1"/>
       <c r="V254" s="1"/>
     </row>
-    <row r="255" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A255" s="1" t="s">
         <v>6</v>
       </c>
@@ -20186,7 +20184,7 @@
       <c r="U255" s="1"/>
       <c r="V255" s="1"/>
     </row>
-    <row r="256" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A256" s="1" t="s">
         <v>6</v>
       </c>
@@ -20238,7 +20236,7 @@
       <c r="U256" s="1"/>
       <c r="V256" s="1"/>
     </row>
-    <row r="257" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A257" s="1" t="s">
         <v>6</v>
       </c>
@@ -20290,7 +20288,7 @@
       <c r="U257" s="1"/>
       <c r="V257" s="1"/>
     </row>
-    <row r="258" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A258" s="1" t="s">
         <v>6</v>
       </c>
@@ -20342,7 +20340,7 @@
       <c r="U258" s="1"/>
       <c r="V258" s="1"/>
     </row>
-    <row r="259" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A259" s="1" t="s">
         <v>6</v>
       </c>
@@ -20394,7 +20392,7 @@
       <c r="U259" s="1"/>
       <c r="V259" s="1"/>
     </row>
-    <row r="260" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A260" s="1" t="s">
         <v>6</v>
       </c>
@@ -20446,7 +20444,7 @@
       <c r="U260" s="1"/>
       <c r="V260" s="1"/>
     </row>
-    <row r="261" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A261" s="1" t="s">
         <v>6</v>
       </c>
@@ -20500,7 +20498,7 @@
       <c r="U261" s="1"/>
       <c r="V261" s="1"/>
     </row>
-    <row r="262" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A262" s="1" t="s">
         <v>6</v>
       </c>
@@ -20552,7 +20550,7 @@
       <c r="U262" s="1"/>
       <c r="V262" s="1"/>
     </row>
-    <row r="263" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A263" s="1" t="s">
         <v>6</v>
       </c>
@@ -20604,7 +20602,7 @@
       <c r="U263" s="1"/>
       <c r="V263" s="1"/>
     </row>
-    <row r="264" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A264" s="1" t="s">
         <v>6</v>
       </c>
@@ -20656,7 +20654,7 @@
       <c r="U264" s="1"/>
       <c r="V264" s="1"/>
     </row>
-    <row r="265" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A265" s="1" t="s">
         <v>6</v>
       </c>
@@ -20708,7 +20706,7 @@
       <c r="U265" s="1"/>
       <c r="V265" s="1"/>
     </row>
-    <row r="266" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A266" s="1" t="s">
         <v>6</v>
       </c>
@@ -20760,7 +20758,7 @@
       <c r="U266" s="1"/>
       <c r="V266" s="1"/>
     </row>
-    <row r="267" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A267" s="1" t="s">
         <v>6</v>
       </c>
@@ -20812,7 +20810,7 @@
       <c r="U267" s="1"/>
       <c r="V267" s="1"/>
     </row>
-    <row r="268" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A268" s="1" t="s">
         <v>6</v>
       </c>
@@ -20866,7 +20864,7 @@
       <c r="U268" s="1"/>
       <c r="V268" s="1"/>
     </row>
-    <row r="269" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A269" s="1" t="s">
         <v>6</v>
       </c>
@@ -20918,7 +20916,7 @@
       <c r="U269" s="1"/>
       <c r="V269" s="1"/>
     </row>
-    <row r="270" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A270" s="1" t="s">
         <v>6</v>
       </c>
@@ -20970,7 +20968,7 @@
       <c r="U270" s="1"/>
       <c r="V270" s="1"/>
     </row>
-    <row r="271" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A271" s="1" t="s">
         <v>6</v>
       </c>
@@ -21022,7 +21020,7 @@
       <c r="U271" s="1"/>
       <c r="V271" s="1"/>
     </row>
-    <row r="272" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A272" s="1" t="s">
         <v>6</v>
       </c>
@@ -21076,7 +21074,7 @@
       <c r="U272" s="1"/>
       <c r="V272" s="1"/>
     </row>
-    <row r="273" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A273" s="1" t="s">
         <v>6</v>
       </c>
@@ -21130,7 +21128,7 @@
       <c r="U273" s="1"/>
       <c r="V273" s="1"/>
     </row>
-    <row r="274" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A274" s="1" t="s">
         <v>6</v>
       </c>
@@ -21184,7 +21182,7 @@
       <c r="U274" s="1"/>
       <c r="V274" s="1"/>
     </row>
-    <row r="275" spans="1:22" s="2" customFormat="1" ht="377" hidden="1" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:22" s="2" customFormat="1" ht="377" x14ac:dyDescent="0.35">
       <c r="A275" s="1" t="s">
         <v>6</v>
       </c>
@@ -21240,7 +21238,7 @@
       <c r="U275" s="1"/>
       <c r="V275" s="1"/>
     </row>
-    <row r="276" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A276" s="1" t="s">
         <v>6</v>
       </c>
@@ -21294,7 +21292,7 @@
       <c r="U276" s="1"/>
       <c r="V276" s="1"/>
     </row>
-    <row r="277" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A277" s="1" t="s">
         <v>6</v>
       </c>
@@ -21348,7 +21346,7 @@
       <c r="U277" s="1"/>
       <c r="V277" s="1"/>
     </row>
-    <row r="278" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A278" s="1" t="s">
         <v>6</v>
       </c>
@@ -21402,7 +21400,7 @@
       <c r="U278" s="1"/>
       <c r="V278" s="1"/>
     </row>
-    <row r="279" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A279" s="1" t="s">
         <v>6</v>
       </c>
@@ -21456,7 +21454,7 @@
       <c r="U279" s="1"/>
       <c r="V279" s="1"/>
     </row>
-    <row r="280" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A280" s="1" t="s">
         <v>6</v>
       </c>
@@ -21512,7 +21510,7 @@
       <c r="U280" s="1"/>
       <c r="V280" s="1"/>
     </row>
-    <row r="281" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A281" s="1" t="s">
         <v>6</v>
       </c>
@@ -21566,7 +21564,7 @@
       <c r="U281" s="1"/>
       <c r="V281" s="1"/>
     </row>
-    <row r="282" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A282" s="1" t="s">
         <v>6</v>
       </c>
@@ -21620,7 +21618,7 @@
       <c r="U282" s="1"/>
       <c r="V282" s="1"/>
     </row>
-    <row r="283" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A283" s="1" t="s">
         <v>6</v>
       </c>
@@ -21674,7 +21672,7 @@
       <c r="U283" s="1"/>
       <c r="V283" s="1"/>
     </row>
-    <row r="284" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A284" s="1" t="s">
         <v>6</v>
       </c>
@@ -21728,7 +21726,7 @@
       <c r="U284" s="1"/>
       <c r="V284" s="1"/>
     </row>
-    <row r="285" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A285" s="1" t="s">
         <v>6</v>
       </c>
@@ -21780,7 +21778,7 @@
       <c r="U285" s="1"/>
       <c r="V285" s="1"/>
     </row>
-    <row r="286" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A286" s="1" t="s">
         <v>6</v>
       </c>
@@ -21832,7 +21830,7 @@
       <c r="U286" s="1"/>
       <c r="V286" s="1"/>
     </row>
-    <row r="287" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A287" s="1" t="s">
         <v>6</v>
       </c>
@@ -21884,7 +21882,7 @@
       <c r="U287" s="1"/>
       <c r="V287" s="1"/>
     </row>
-    <row r="288" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A288" s="1" t="s">
         <v>6</v>
       </c>
@@ -21936,7 +21934,7 @@
       <c r="U288" s="1"/>
       <c r="V288" s="1"/>
     </row>
-    <row r="289" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A289" s="1" t="s">
         <v>6</v>
       </c>
@@ -21988,7 +21986,7 @@
       <c r="U289" s="1"/>
       <c r="V289" s="1"/>
     </row>
-    <row r="290" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A290" s="1" t="s">
         <v>6</v>
       </c>
@@ -22040,7 +22038,7 @@
       <c r="U290" s="1"/>
       <c r="V290" s="1"/>
     </row>
-    <row r="291" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A291" s="1" t="s">
         <v>6</v>
       </c>
@@ -22092,7 +22090,7 @@
       <c r="U291" s="1"/>
       <c r="V291" s="1"/>
     </row>
-    <row r="292" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A292" s="1" t="s">
         <v>6</v>
       </c>
@@ -22144,7 +22142,7 @@
       <c r="U292" s="1"/>
       <c r="V292" s="1"/>
     </row>
-    <row r="293" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A293" s="1" t="s">
         <v>6</v>
       </c>
@@ -22196,7 +22194,7 @@
       <c r="U293" s="1"/>
       <c r="V293" s="1"/>
     </row>
-    <row r="294" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A294" s="1" t="s">
         <v>6</v>
       </c>
@@ -22248,7 +22246,7 @@
       <c r="U294" s="1"/>
       <c r="V294" s="1"/>
     </row>
-    <row r="295" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A295" s="1" t="s">
         <v>6</v>
       </c>
@@ -22300,7 +22298,7 @@
       <c r="U295" s="1"/>
       <c r="V295" s="1"/>
     </row>
-    <row r="296" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A296" s="1" t="s">
         <v>6</v>
       </c>
@@ -22352,7 +22350,7 @@
       <c r="U296" s="1"/>
       <c r="V296" s="1"/>
     </row>
-    <row r="297" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A297" s="1" t="s">
         <v>6</v>
       </c>
@@ -22404,7 +22402,7 @@
       <c r="U297" s="1"/>
       <c r="V297" s="1"/>
     </row>
-    <row r="298" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A298" s="1" t="s">
         <v>6</v>
       </c>
@@ -22456,7 +22454,7 @@
       <c r="U298" s="1"/>
       <c r="V298" s="1"/>
     </row>
-    <row r="299" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A299" s="1" t="s">
         <v>6</v>
       </c>
@@ -22508,7 +22506,7 @@
       <c r="U299" s="1"/>
       <c r="V299" s="1"/>
     </row>
-    <row r="300" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A300" s="1" t="s">
         <v>6</v>
       </c>
@@ -22560,7 +22558,7 @@
       <c r="U300" s="1"/>
       <c r="V300" s="1"/>
     </row>
-    <row r="301" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A301" s="1" t="s">
         <v>6</v>
       </c>
@@ -22612,7 +22610,7 @@
       <c r="U301" s="1"/>
       <c r="V301" s="1"/>
     </row>
-    <row r="302" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A302" s="1" t="s">
         <v>6</v>
       </c>
@@ -22664,7 +22662,7 @@
       <c r="U302" s="1"/>
       <c r="V302" s="1"/>
     </row>
-    <row r="303" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A303" s="1" t="s">
         <v>6</v>
       </c>
@@ -22718,7 +22716,7 @@
       <c r="U303" s="1"/>
       <c r="V303" s="1"/>
     </row>
-    <row r="304" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A304" s="1" t="s">
         <v>6</v>
       </c>
@@ -22770,7 +22768,7 @@
       <c r="U304" s="1"/>
       <c r="V304" s="1"/>
     </row>
-    <row r="305" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A305" s="1" t="s">
         <v>6</v>
       </c>
@@ -22822,7 +22820,7 @@
       <c r="U305" s="1"/>
       <c r="V305" s="1"/>
     </row>
-    <row r="306" spans="1:22" s="2" customFormat="1" ht="76.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:22" s="2" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A306" s="1" t="s">
         <v>6</v>
       </c>
@@ -22874,7 +22872,7 @@
       <c r="U306" s="1"/>
       <c r="V306" s="1"/>
     </row>
-    <row r="307" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A307" s="1" t="s">
         <v>6</v>
       </c>
@@ -22926,7 +22924,7 @@
       <c r="U307" s="1"/>
       <c r="V307" s="1"/>
     </row>
-    <row r="308" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A308" s="1" t="s">
         <v>6</v>
       </c>
@@ -22978,7 +22976,7 @@
       <c r="U308" s="1"/>
       <c r="V308" s="1"/>
     </row>
-    <row r="309" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A309" s="1" t="s">
         <v>6</v>
       </c>
@@ -23030,7 +23028,7 @@
       <c r="U309" s="1"/>
       <c r="V309" s="1"/>
     </row>
-    <row r="310" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A310" s="1" t="s">
         <v>6</v>
       </c>
@@ -23082,7 +23080,7 @@
       <c r="U310" s="1"/>
       <c r="V310" s="1"/>
     </row>
-    <row r="311" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A311" s="1" t="s">
         <v>6</v>
       </c>
@@ -23134,7 +23132,7 @@
       <c r="U311" s="1"/>
       <c r="V311" s="1"/>
     </row>
-    <row r="312" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A312" s="1" t="s">
         <v>6</v>
       </c>
@@ -23186,7 +23184,7 @@
       <c r="U312" s="1"/>
       <c r="V312" s="1"/>
     </row>
-    <row r="313" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A313" s="1" t="s">
         <v>6</v>
       </c>
@@ -23238,7 +23236,7 @@
       <c r="U313" s="1"/>
       <c r="V313" s="1"/>
     </row>
-    <row r="314" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A314" s="1" t="s">
         <v>6</v>
       </c>
@@ -23294,7 +23292,7 @@
       <c r="U314" s="1"/>
       <c r="V314" s="1"/>
     </row>
-    <row r="315" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A315" s="1" t="s">
         <v>6</v>
       </c>
@@ -23352,7 +23350,7 @@
       <c r="U315" s="1"/>
       <c r="V315" s="1"/>
     </row>
-    <row r="316" spans="1:22" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:22" ht="87" x14ac:dyDescent="0.35">
       <c r="A316" s="1" t="s">
         <v>6</v>
       </c>
@@ -23408,7 +23406,7 @@
       <c r="U316" s="1"/>
       <c r="V316" s="1"/>
     </row>
-    <row r="317" spans="1:22" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:22" ht="87" x14ac:dyDescent="0.35">
       <c r="A317" s="1" t="s">
         <v>6</v>
       </c>
@@ -23462,7 +23460,7 @@
       <c r="U317" s="1"/>
       <c r="V317" s="1"/>
     </row>
-    <row r="318" spans="1:22" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:22" ht="87" x14ac:dyDescent="0.35">
       <c r="A318" s="1" t="s">
         <v>6</v>
       </c>
@@ -23512,7 +23510,7 @@
       <c r="U318" s="1"/>
       <c r="V318" s="1"/>
     </row>
-    <row r="319" spans="1:22" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:22" ht="87" x14ac:dyDescent="0.35">
       <c r="A319" s="1" t="s">
         <v>6</v>
       </c>
@@ -23568,7 +23566,7 @@
       <c r="U319" s="1"/>
       <c r="V319" s="1"/>
     </row>
-    <row r="320" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A320" s="1" t="s">
         <v>6</v>
       </c>
@@ -23620,7 +23618,7 @@
       <c r="U320" s="1"/>
       <c r="V320" s="1"/>
     </row>
-    <row r="321" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A321" s="1" t="s">
         <v>6</v>
       </c>
@@ -23674,7 +23672,7 @@
       <c r="U321" s="1"/>
       <c r="V321" s="1"/>
     </row>
-    <row r="322" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A322" s="1" t="s">
         <v>6</v>
       </c>
@@ -23726,7 +23724,7 @@
       <c r="U322" s="1"/>
       <c r="V322" s="1"/>
     </row>
-    <row r="323" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A323" s="1" t="s">
         <v>6</v>
       </c>
@@ -23782,7 +23780,7 @@
       <c r="U323" s="1"/>
       <c r="V323" s="1"/>
     </row>
-    <row r="324" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A324" s="1" t="s">
         <v>6</v>
       </c>
@@ -23834,7 +23832,7 @@
       <c r="U324" s="1"/>
       <c r="V324" s="1"/>
     </row>
-    <row r="325" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A325" s="1" t="s">
         <v>6</v>
       </c>
@@ -23886,7 +23884,7 @@
       <c r="U325" s="1"/>
       <c r="V325" s="1"/>
     </row>
-    <row r="326" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A326" s="1" t="s">
         <v>6</v>
       </c>
@@ -23938,7 +23936,7 @@
       <c r="U326" s="1"/>
       <c r="V326" s="1"/>
     </row>
-    <row r="327" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A327" s="1" t="s">
         <v>6</v>
       </c>
@@ -23990,7 +23988,7 @@
       <c r="U327" s="1"/>
       <c r="V327" s="1"/>
     </row>
-    <row r="328" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A328" s="1" t="s">
         <v>6</v>
       </c>
@@ -24042,7 +24040,7 @@
       <c r="U328" s="1"/>
       <c r="V328" s="1"/>
     </row>
-    <row r="329" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A329" s="1" t="s">
         <v>6</v>
       </c>
@@ -24094,7 +24092,7 @@
       <c r="U329" s="1"/>
       <c r="V329" s="1"/>
     </row>
-    <row r="330" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A330" s="1" t="s">
         <v>6</v>
       </c>
@@ -24146,7 +24144,7 @@
       <c r="U330" s="1"/>
       <c r="V330" s="1"/>
     </row>
-    <row r="331" spans="1:22" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:22" ht="58" x14ac:dyDescent="0.35">
       <c r="A331" s="1" t="s">
         <v>6</v>
       </c>
@@ -24198,7 +24196,7 @@
       <c r="U331" s="1"/>
       <c r="V331" s="1"/>
     </row>
-    <row r="332" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A332" s="1" t="s">
         <v>6</v>
       </c>
@@ -24252,7 +24250,7 @@
       <c r="U332" s="1"/>
       <c r="V332" s="1"/>
     </row>
-    <row r="333" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A333" s="1" t="s">
         <v>6</v>
       </c>
@@ -24306,7 +24304,7 @@
       <c r="U333" s="1"/>
       <c r="V333" s="1"/>
     </row>
-    <row r="334" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A334" s="1" t="s">
         <v>6</v>
       </c>
@@ -24360,7 +24358,7 @@
       <c r="U334" s="1"/>
       <c r="V334" s="1"/>
     </row>
-    <row r="335" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A335" s="1" t="s">
         <v>6</v>
       </c>
@@ -24412,7 +24410,7 @@
       <c r="U335" s="1"/>
       <c r="V335" s="1"/>
     </row>
-    <row r="336" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A336" s="1" t="s">
         <v>6</v>
       </c>
@@ -24464,7 +24462,7 @@
       <c r="U336" s="1"/>
       <c r="V336" s="1"/>
     </row>
-    <row r="337" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A337" s="1" t="s">
         <v>6</v>
       </c>
@@ -24516,7 +24514,7 @@
       <c r="U337" s="1"/>
       <c r="V337" s="1"/>
     </row>
-    <row r="338" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A338" s="1" t="s">
         <v>6</v>
       </c>
@@ -24570,7 +24568,7 @@
       <c r="U338" s="1"/>
       <c r="V338" s="1"/>
     </row>
-    <row r="339" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A339" s="1" t="s">
         <v>6</v>
       </c>
@@ -24622,7 +24620,7 @@
       <c r="U339" s="1"/>
       <c r="V339" s="1"/>
     </row>
-    <row r="340" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A340" s="1" t="s">
         <v>6</v>
       </c>
@@ -24674,7 +24672,7 @@
       <c r="U340" s="1"/>
       <c r="V340" s="1"/>
     </row>
-    <row r="341" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A341" s="1" t="s">
         <v>6</v>
       </c>
@@ -24726,7 +24724,7 @@
       <c r="U341" s="1"/>
       <c r="V341" s="1"/>
     </row>
-    <row r="342" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A342" s="1" t="s">
         <v>6</v>
       </c>
@@ -24780,7 +24778,7 @@
       <c r="U342" s="1"/>
       <c r="V342" s="1"/>
     </row>
-    <row r="343" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A343" s="1" t="s">
         <v>6</v>
       </c>
@@ -24834,7 +24832,7 @@
       <c r="U343" s="1"/>
       <c r="V343" s="1"/>
     </row>
-    <row r="344" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A344" s="1" t="s">
         <v>6</v>
       </c>
@@ -24886,7 +24884,7 @@
       <c r="U344" s="1"/>
       <c r="V344" s="1"/>
     </row>
-    <row r="345" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A345" s="1" t="s">
         <v>6</v>
       </c>
@@ -24938,7 +24936,7 @@
       <c r="U345" s="1"/>
       <c r="V345" s="1"/>
     </row>
-    <row r="346" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A346" s="1" t="s">
         <v>6</v>
       </c>
@@ -24990,7 +24988,7 @@
       <c r="U346" s="1"/>
       <c r="V346" s="1"/>
     </row>
-    <row r="347" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A347" s="1" t="s">
         <v>6</v>
       </c>
@@ -25044,7 +25042,7 @@
       <c r="U347" s="1"/>
       <c r="V347" s="1"/>
     </row>
-    <row r="348" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A348" s="1" t="s">
         <v>6</v>
       </c>
@@ -25096,7 +25094,7 @@
       <c r="U348" s="1"/>
       <c r="V348" s="1"/>
     </row>
-    <row r="349" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A349" s="1" t="s">
         <v>6</v>
       </c>
@@ -25150,7 +25148,7 @@
       <c r="U349" s="1"/>
       <c r="V349" s="1"/>
     </row>
-    <row r="350" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A350" s="1" t="s">
         <v>6</v>
       </c>
@@ -25202,7 +25200,7 @@
       <c r="U350" s="1"/>
       <c r="V350" s="1"/>
     </row>
-    <row r="351" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A351" s="1" t="s">
         <v>6</v>
       </c>
@@ -25254,7 +25252,7 @@
       <c r="U351" s="1"/>
       <c r="V351" s="1"/>
     </row>
-    <row r="352" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A352" s="1" t="s">
         <v>6</v>
       </c>
@@ -25308,7 +25306,7 @@
       <c r="U352" s="1"/>
       <c r="V352" s="1"/>
     </row>
-    <row r="353" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A353" s="1" t="s">
         <v>6</v>
       </c>
@@ -25358,7 +25356,7 @@
       <c r="U353" s="1"/>
       <c r="V353" s="1"/>
     </row>
-    <row r="354" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A354" s="1" t="s">
         <v>6</v>
       </c>
@@ -25408,7 +25406,7 @@
       <c r="U354" s="1"/>
       <c r="V354" s="1"/>
     </row>
-    <row r="355" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A355" s="1" t="s">
         <v>6</v>
       </c>
@@ -25460,7 +25458,7 @@
       <c r="U355" s="1"/>
       <c r="V355" s="1"/>
     </row>
-    <row r="356" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A356" s="1" t="s">
         <v>6</v>
       </c>
@@ -25512,7 +25510,7 @@
       <c r="U356" s="1"/>
       <c r="V356" s="1"/>
     </row>
-    <row r="357" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A357" s="1" t="s">
         <v>6</v>
       </c>
@@ -25564,7 +25562,7 @@
       <c r="U357" s="1"/>
       <c r="V357" s="1"/>
     </row>
-    <row r="358" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A358" s="1" t="s">
         <v>6</v>
       </c>
@@ -25616,7 +25614,7 @@
       <c r="U358" s="1"/>
       <c r="V358" s="1"/>
     </row>
-    <row r="359" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A359" s="1" t="s">
         <v>6</v>
       </c>
@@ -25670,7 +25668,7 @@
       <c r="U359" s="1"/>
       <c r="V359" s="1"/>
     </row>
-    <row r="360" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A360" s="1" t="s">
         <v>6</v>
       </c>
@@ -25722,7 +25720,7 @@
       <c r="U360" s="1"/>
       <c r="V360" s="1"/>
     </row>
-    <row r="361" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A361" s="1" t="s">
         <v>6</v>
       </c>
@@ -25774,7 +25772,7 @@
       <c r="U361" s="1"/>
       <c r="V361" s="1"/>
     </row>
-    <row r="362" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A362" s="1" t="s">
         <v>6</v>
       </c>
@@ -25826,7 +25824,7 @@
       <c r="U362" s="1"/>
       <c r="V362" s="1"/>
     </row>
-    <row r="363" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A363" s="1" t="s">
         <v>6</v>
       </c>
@@ -25880,7 +25878,7 @@
       <c r="U363" s="1"/>
       <c r="V363" s="1"/>
     </row>
-    <row r="364" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A364" s="1" t="s">
         <v>6</v>
       </c>
@@ -25932,7 +25930,7 @@
       <c r="U364" s="1"/>
       <c r="V364" s="1"/>
     </row>
-    <row r="365" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A365" s="1" t="s">
         <v>6</v>
       </c>
@@ -25984,7 +25982,7 @@
       <c r="U365" s="1"/>
       <c r="V365" s="1"/>
     </row>
-    <row r="366" spans="1:22" s="2" customFormat="1" ht="159.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:22" s="2" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A366" s="1" t="s">
         <v>6</v>
       </c>
@@ -26036,7 +26034,7 @@
       <c r="U366" s="1"/>
       <c r="V366" s="1"/>
     </row>
-    <row r="367" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A367" s="1" t="s">
         <v>6</v>
       </c>
@@ -26088,7 +26086,7 @@
       <c r="U367" s="1"/>
       <c r="V367" s="1"/>
     </row>
-    <row r="368" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A368" s="1" t="s">
         <v>6</v>
       </c>
@@ -26140,7 +26138,7 @@
       <c r="U368" s="1"/>
       <c r="V368" s="1"/>
     </row>
-    <row r="369" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A369" s="1" t="s">
         <v>6</v>
       </c>
@@ -26192,7 +26190,7 @@
       <c r="U369" s="1"/>
       <c r="V369" s="1"/>
     </row>
-    <row r="370" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A370" s="1" t="s">
         <v>6</v>
       </c>
@@ -26246,7 +26244,7 @@
       <c r="U370" s="1"/>
       <c r="V370" s="1"/>
     </row>
-    <row r="371" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A371" s="1" t="s">
         <v>6</v>
       </c>
@@ -26298,7 +26296,7 @@
       <c r="U371" s="1"/>
       <c r="V371" s="1"/>
     </row>
-    <row r="372" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A372" s="1" t="s">
         <v>6</v>
       </c>
@@ -26350,7 +26348,7 @@
       <c r="U372" s="1"/>
       <c r="V372" s="1"/>
     </row>
-    <row r="373" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A373" s="1" t="s">
         <v>6</v>
       </c>
@@ -26402,7 +26400,7 @@
       <c r="U373" s="1"/>
       <c r="V373" s="1"/>
     </row>
-    <row r="374" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A374" s="1" t="s">
         <v>6</v>
       </c>
@@ -26456,7 +26454,7 @@
       <c r="U374" s="1"/>
       <c r="V374" s="1"/>
     </row>
-    <row r="375" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A375" s="1" t="s">
         <v>6</v>
       </c>
@@ -26510,7 +26508,7 @@
       <c r="U375" s="1"/>
       <c r="V375" s="1"/>
     </row>
-    <row r="376" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A376" s="1" t="s">
         <v>6</v>
       </c>
@@ -26566,7 +26564,7 @@
       <c r="U376" s="1"/>
       <c r="V376" s="1"/>
     </row>
-    <row r="377" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A377" s="1" t="s">
         <v>6</v>
       </c>
@@ -26620,7 +26618,7 @@
       <c r="U377" s="1"/>
       <c r="V377" s="1"/>
     </row>
-    <row r="378" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A378" s="1" t="s">
         <v>6</v>
       </c>
@@ -26674,7 +26672,7 @@
       <c r="U378" s="1"/>
       <c r="V378" s="1"/>
     </row>
-    <row r="379" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A379" s="1" t="s">
         <v>6</v>
       </c>
@@ -26730,7 +26728,7 @@
       <c r="U379" s="1"/>
       <c r="V379" s="1"/>
     </row>
-    <row r="380" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A380" s="1" t="s">
         <v>6</v>
       </c>
@@ -26786,7 +26784,7 @@
       <c r="U380" s="1"/>
       <c r="V380" s="1"/>
     </row>
-    <row r="381" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A381" s="1" t="s">
         <v>6</v>
       </c>
@@ -26840,7 +26838,7 @@
       <c r="U381" s="1"/>
       <c r="V381" s="1"/>
     </row>
-    <row r="382" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A382" s="1" t="s">
         <v>6</v>
       </c>
@@ -26896,7 +26894,7 @@
       <c r="U382" s="1"/>
       <c r="V382" s="1"/>
     </row>
-    <row r="383" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="383" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A383" s="1" t="s">
         <v>6</v>
       </c>
@@ -26950,7 +26948,7 @@
       <c r="U383" s="1"/>
       <c r="V383" s="1"/>
     </row>
-    <row r="384" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="384" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A384" s="1" t="s">
         <v>6</v>
       </c>
@@ -27002,7 +27000,7 @@
       <c r="U384" s="1"/>
       <c r="V384" s="1"/>
     </row>
-    <row r="385" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="385" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A385" s="1" t="s">
         <v>6</v>
       </c>
@@ -27056,7 +27054,7 @@
       <c r="U385" s="1"/>
       <c r="V385" s="1"/>
     </row>
-    <row r="386" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="386" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A386" s="1" t="s">
         <v>6</v>
       </c>
@@ -27112,7 +27110,7 @@
       <c r="U386" s="1"/>
       <c r="V386" s="1"/>
     </row>
-    <row r="387" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="387" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A387" s="1" t="s">
         <v>6</v>
       </c>
@@ -27166,7 +27164,7 @@
       <c r="U387" s="1"/>
       <c r="V387" s="1"/>
     </row>
-    <row r="388" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="388" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A388" s="1" t="s">
         <v>6</v>
       </c>
@@ -27220,7 +27218,7 @@
       <c r="U388" s="1"/>
       <c r="V388" s="1"/>
     </row>
-    <row r="389" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="389" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A389" s="1" t="s">
         <v>6</v>
       </c>
@@ -27274,7 +27272,7 @@
       <c r="U389" s="1"/>
       <c r="V389" s="1"/>
     </row>
-    <row r="390" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="390" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A390" s="1" t="s">
         <v>6</v>
       </c>
@@ -27328,7 +27326,7 @@
       <c r="U390" s="1"/>
       <c r="V390" s="1"/>
     </row>
-    <row r="391" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="391" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A391" s="1" t="s">
         <v>6</v>
       </c>
@@ -27384,7 +27382,7 @@
       <c r="U391" s="1"/>
       <c r="V391" s="1"/>
     </row>
-    <row r="392" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="392" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A392" s="1" t="s">
         <v>6</v>
       </c>
@@ -27438,7 +27436,7 @@
       <c r="U392" s="1"/>
       <c r="V392" s="1"/>
     </row>
-    <row r="393" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="393" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A393" s="1" t="s">
         <v>6</v>
       </c>
@@ -27492,7 +27490,7 @@
       <c r="U393" s="1"/>
       <c r="V393" s="1"/>
     </row>
-    <row r="394" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="394" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A394" s="1" t="s">
         <v>6</v>
       </c>
@@ -27546,7 +27544,7 @@
       <c r="U394" s="1"/>
       <c r="V394" s="1"/>
     </row>
-    <row r="395" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="395" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A395" s="1" t="s">
         <v>6</v>
       </c>
@@ -27600,7 +27598,7 @@
       <c r="U395" s="1"/>
       <c r="V395" s="1"/>
     </row>
-    <row r="396" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="396" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A396" s="1" t="s">
         <v>6</v>
       </c>
@@ -27656,7 +27654,7 @@
       <c r="U396" s="1"/>
       <c r="V396" s="1"/>
     </row>
-    <row r="397" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="397" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A397" s="1" t="s">
         <v>6</v>
       </c>
@@ -27712,7 +27710,7 @@
       <c r="U397" s="1"/>
       <c r="V397" s="1"/>
     </row>
-    <row r="398" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="398" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A398" s="1" t="s">
         <v>6</v>
       </c>
@@ -27766,7 +27764,7 @@
       <c r="U398" s="1"/>
       <c r="V398" s="1"/>
     </row>
-    <row r="399" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="399" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A399" s="1" t="s">
         <v>6</v>
       </c>
@@ -27820,7 +27818,7 @@
       <c r="U399" s="1"/>
       <c r="V399" s="1"/>
     </row>
-    <row r="400" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="400" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A400" s="1" t="s">
         <v>6</v>
       </c>
@@ -27876,7 +27874,7 @@
       <c r="U400" s="1"/>
       <c r="V400" s="1"/>
     </row>
-    <row r="401" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="401" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A401" s="1" t="s">
         <v>6</v>
       </c>
@@ -27930,7 +27928,7 @@
       <c r="U401" s="1"/>
       <c r="V401" s="1"/>
     </row>
-    <row r="402" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="402" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A402" s="1" t="s">
         <v>6</v>
       </c>
@@ -27984,7 +27982,7 @@
       <c r="U402" s="1"/>
       <c r="V402" s="1"/>
     </row>
-    <row r="403" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="403" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A403" s="1" t="s">
         <v>6</v>
       </c>
@@ -28038,7 +28036,7 @@
       <c r="U403" s="1"/>
       <c r="V403" s="1"/>
     </row>
-    <row r="404" spans="1:22" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="404" spans="1:22" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A404" s="1" t="s">
         <v>6</v>
       </c>
@@ -28092,7 +28090,7 @@
       <c r="U404" s="1"/>
       <c r="V404" s="1"/>
     </row>
-    <row r="405" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="405" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A405" s="1" t="s">
         <v>6</v>
       </c>
@@ -28146,7 +28144,7 @@
       <c r="U405" s="1"/>
       <c r="V405" s="1"/>
     </row>
-    <row r="406" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="406" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A406" s="1" t="s">
         <v>6</v>
       </c>
@@ -28200,7 +28198,7 @@
       <c r="U406" s="1"/>
       <c r="V406" s="1"/>
     </row>
-    <row r="407" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="407" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A407" s="1" t="s">
         <v>6</v>
       </c>
@@ -28254,7 +28252,7 @@
       <c r="U407" s="1"/>
       <c r="V407" s="1"/>
     </row>
-    <row r="408" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="408" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A408" s="1" t="s">
         <v>6</v>
       </c>
@@ -28308,7 +28306,7 @@
       <c r="U408" s="1"/>
       <c r="V408" s="1"/>
     </row>
-    <row r="409" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="409" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A409" s="1" t="s">
         <v>6</v>
       </c>
@@ -28362,7 +28360,7 @@
       <c r="U409" s="1"/>
       <c r="V409" s="1"/>
     </row>
-    <row r="410" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="410" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A410" s="1" t="s">
         <v>6</v>
       </c>
@@ -28416,7 +28414,7 @@
       <c r="U410" s="1"/>
       <c r="V410" s="1"/>
     </row>
-    <row r="411" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="411" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A411" s="1" t="s">
         <v>6</v>
       </c>
@@ -28470,7 +28468,7 @@
       <c r="U411" s="1"/>
       <c r="V411" s="1"/>
     </row>
-    <row r="412" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="412" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A412" s="1" t="s">
         <v>6</v>
       </c>
@@ -28524,7 +28522,7 @@
       <c r="U412" s="1"/>
       <c r="V412" s="1"/>
     </row>
-    <row r="413" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="413" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A413" s="1" t="s">
         <v>6</v>
       </c>
@@ -28576,7 +28574,7 @@
       <c r="U413" s="1"/>
       <c r="V413" s="1"/>
     </row>
-    <row r="414" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="414" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A414" s="1" t="s">
         <v>6</v>
       </c>
@@ -28628,7 +28626,7 @@
       <c r="U414" s="1"/>
       <c r="V414" s="1"/>
     </row>
-    <row r="415" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="415" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A415" s="1" t="s">
         <v>6</v>
       </c>
@@ -28680,7 +28678,7 @@
       <c r="U415" s="1"/>
       <c r="V415" s="1"/>
     </row>
-    <row r="416" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="416" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A416" s="1" t="s">
         <v>6</v>
       </c>
@@ -28732,7 +28730,7 @@
       <c r="U416" s="1"/>
       <c r="V416" s="1"/>
     </row>
-    <row r="417" spans="1:22" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="417" spans="1:22" ht="58" x14ac:dyDescent="0.35">
       <c r="A417" s="1" t="s">
         <v>6</v>
       </c>
@@ -28786,7 +28784,7 @@
       <c r="U417" s="1"/>
       <c r="V417" s="1"/>
     </row>
-    <row r="418" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="418" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A418" s="1" t="s">
         <v>6</v>
       </c>
@@ -28840,7 +28838,7 @@
       <c r="U418" s="1"/>
       <c r="V418" s="1"/>
     </row>
-    <row r="419" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="419" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A419" s="1" t="s">
         <v>6</v>
       </c>
@@ -28894,159 +28892,8 @@
       <c r="U419" s="1"/>
       <c r="V419" s="1"/>
     </row>
-    <row r="690" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O690" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="691" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O691" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="692" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O692" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="693" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O693" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="694" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O694" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="695" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O695" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="696" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O696" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="697" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O697" s="54">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="698" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O698" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="699" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O699" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="700" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O700" s="54">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="701" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O701" s="54">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="703" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O703" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="704" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O704" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="705" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O705" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="706" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O706" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="707" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O707" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="708" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O708" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="709" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O709" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="710" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O710" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="711" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O711" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="712" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O712" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="713" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O713" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="714" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O714" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="715" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O715" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="716" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O716" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="717" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O717" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="718" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O718" s="54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="719" spans="15:15" x14ac:dyDescent="0.35">
-      <c r="O719" s="54">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:V419" xr:uid="{00000000-0001-0000-0100-000000000000}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="Philippe Ciais"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:V419" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L229">
     <sortCondition ref="C2:C424"/>
   </sortState>

</xml_diff>

<commit_message>
modif tableaux de synthese
</commit_message>
<xml_diff>
--- a/Data/FairCarboN_Datas_Contacts.xlsx
+++ b/Data/FairCarboN_Datas_Contacts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dutroncj\Documents\Outils\FairCarboN_datas\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FCEAADA-B3E8-4D79-92A3-240B48ACC832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{708A70D1-E731-49F8-8410-634B75BE5859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Liste" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
améliorations + modif sources
</commit_message>
<xml_diff>
--- a/Data/FairCarboN_Datas_Contacts.xlsx
+++ b/Data/FairCarboN_Datas_Contacts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dutroncj\Documents\Outils\FairCarboN_datas\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB251C0A-F855-45B3-BCF4-2A2CAD47CDEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97E22647-15D3-4EDC-8CEA-2959004EF425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Liste" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Liste!$A$1:$T$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Liste!$A$1:$T$418</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5932" uniqueCount="1848">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5933" uniqueCount="1849">
   <si>
     <t>Acronyme PEPR</t>
   </si>
@@ -5597,6 +5597,9 @@
   </si>
   <si>
     <t>2023-A long-term monthly surface water storage dataset for the Congo basin from 1992 to 2015/2023-Panta Rhei benchmark dataset: socio-hydrological data of paired events of floods and droughts/2022-Oil slicks in the Gulf of Guinea – 10 years of Envisat Advanced Synthetic Aperture Radar observations</t>
+  </si>
+  <si>
+    <t>lionel.alletto@inrae.fr</t>
   </si>
 </sst>
 </file>
@@ -25279,7 +25282,9 @@
       <c r="C348" s="21" t="s">
         <v>1540</v>
       </c>
-      <c r="D348" s="26"/>
+      <c r="D348" s="16" t="s">
+        <v>1848</v>
+      </c>
       <c r="E348" s="34" t="s">
         <v>1539</v>
       </c>
@@ -27847,7 +27852,7 @@
       <c r="C396" s="21" t="s">
         <v>1666</v>
       </c>
-      <c r="D396" s="19" t="s">
+      <c r="D396" s="16" t="s">
         <v>1634</v>
       </c>
       <c r="E396" s="37" t="s">
@@ -29076,7 +29081,7 @@
       <c r="T418" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T1" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <autoFilter ref="A1:T418" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L228">
     <sortCondition ref="C2:C423"/>
   </sortState>
@@ -29329,7 +29334,7 @@
     <hyperlink ref="D393" r:id="rId245" display="mailto:edouard.metzger@univ-angers.fr" xr:uid="{59E61568-78B5-41C8-85D1-CC43DBA55D0D}"/>
     <hyperlink ref="D394" r:id="rId246" display="mailto:jean-sebastien.moquet@cnrs-orleans.fr" xr:uid="{0517E78E-5BA6-4C99-95AF-C7D28D0EC215}"/>
     <hyperlink ref="D395" r:id="rId247" display="mailto:Julien.Nemery@grenoble-inp.fr" xr:uid="{6FDF451D-F42A-43B7-8022-12E0F273F4D3}"/>
-    <hyperlink ref="D396" r:id="rId248" display="mailto:Pierre.Polsenaere@Ifremer.fr" xr:uid="{4178A1DF-1C5B-4C5A-B6DD-D1A40885B42D}"/>
+    <hyperlink ref="D396" r:id="rId248" xr:uid="{4178A1DF-1C5B-4C5A-B6DD-D1A40885B42D}"/>
     <hyperlink ref="D397" r:id="rId249" display="mailto:cristina.ribaudo@ensegid.fr" xr:uid="{E0F33667-16B4-4954-A6A2-B927FEFD3616}"/>
     <hyperlink ref="D398" r:id="rId250" display="mailto:philippe.rosa@univ-nantes.fr" xr:uid="{399C084D-0179-479B-97B1-866B4936755B}"/>
     <hyperlink ref="D399" r:id="rId251" display="mailto:nicolas.savoye@u-bordeaux.fr" xr:uid="{9B1C3AF1-9F70-472A-9B83-1576E6459B24}"/>
@@ -29356,8 +29361,9 @@
     <hyperlink ref="D363" r:id="rId272" xr:uid="{B64D5E0B-23AE-4FDD-AA57-B0FBC122B4F1}"/>
     <hyperlink ref="D104" r:id="rId273" xr:uid="{7089C2BE-4027-4FC6-A1F9-6A1AE4B8725E}"/>
     <hyperlink ref="D101" r:id="rId274" xr:uid="{71155148-E90E-47B9-8E3F-E19F3F36A0ED}"/>
+    <hyperlink ref="D348" r:id="rId275" xr:uid="{81D62058-B298-48D5-BEA8-2A123AB178FF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId275"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId276"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
correction extraction ORCID avec gestion des champs vides
</commit_message>
<xml_diff>
--- a/Data/FairCarboN_Datas_Contacts.xlsx
+++ b/Data/FairCarboN_Datas_Contacts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dutroncj\Documents\Outils\FairCarboN_datas\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E00446C-74D1-4C3A-B380-8DC361E31816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3AE8110-ACA6-4C34-A0BE-221BC680E754}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7670,7 +7670,7 @@
     <col min="23" max="16384" width="8.7265625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="46" t="s">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
fichiers contacts à jour
</commit_message>
<xml_diff>
--- a/Data/FairCarboN_Datas_Contacts.xlsx
+++ b/Data/FairCarboN_Datas_Contacts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dutroncj\Documents\Outils\FairCarboN_datas\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBE6A123-8EF9-498C-97C8-5B653B74AF7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3C8DF57-CD37-4F7B-A56D-45D3118E2B11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6846" uniqueCount="2359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6848" uniqueCount="2361">
   <si>
     <t>Acronyme PEPR</t>
   </si>
@@ -7162,6 +7162,12 @@
   </si>
   <si>
     <t>christophe.proisy@ird.fr</t>
+  </si>
+  <si>
+    <t>marie.arnaud.1@sorbonne-universite.fr</t>
+  </si>
+  <si>
+    <t>adrien.baysse-laine@umrpacte.fr</t>
   </si>
 </sst>
 </file>
@@ -7901,7 +7907,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:V417"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -7994,7 +7999,7 @@
         <v>2290</v>
       </c>
     </row>
-    <row r="2" spans="1:22" s="2" customFormat="1" ht="188.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" s="2" customFormat="1" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -8054,7 +8059,7 @@
       </c>
       <c r="V2" s="1"/>
     </row>
-    <row r="3" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -8114,7 +8119,7 @@
       </c>
       <c r="V3" s="1"/>
     </row>
-    <row r="4" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -8174,7 +8179,7 @@
       </c>
       <c r="V4" s="1"/>
     </row>
-    <row r="5" spans="1:22" s="2" customFormat="1" ht="188.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" s="2" customFormat="1" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -8234,7 +8239,7 @@
       </c>
       <c r="V5" s="1"/>
     </row>
-    <row r="6" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -8296,7 +8301,7 @@
       </c>
       <c r="V6" s="1"/>
     </row>
-    <row r="7" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
@@ -8358,7 +8363,7 @@
       </c>
       <c r="V7" s="1"/>
     </row>
-    <row r="8" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -8418,7 +8423,7 @@
       </c>
       <c r="V8" s="1"/>
     </row>
-    <row r="9" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
@@ -8478,7 +8483,7 @@
       </c>
       <c r="V9" s="1"/>
     </row>
-    <row r="10" spans="1:22" s="2" customFormat="1" ht="159.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" s="2" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
@@ -8538,7 +8543,7 @@
       </c>
       <c r="V10" s="1"/>
     </row>
-    <row r="11" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>6</v>
       </c>
@@ -8598,7 +8603,7 @@
       </c>
       <c r="V11" s="1"/>
     </row>
-    <row r="12" spans="1:22" s="2" customFormat="1" ht="188.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" s="2" customFormat="1" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>6</v>
       </c>
@@ -8658,7 +8663,7 @@
       </c>
       <c r="V12" s="1"/>
     </row>
-    <row r="13" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>6</v>
       </c>
@@ -8718,7 +8723,7 @@
       </c>
       <c r="V13" s="1"/>
     </row>
-    <row r="14" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>6</v>
       </c>
@@ -8780,7 +8785,7 @@
       </c>
       <c r="V14" s="1"/>
     </row>
-    <row r="15" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>6</v>
       </c>
@@ -8840,7 +8845,7 @@
       </c>
       <c r="V15" s="1"/>
     </row>
-    <row r="16" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>6</v>
       </c>
@@ -8902,7 +8907,7 @@
       </c>
       <c r="V16" s="1"/>
     </row>
-    <row r="17" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>6</v>
       </c>
@@ -8962,7 +8967,7 @@
       </c>
       <c r="V17" s="1"/>
     </row>
-    <row r="18" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>6</v>
       </c>
@@ -9022,7 +9027,7 @@
       </c>
       <c r="V18" s="1"/>
     </row>
-    <row r="19" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>6</v>
       </c>
@@ -9082,7 +9087,7 @@
       </c>
       <c r="V19" s="1"/>
     </row>
-    <row r="20" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>6</v>
       </c>
@@ -9142,7 +9147,7 @@
       </c>
       <c r="V20" s="1"/>
     </row>
-    <row r="21" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>6</v>
       </c>
@@ -9202,7 +9207,7 @@
       </c>
       <c r="V21" s="1"/>
     </row>
-    <row r="22" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>6</v>
       </c>
@@ -9262,7 +9267,7 @@
       </c>
       <c r="V22" s="1"/>
     </row>
-    <row r="23" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>6</v>
       </c>
@@ -9322,7 +9327,7 @@
       </c>
       <c r="V23" s="1"/>
     </row>
-    <row r="24" spans="1:22" s="2" customFormat="1" ht="275.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:22" s="2" customFormat="1" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>6</v>
       </c>
@@ -9388,7 +9393,7 @@
         <v>2331</v>
       </c>
     </row>
-    <row r="25" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>6</v>
       </c>
@@ -9450,7 +9455,7 @@
       </c>
       <c r="V25" s="1"/>
     </row>
-    <row r="26" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>6</v>
       </c>
@@ -9510,7 +9515,7 @@
       </c>
       <c r="V26" s="1"/>
     </row>
-    <row r="27" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>6</v>
       </c>
@@ -9570,7 +9575,7 @@
       </c>
       <c r="V27" s="1"/>
     </row>
-    <row r="28" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>6</v>
       </c>
@@ -9630,7 +9635,7 @@
       </c>
       <c r="V28" s="1"/>
     </row>
-    <row r="29" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>6</v>
       </c>
@@ -9690,7 +9695,7 @@
       </c>
       <c r="V29" s="1"/>
     </row>
-    <row r="30" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>6</v>
       </c>
@@ -9750,7 +9755,7 @@
       </c>
       <c r="V30" s="1"/>
     </row>
-    <row r="31" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>6</v>
       </c>
@@ -9812,7 +9817,7 @@
       </c>
       <c r="V31" s="1"/>
     </row>
-    <row r="32" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>6</v>
       </c>
@@ -9872,7 +9877,7 @@
       </c>
       <c r="V32" s="1"/>
     </row>
-    <row r="33" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>6</v>
       </c>
@@ -9932,7 +9937,7 @@
       </c>
       <c r="V33" s="1"/>
     </row>
-    <row r="34" spans="1:22" s="2" customFormat="1" ht="232" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:22" s="2" customFormat="1" ht="232" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>6</v>
       </c>
@@ -9994,7 +9999,7 @@
       </c>
       <c r="V34" s="1"/>
     </row>
-    <row r="35" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>6</v>
       </c>
@@ -10054,7 +10059,7 @@
       </c>
       <c r="V35" s="1"/>
     </row>
-    <row r="36" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>6</v>
       </c>
@@ -10114,7 +10119,7 @@
       </c>
       <c r="V36" s="1"/>
     </row>
-    <row r="37" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>6</v>
       </c>
@@ -10174,7 +10179,7 @@
       </c>
       <c r="V37" s="1"/>
     </row>
-    <row r="38" spans="1:22" s="2" customFormat="1" ht="159.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:22" s="2" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>6</v>
       </c>
@@ -10234,7 +10239,7 @@
       </c>
       <c r="V38" s="1"/>
     </row>
-    <row r="39" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>6</v>
       </c>
@@ -10294,7 +10299,7 @@
       </c>
       <c r="V39" s="1"/>
     </row>
-    <row r="40" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>6</v>
       </c>
@@ -10354,7 +10359,7 @@
       </c>
       <c r="V40" s="1"/>
     </row>
-    <row r="41" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>6</v>
       </c>
@@ -10414,7 +10419,7 @@
       </c>
       <c r="V41" s="1"/>
     </row>
-    <row r="42" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>6</v>
       </c>
@@ -10474,7 +10479,7 @@
       </c>
       <c r="V42" s="1"/>
     </row>
-    <row r="43" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>6</v>
       </c>
@@ -10534,7 +10539,7 @@
       </c>
       <c r="V43" s="1"/>
     </row>
-    <row r="44" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>6</v>
       </c>
@@ -10594,7 +10599,7 @@
       </c>
       <c r="V44" s="1"/>
     </row>
-    <row r="45" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>6</v>
       </c>
@@ -10654,7 +10659,7 @@
       </c>
       <c r="V45" s="1"/>
     </row>
-    <row r="46" spans="1:22" s="2" customFormat="1" ht="275.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:22" s="2" customFormat="1" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>6</v>
       </c>
@@ -10718,7 +10723,7 @@
       </c>
       <c r="V46" s="1"/>
     </row>
-    <row r="47" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>6</v>
       </c>
@@ -10778,7 +10783,7 @@
       </c>
       <c r="V47" s="1"/>
     </row>
-    <row r="48" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>6</v>
       </c>
@@ -10840,7 +10845,7 @@
       </c>
       <c r="V48" s="1"/>
     </row>
-    <row r="49" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>6</v>
       </c>
@@ -10900,7 +10905,7 @@
       </c>
       <c r="V49" s="1"/>
     </row>
-    <row r="50" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>6</v>
       </c>
@@ -10960,7 +10965,7 @@
       </c>
       <c r="V50" s="1"/>
     </row>
-    <row r="51" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>6</v>
       </c>
@@ -11020,7 +11025,7 @@
       </c>
       <c r="V51" s="1"/>
     </row>
-    <row r="52" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>6</v>
       </c>
@@ -11080,7 +11085,7 @@
       </c>
       <c r="V52" s="1"/>
     </row>
-    <row r="53" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>6</v>
       </c>
@@ -11140,7 +11145,7 @@
       </c>
       <c r="V53" s="1"/>
     </row>
-    <row r="54" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>6</v>
       </c>
@@ -11200,7 +11205,7 @@
       </c>
       <c r="V54" s="1"/>
     </row>
-    <row r="55" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>6</v>
       </c>
@@ -11260,7 +11265,7 @@
       </c>
       <c r="V55" s="1"/>
     </row>
-    <row r="56" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>6</v>
       </c>
@@ -11320,7 +11325,7 @@
       </c>
       <c r="V56" s="1"/>
     </row>
-    <row r="57" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>6</v>
       </c>
@@ -11380,7 +11385,7 @@
       </c>
       <c r="V57" s="1"/>
     </row>
-    <row r="58" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>6</v>
       </c>
@@ -11442,7 +11447,7 @@
       </c>
       <c r="V58" s="1"/>
     </row>
-    <row r="59" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>6</v>
       </c>
@@ -11504,7 +11509,7 @@
       </c>
       <c r="V59" s="1"/>
     </row>
-    <row r="60" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>6</v>
       </c>
@@ -11566,7 +11571,7 @@
       </c>
       <c r="V60" s="1"/>
     </row>
-    <row r="61" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>6</v>
       </c>
@@ -11628,7 +11633,7 @@
       </c>
       <c r="V61" s="1"/>
     </row>
-    <row r="62" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>6</v>
       </c>
@@ -11688,7 +11693,7 @@
       </c>
       <c r="V62" s="1"/>
     </row>
-    <row r="63" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>6</v>
       </c>
@@ -11750,7 +11755,7 @@
       </c>
       <c r="V63" s="1"/>
     </row>
-    <row r="64" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>6</v>
       </c>
@@ -11810,7 +11815,7 @@
       </c>
       <c r="V64" s="1"/>
     </row>
-    <row r="65" spans="1:22" s="2" customFormat="1" ht="409.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:22" s="2" customFormat="1" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>6</v>
       </c>
@@ -11874,7 +11879,7 @@
       </c>
       <c r="V65" s="1"/>
     </row>
-    <row r="66" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>6</v>
       </c>
@@ -11934,7 +11939,7 @@
       </c>
       <c r="V66" s="1"/>
     </row>
-    <row r="67" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>6</v>
       </c>
@@ -11996,7 +12001,7 @@
       </c>
       <c r="V67" s="1"/>
     </row>
-    <row r="68" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>6</v>
       </c>
@@ -12056,7 +12061,7 @@
       </c>
       <c r="V68" s="1"/>
     </row>
-    <row r="69" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>6</v>
       </c>
@@ -12116,7 +12121,7 @@
       </c>
       <c r="V69" s="1"/>
     </row>
-    <row r="70" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>6</v>
       </c>
@@ -12176,7 +12181,7 @@
       </c>
       <c r="V70" s="1"/>
     </row>
-    <row r="71" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>6</v>
       </c>
@@ -12238,7 +12243,7 @@
         <v>2291</v>
       </c>
     </row>
-    <row r="72" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>6</v>
       </c>
@@ -12298,7 +12303,7 @@
       </c>
       <c r="V72" s="1"/>
     </row>
-    <row r="73" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>6</v>
       </c>
@@ -12358,7 +12363,7 @@
       </c>
       <c r="V73" s="1"/>
     </row>
-    <row r="74" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>6</v>
       </c>
@@ -12418,7 +12423,7 @@
       </c>
       <c r="V74" s="1"/>
     </row>
-    <row r="75" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>6</v>
       </c>
@@ -12478,7 +12483,7 @@
       </c>
       <c r="V75" s="1"/>
     </row>
-    <row r="76" spans="1:22" s="2" customFormat="1" ht="27.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:22" s="2" customFormat="1" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>6</v>
       </c>
@@ -12540,7 +12545,7 @@
       </c>
       <c r="V76" s="1"/>
     </row>
-    <row r="77" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>6</v>
       </c>
@@ -12600,7 +12605,7 @@
       </c>
       <c r="V77" s="1"/>
     </row>
-    <row r="78" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>6</v>
       </c>
@@ -12660,7 +12665,7 @@
       </c>
       <c r="V78" s="1"/>
     </row>
-    <row r="79" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>6</v>
       </c>
@@ -12720,7 +12725,7 @@
       </c>
       <c r="V79" s="1"/>
     </row>
-    <row r="80" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>6</v>
       </c>
@@ -12782,7 +12787,7 @@
       </c>
       <c r="V80" s="1"/>
     </row>
-    <row r="81" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>6</v>
       </c>
@@ -12842,7 +12847,7 @@
       </c>
       <c r="V81" s="1"/>
     </row>
-    <row r="82" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>6</v>
       </c>
@@ -12904,7 +12909,7 @@
       </c>
       <c r="V82" s="1"/>
     </row>
-    <row r="83" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>6</v>
       </c>
@@ -12966,7 +12971,7 @@
       </c>
       <c r="V83" s="1"/>
     </row>
-    <row r="84" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>6</v>
       </c>
@@ -13028,7 +13033,7 @@
       </c>
       <c r="V84" s="1"/>
     </row>
-    <row r="85" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>6</v>
       </c>
@@ -13092,7 +13097,7 @@
       </c>
       <c r="V85" s="1"/>
     </row>
-    <row r="86" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>6</v>
       </c>
@@ -13154,7 +13159,7 @@
       </c>
       <c r="V86" s="1"/>
     </row>
-    <row r="87" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>6</v>
       </c>
@@ -13216,7 +13221,7 @@
       </c>
       <c r="V87" s="1"/>
     </row>
-    <row r="88" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>6</v>
       </c>
@@ -13276,7 +13281,7 @@
       </c>
       <c r="V88" s="1"/>
     </row>
-    <row r="89" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>6</v>
       </c>
@@ -13340,7 +13345,7 @@
       </c>
       <c r="V89" s="1"/>
     </row>
-    <row r="90" spans="1:22" s="2" customFormat="1" ht="159.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:22" s="2" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>6</v>
       </c>
@@ -13402,7 +13407,7 @@
       </c>
       <c r="V90" s="1"/>
     </row>
-    <row r="91" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>6</v>
       </c>
@@ -13464,7 +13469,7 @@
       </c>
       <c r="V91" s="1"/>
     </row>
-    <row r="92" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>6</v>
       </c>
@@ -13526,7 +13531,7 @@
       </c>
       <c r="V92" s="1"/>
     </row>
-    <row r="93" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
         <v>6</v>
       </c>
@@ -13586,7 +13591,7 @@
       </c>
       <c r="V93" s="1"/>
     </row>
-    <row r="94" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
         <v>6</v>
       </c>
@@ -13648,7 +13653,7 @@
       </c>
       <c r="V94" s="1"/>
     </row>
-    <row r="95" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
         <v>6</v>
       </c>
@@ -13710,7 +13715,7 @@
       </c>
       <c r="V95" s="1"/>
     </row>
-    <row r="96" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>6</v>
       </c>
@@ -13772,7 +13777,7 @@
       </c>
       <c r="V96" s="1"/>
     </row>
-    <row r="97" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>6</v>
       </c>
@@ -13834,7 +13839,7 @@
       </c>
       <c r="V97" s="1"/>
     </row>
-    <row r="98" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>6</v>
       </c>
@@ -13896,7 +13901,7 @@
       </c>
       <c r="V98" s="1"/>
     </row>
-    <row r="99" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>6</v>
       </c>
@@ -13958,7 +13963,7 @@
       </c>
       <c r="V99" s="1"/>
     </row>
-    <row r="100" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
         <v>6</v>
       </c>
@@ -14020,7 +14025,7 @@
       </c>
       <c r="V100" s="1"/>
     </row>
-    <row r="101" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>6</v>
       </c>
@@ -14084,7 +14089,7 @@
       </c>
       <c r="V101" s="1"/>
     </row>
-    <row r="102" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
         <v>6</v>
       </c>
@@ -14146,7 +14151,7 @@
       </c>
       <c r="V102" s="1"/>
     </row>
-    <row r="103" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>6</v>
       </c>
@@ -14208,7 +14213,7 @@
       </c>
       <c r="V103" s="1"/>
     </row>
-    <row r="104" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
         <v>6</v>
       </c>
@@ -14272,7 +14277,7 @@
       </c>
       <c r="V104" s="1"/>
     </row>
-    <row r="105" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>6</v>
       </c>
@@ -14334,7 +14339,7 @@
       </c>
       <c r="V105" s="1"/>
     </row>
-    <row r="106" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>6</v>
       </c>
@@ -14394,7 +14399,7 @@
       </c>
       <c r="V106" s="1"/>
     </row>
-    <row r="107" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
         <v>6</v>
       </c>
@@ -14456,7 +14461,7 @@
       </c>
       <c r="V107" s="1"/>
     </row>
-    <row r="108" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
         <v>6</v>
       </c>
@@ -14514,7 +14519,7 @@
       </c>
       <c r="V108" s="1"/>
     </row>
-    <row r="109" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
         <v>6</v>
       </c>
@@ -14576,7 +14581,7 @@
       </c>
       <c r="V109" s="1"/>
     </row>
-    <row r="110" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
         <v>6</v>
       </c>
@@ -14640,7 +14645,7 @@
       </c>
       <c r="V110" s="1"/>
     </row>
-    <row r="111" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>6</v>
       </c>
@@ -14702,7 +14707,7 @@
       </c>
       <c r="V111" s="1"/>
     </row>
-    <row r="112" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>6</v>
       </c>
@@ -14764,7 +14769,7 @@
       </c>
       <c r="V112" s="1"/>
     </row>
-    <row r="113" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
         <v>6</v>
       </c>
@@ -14826,7 +14831,7 @@
       </c>
       <c r="V113" s="1"/>
     </row>
-    <row r="114" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
         <v>6</v>
       </c>
@@ -14886,7 +14891,7 @@
       </c>
       <c r="V114" s="1"/>
     </row>
-    <row r="115" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A115" s="1" t="s">
         <v>6</v>
       </c>
@@ -14948,7 +14953,7 @@
       </c>
       <c r="V115" s="1"/>
     </row>
-    <row r="116" spans="1:22" s="2" customFormat="1" ht="409.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:22" s="2" customFormat="1" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
         <v>6</v>
       </c>
@@ -15012,7 +15017,7 @@
         <v>2321</v>
       </c>
     </row>
-    <row r="117" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
         <v>6</v>
       </c>
@@ -15074,7 +15079,7 @@
       </c>
       <c r="V117" s="1"/>
     </row>
-    <row r="118" spans="1:22" s="2" customFormat="1" ht="406" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:22" s="2" customFormat="1" ht="406" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
         <v>6</v>
       </c>
@@ -15138,7 +15143,7 @@
         <v>2356</v>
       </c>
     </row>
-    <row r="119" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
         <v>6</v>
       </c>
@@ -15200,7 +15205,7 @@
       </c>
       <c r="V119" s="1"/>
     </row>
-    <row r="120" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
         <v>6</v>
       </c>
@@ -15264,7 +15269,7 @@
       </c>
       <c r="V120" s="1"/>
     </row>
-    <row r="121" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
         <v>6</v>
       </c>
@@ -15326,7 +15331,7 @@
       </c>
       <c r="V121" s="1"/>
     </row>
-    <row r="122" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A122" s="1" t="s">
         <v>6</v>
       </c>
@@ -15388,7 +15393,7 @@
       </c>
       <c r="V122" s="1"/>
     </row>
-    <row r="123" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
         <v>6</v>
       </c>
@@ -15450,7 +15455,7 @@
       </c>
       <c r="V123" s="1"/>
     </row>
-    <row r="124" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
         <v>6</v>
       </c>
@@ -15512,7 +15517,7 @@
       </c>
       <c r="V124" s="1"/>
     </row>
-    <row r="125" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
         <v>6</v>
       </c>
@@ -15574,7 +15579,7 @@
       </c>
       <c r="V125" s="1"/>
     </row>
-    <row r="126" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
         <v>6</v>
       </c>
@@ -15636,7 +15641,7 @@
       </c>
       <c r="V126" s="1"/>
     </row>
-    <row r="127" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
         <v>6</v>
       </c>
@@ -15698,7 +15703,7 @@
       </c>
       <c r="V127" s="1"/>
     </row>
-    <row r="128" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A128" s="1" t="s">
         <v>6</v>
       </c>
@@ -15760,7 +15765,7 @@
       </c>
       <c r="V128" s="1"/>
     </row>
-    <row r="129" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A129" s="1" t="s">
         <v>6</v>
       </c>
@@ -15822,7 +15827,7 @@
       </c>
       <c r="V129" s="1"/>
     </row>
-    <row r="130" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A130" s="1" t="s">
         <v>6</v>
       </c>
@@ -15884,7 +15889,7 @@
       </c>
       <c r="V130" s="1"/>
     </row>
-    <row r="131" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A131" s="1" t="s">
         <v>6</v>
       </c>
@@ -15946,7 +15951,7 @@
       </c>
       <c r="V131" s="1"/>
     </row>
-    <row r="132" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A132" s="1" t="s">
         <v>6</v>
       </c>
@@ -16008,7 +16013,7 @@
       </c>
       <c r="V132" s="1"/>
     </row>
-    <row r="133" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A133" s="1" t="s">
         <v>6</v>
       </c>
@@ -16070,7 +16075,7 @@
       </c>
       <c r="V133" s="1"/>
     </row>
-    <row r="134" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A134" s="1" t="s">
         <v>6</v>
       </c>
@@ -16132,7 +16137,7 @@
       </c>
       <c r="V134" s="1"/>
     </row>
-    <row r="135" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
         <v>6</v>
       </c>
@@ -16194,7 +16199,7 @@
       </c>
       <c r="V135" s="1"/>
     </row>
-    <row r="136" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A136" s="1" t="s">
         <v>6</v>
       </c>
@@ -16256,7 +16261,7 @@
       </c>
       <c r="V136" s="1"/>
     </row>
-    <row r="137" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
         <v>6</v>
       </c>
@@ -16318,7 +16323,7 @@
       </c>
       <c r="V137" s="1"/>
     </row>
-    <row r="138" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
         <v>6</v>
       </c>
@@ -16380,7 +16385,7 @@
       </c>
       <c r="V138" s="1"/>
     </row>
-    <row r="139" spans="1:22" s="2" customFormat="1" ht="275.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:22" s="2" customFormat="1" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A139" s="1" t="s">
         <v>6</v>
       </c>
@@ -16446,7 +16451,7 @@
         <v>2331</v>
       </c>
     </row>
-    <row r="140" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A140" s="1" t="s">
         <v>6</v>
       </c>
@@ -16508,7 +16513,7 @@
       </c>
       <c r="V140" s="1"/>
     </row>
-    <row r="141" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A141" s="1" t="s">
         <v>6</v>
       </c>
@@ -16570,7 +16575,7 @@
       </c>
       <c r="V141" s="1"/>
     </row>
-    <row r="142" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A142" s="1" t="s">
         <v>6</v>
       </c>
@@ -16632,7 +16637,7 @@
       </c>
       <c r="V142" s="1"/>
     </row>
-    <row r="143" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A143" s="1" t="s">
         <v>6</v>
       </c>
@@ -16696,7 +16701,7 @@
       </c>
       <c r="V143" s="1"/>
     </row>
-    <row r="144" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A144" s="1" t="s">
         <v>6</v>
       </c>
@@ -16758,7 +16763,7 @@
       </c>
       <c r="V144" s="1"/>
     </row>
-    <row r="145" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
         <v>6</v>
       </c>
@@ -16820,7 +16825,7 @@
       </c>
       <c r="V145" s="1"/>
     </row>
-    <row r="146" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A146" s="1" t="s">
         <v>6</v>
       </c>
@@ -16884,7 +16889,7 @@
       </c>
       <c r="V146" s="1"/>
     </row>
-    <row r="147" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A147" s="1" t="s">
         <v>6</v>
       </c>
@@ -16946,7 +16951,7 @@
       </c>
       <c r="V147" s="1"/>
     </row>
-    <row r="148" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A148" s="1" t="s">
         <v>6</v>
       </c>
@@ -17008,7 +17013,7 @@
       </c>
       <c r="V148" s="1"/>
     </row>
-    <row r="149" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A149" s="1" t="s">
         <v>6</v>
       </c>
@@ -17070,7 +17075,7 @@
       </c>
       <c r="V149" s="1"/>
     </row>
-    <row r="150" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A150" s="1" t="s">
         <v>6</v>
       </c>
@@ -17132,7 +17137,7 @@
       </c>
       <c r="V150" s="1"/>
     </row>
-    <row r="151" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A151" s="1" t="s">
         <v>6</v>
       </c>
@@ -17194,7 +17199,7 @@
       </c>
       <c r="V151" s="1"/>
     </row>
-    <row r="152" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A152" s="1" t="s">
         <v>6</v>
       </c>
@@ -17256,7 +17261,7 @@
       </c>
       <c r="V152" s="1"/>
     </row>
-    <row r="153" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A153" s="1" t="s">
         <v>6</v>
       </c>
@@ -17318,7 +17323,7 @@
       </c>
       <c r="V153" s="1"/>
     </row>
-    <row r="154" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A154" s="1" t="s">
         <v>6</v>
       </c>
@@ -17380,7 +17385,7 @@
       </c>
       <c r="V154" s="1"/>
     </row>
-    <row r="155" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A155" s="1" t="s">
         <v>6</v>
       </c>
@@ -17442,7 +17447,7 @@
       </c>
       <c r="V155" s="1"/>
     </row>
-    <row r="156" spans="1:22" s="2" customFormat="1" ht="65" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:22" s="2" customFormat="1" ht="65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A156" s="1" t="s">
         <v>6</v>
       </c>
@@ -17504,7 +17509,7 @@
       </c>
       <c r="V156" s="1"/>
     </row>
-    <row r="157" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A157" s="1" t="s">
         <v>6</v>
       </c>
@@ -17566,7 +17571,7 @@
       </c>
       <c r="V157" s="1"/>
     </row>
-    <row r="158" spans="1:22" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:22" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A158" s="1" t="s">
         <v>6</v>
       </c>
@@ -17628,7 +17633,7 @@
       </c>
       <c r="V158" s="1"/>
     </row>
-    <row r="159" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
       <c r="A159" s="1" t="s">
         <v>6</v>
       </c>
@@ -17690,7 +17695,7 @@
       </c>
       <c r="V159" s="1"/>
     </row>
-    <row r="160" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
       <c r="A160" s="1" t="s">
         <v>6</v>
       </c>
@@ -17754,7 +17759,7 @@
       </c>
       <c r="V160" s="1"/>
     </row>
-    <row r="161" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A161" s="1" t="s">
         <v>6</v>
       </c>
@@ -17816,7 +17821,7 @@
       </c>
       <c r="V161" s="1"/>
     </row>
-    <row r="162" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A162" s="1" t="s">
         <v>6</v>
       </c>
@@ -17878,7 +17883,7 @@
       </c>
       <c r="V162" s="1"/>
     </row>
-    <row r="163" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A163" s="1" t="s">
         <v>6</v>
       </c>
@@ -17940,7 +17945,7 @@
       </c>
       <c r="V163" s="1"/>
     </row>
-    <row r="164" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A164" s="1" t="s">
         <v>6</v>
       </c>
@@ -18002,7 +18007,7 @@
       </c>
       <c r="V164" s="1"/>
     </row>
-    <row r="165" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
       <c r="A165" s="1" t="s">
         <v>6</v>
       </c>
@@ -18066,7 +18071,7 @@
       </c>
       <c r="V165" s="1"/>
     </row>
-    <row r="166" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
       <c r="A166" s="1" t="s">
         <v>6</v>
       </c>
@@ -18132,7 +18137,7 @@
       </c>
       <c r="V166" s="1"/>
     </row>
-    <row r="167" spans="1:22" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:22" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A167" s="1" t="s">
         <v>6</v>
       </c>
@@ -18194,7 +18199,7 @@
       </c>
       <c r="V167" s="1"/>
     </row>
-    <row r="168" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A168" s="1" t="s">
         <v>6</v>
       </c>
@@ -18256,7 +18261,7 @@
       </c>
       <c r="V168" s="1"/>
     </row>
-    <row r="169" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
       <c r="A169" s="1" t="s">
         <v>6</v>
       </c>
@@ -18318,7 +18323,7 @@
       </c>
       <c r="V169" s="1"/>
     </row>
-    <row r="170" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A170" s="1" t="s">
         <v>6</v>
       </c>
@@ -18380,7 +18385,7 @@
       </c>
       <c r="V170" s="1"/>
     </row>
-    <row r="171" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A171" s="1" t="s">
         <v>6</v>
       </c>
@@ -18442,7 +18447,7 @@
       </c>
       <c r="V171" s="1"/>
     </row>
-    <row r="172" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A172" s="1" t="s">
         <v>6</v>
       </c>
@@ -18504,7 +18509,7 @@
       </c>
       <c r="V172" s="1"/>
     </row>
-    <row r="173" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A173" s="1" t="s">
         <v>6</v>
       </c>
@@ -18566,7 +18571,7 @@
       </c>
       <c r="V173" s="1"/>
     </row>
-    <row r="174" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A174" s="1" t="s">
         <v>6</v>
       </c>
@@ -18628,7 +18633,7 @@
       </c>
       <c r="V174" s="1"/>
     </row>
-    <row r="175" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A175" s="1" t="s">
         <v>6</v>
       </c>
@@ -18690,7 +18695,7 @@
       </c>
       <c r="V175" s="1"/>
     </row>
-    <row r="176" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
       <c r="A176" s="1" t="s">
         <v>6</v>
       </c>
@@ -18752,7 +18757,7 @@
       </c>
       <c r="V176" s="1"/>
     </row>
-    <row r="177" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
       <c r="A177" s="1" t="s">
         <v>6</v>
       </c>
@@ -18814,7 +18819,7 @@
       </c>
       <c r="V177" s="1"/>
     </row>
-    <row r="178" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A178" s="1" t="s">
         <v>6</v>
       </c>
@@ -18876,7 +18881,7 @@
       </c>
       <c r="V178" s="1"/>
     </row>
-    <row r="179" spans="1:22" s="2" customFormat="1" ht="174" hidden="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:22" s="2" customFormat="1" ht="174" x14ac:dyDescent="0.35">
       <c r="A179" s="1" t="s">
         <v>6</v>
       </c>
@@ -18940,7 +18945,7 @@
       </c>
       <c r="V179" s="1"/>
     </row>
-    <row r="180" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A180" s="1" t="s">
         <v>6</v>
       </c>
@@ -19002,7 +19007,7 @@
       </c>
       <c r="V180" s="1"/>
     </row>
-    <row r="181" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A181" s="1" t="s">
         <v>6</v>
       </c>
@@ -19064,7 +19069,7 @@
       </c>
       <c r="V181" s="1"/>
     </row>
-    <row r="182" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A182" s="1" t="s">
         <v>6</v>
       </c>
@@ -19126,7 +19131,7 @@
       </c>
       <c r="V182" s="1"/>
     </row>
-    <row r="183" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A183" s="1" t="s">
         <v>6</v>
       </c>
@@ -19188,7 +19193,7 @@
       </c>
       <c r="V183" s="1"/>
     </row>
-    <row r="184" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A184" s="1" t="s">
         <v>6</v>
       </c>
@@ -19252,7 +19257,7 @@
       </c>
       <c r="V184" s="1"/>
     </row>
-    <row r="185" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A185" s="1" t="s">
         <v>6</v>
       </c>
@@ -19314,7 +19319,7 @@
       </c>
       <c r="V185" s="1"/>
     </row>
-    <row r="186" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A186" s="1" t="s">
         <v>6</v>
       </c>
@@ -19376,7 +19381,7 @@
       </c>
       <c r="V186" s="1"/>
     </row>
-    <row r="187" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A187" s="1" t="s">
         <v>6</v>
       </c>
@@ -19438,7 +19443,7 @@
       </c>
       <c r="V187" s="1"/>
     </row>
-    <row r="188" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A188" s="1" t="s">
         <v>6</v>
       </c>
@@ -19500,7 +19505,7 @@
       </c>
       <c r="V188" s="1"/>
     </row>
-    <row r="189" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A189" s="1" t="s">
         <v>6</v>
       </c>
@@ -19562,7 +19567,7 @@
       </c>
       <c r="V189" s="1"/>
     </row>
-    <row r="190" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A190" s="1" t="s">
         <v>6</v>
       </c>
@@ -19622,7 +19627,7 @@
       </c>
       <c r="V190" s="1"/>
     </row>
-    <row r="191" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A191" s="1" t="s">
         <v>6</v>
       </c>
@@ -19684,7 +19689,7 @@
       </c>
       <c r="V191" s="1"/>
     </row>
-    <row r="192" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A192" s="1" t="s">
         <v>6</v>
       </c>
@@ -19746,7 +19751,7 @@
       </c>
       <c r="V192" s="1"/>
     </row>
-    <row r="193" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A193" s="1" t="s">
         <v>6</v>
       </c>
@@ -19808,7 +19813,7 @@
       </c>
       <c r="V193" s="1"/>
     </row>
-    <row r="194" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A194" s="1" t="s">
         <v>6</v>
       </c>
@@ -19868,7 +19873,7 @@
       </c>
       <c r="V194" s="1"/>
     </row>
-    <row r="195" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A195" s="1" t="s">
         <v>6</v>
       </c>
@@ -19928,7 +19933,7 @@
       </c>
       <c r="V195" s="1"/>
     </row>
-    <row r="196" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A196" s="1" t="s">
         <v>6</v>
       </c>
@@ -19988,7 +19993,7 @@
       </c>
       <c r="V196" s="1"/>
     </row>
-    <row r="197" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A197" s="1" t="s">
         <v>6</v>
       </c>
@@ -20050,7 +20055,7 @@
       </c>
       <c r="V197" s="1"/>
     </row>
-    <row r="198" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A198" s="1" t="s">
         <v>6</v>
       </c>
@@ -20112,7 +20117,7 @@
       </c>
       <c r="V198" s="1"/>
     </row>
-    <row r="199" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A199" s="1" t="s">
         <v>6</v>
       </c>
@@ -20174,7 +20179,7 @@
       </c>
       <c r="V199" s="1"/>
     </row>
-    <row r="200" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A200" s="1" t="s">
         <v>6</v>
       </c>
@@ -20236,7 +20241,7 @@
       </c>
       <c r="V200" s="1"/>
     </row>
-    <row r="201" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A201" s="1" t="s">
         <v>6</v>
       </c>
@@ -20298,7 +20303,7 @@
       </c>
       <c r="V201" s="1"/>
     </row>
-    <row r="202" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A202" s="1" t="s">
         <v>6</v>
       </c>
@@ -20360,7 +20365,7 @@
       </c>
       <c r="V202" s="1"/>
     </row>
-    <row r="203" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A203" s="1" t="s">
         <v>6</v>
       </c>
@@ -20422,7 +20427,7 @@
       </c>
       <c r="V203" s="1"/>
     </row>
-    <row r="204" spans="1:22" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:22" ht="87" x14ac:dyDescent="0.35">
       <c r="A204" s="1" t="s">
         <v>6</v>
       </c>
@@ -20484,7 +20489,7 @@
       </c>
       <c r="V204" s="1"/>
     </row>
-    <row r="205" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A205" s="1" t="s">
         <v>6</v>
       </c>
@@ -20546,7 +20551,7 @@
       </c>
       <c r="V205" s="1"/>
     </row>
-    <row r="206" spans="1:22" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:22" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A206" s="1" t="s">
         <v>6</v>
       </c>
@@ -20606,7 +20611,7 @@
       </c>
       <c r="V206" s="1"/>
     </row>
-    <row r="207" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A207" s="1" t="s">
         <v>6</v>
       </c>
@@ -20668,7 +20673,7 @@
       </c>
       <c r="V207" s="1"/>
     </row>
-    <row r="208" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A208" s="1" t="s">
         <v>6</v>
       </c>
@@ -20730,7 +20735,7 @@
       </c>
       <c r="V208" s="1"/>
     </row>
-    <row r="209" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A209" s="1" t="s">
         <v>6</v>
       </c>
@@ -20790,7 +20795,7 @@
       </c>
       <c r="V209" s="1"/>
     </row>
-    <row r="210" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A210" s="1" t="s">
         <v>6</v>
       </c>
@@ -20850,7 +20855,7 @@
       </c>
       <c r="V210" s="1"/>
     </row>
-    <row r="211" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A211" s="1" t="s">
         <v>6</v>
       </c>
@@ -20910,7 +20915,7 @@
       </c>
       <c r="V211" s="1"/>
     </row>
-    <row r="212" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A212" s="1" t="s">
         <v>6</v>
       </c>
@@ -20970,7 +20975,7 @@
       </c>
       <c r="V212" s="1"/>
     </row>
-    <row r="213" spans="1:22" s="2" customFormat="1" ht="409.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:22" s="2" customFormat="1" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A213" s="1" t="s">
         <v>6</v>
       </c>
@@ -21032,7 +21037,7 @@
         <v>2294</v>
       </c>
     </row>
-    <row r="214" spans="1:22" s="2" customFormat="1" ht="188.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:22" s="2" customFormat="1" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A214" s="1" t="s">
         <v>6</v>
       </c>
@@ -21092,7 +21097,7 @@
       </c>
       <c r="V214" s="1"/>
     </row>
-    <row r="215" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A215" s="1" t="s">
         <v>6</v>
       </c>
@@ -21152,7 +21157,7 @@
       </c>
       <c r="V215" s="1"/>
     </row>
-    <row r="216" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A216" s="1" t="s">
         <v>6</v>
       </c>
@@ -21212,7 +21217,7 @@
       </c>
       <c r="V216" s="1"/>
     </row>
-    <row r="217" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A217" s="1" t="s">
         <v>6</v>
       </c>
@@ -21272,7 +21277,7 @@
       </c>
       <c r="V217" s="1"/>
     </row>
-    <row r="218" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A218" s="1" t="s">
         <v>6</v>
       </c>
@@ -21334,7 +21339,7 @@
       </c>
       <c r="V218" s="1"/>
     </row>
-    <row r="219" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A219" s="1" t="s">
         <v>6</v>
       </c>
@@ -21396,7 +21401,7 @@
       </c>
       <c r="V219" s="1"/>
     </row>
-    <row r="220" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A220" s="1" t="s">
         <v>6</v>
       </c>
@@ -21458,7 +21463,7 @@
       </c>
       <c r="V220" s="1"/>
     </row>
-    <row r="221" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A221" s="1" t="s">
         <v>6</v>
       </c>
@@ -21518,7 +21523,7 @@
       </c>
       <c r="V221" s="1"/>
     </row>
-    <row r="222" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A222" s="1" t="s">
         <v>6</v>
       </c>
@@ -21580,7 +21585,7 @@
       </c>
       <c r="V222" s="1"/>
     </row>
-    <row r="223" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A223" s="1" t="s">
         <v>6</v>
       </c>
@@ -21642,7 +21647,7 @@
       </c>
       <c r="V223" s="1"/>
     </row>
-    <row r="224" spans="1:22" s="2" customFormat="1" ht="159.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:22" s="2" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A224" s="1" t="s">
         <v>6</v>
       </c>
@@ -21702,7 +21707,7 @@
       </c>
       <c r="V224" s="1"/>
     </row>
-    <row r="225" spans="1:22" s="2" customFormat="1" ht="406" hidden="1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:22" s="2" customFormat="1" ht="406" x14ac:dyDescent="0.35">
       <c r="A225" s="1" t="s">
         <v>6</v>
       </c>
@@ -21764,7 +21769,7 @@
         <v>2356</v>
       </c>
     </row>
-    <row r="226" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A226" s="1" t="s">
         <v>6</v>
       </c>
@@ -21824,7 +21829,7 @@
       </c>
       <c r="V226" s="1"/>
     </row>
-    <row r="227" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A227" s="1" t="s">
         <v>6</v>
       </c>
@@ -21886,7 +21891,7 @@
       </c>
       <c r="V227" s="1"/>
     </row>
-    <row r="228" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A228" s="1" t="s">
         <v>6</v>
       </c>
@@ -21946,7 +21951,7 @@
       </c>
       <c r="V228" s="1"/>
     </row>
-    <row r="229" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A229" s="1" t="s">
         <v>6</v>
       </c>
@@ -22016,7 +22021,9 @@
       <c r="C230" s="21" t="s">
         <v>1262</v>
       </c>
-      <c r="D230" s="1"/>
+      <c r="D230" s="13" t="s">
+        <v>2359</v>
+      </c>
       <c r="E230" s="1" t="s">
         <v>618</v>
       </c>
@@ -22064,7 +22071,7 @@
       </c>
       <c r="V230" s="1"/>
     </row>
-    <row r="231" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A231" s="1" t="s">
         <v>6</v>
       </c>
@@ -22124,7 +22131,7 @@
       </c>
       <c r="V231" s="1"/>
     </row>
-    <row r="232" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A232" s="1" t="s">
         <v>6</v>
       </c>
@@ -22184,7 +22191,7 @@
       </c>
       <c r="V232" s="1"/>
     </row>
-    <row r="233" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A233" s="1" t="s">
         <v>6</v>
       </c>
@@ -22244,7 +22251,7 @@
       </c>
       <c r="V233" s="1"/>
     </row>
-    <row r="234" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A234" s="1" t="s">
         <v>6</v>
       </c>
@@ -22302,7 +22309,7 @@
       </c>
       <c r="V234" s="1"/>
     </row>
-    <row r="235" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A235" s="1" t="s">
         <v>6</v>
       </c>
@@ -22360,7 +22367,7 @@
       </c>
       <c r="V235" s="1"/>
     </row>
-    <row r="236" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A236" s="1" t="s">
         <v>6</v>
       </c>
@@ -22420,7 +22427,7 @@
       </c>
       <c r="V236" s="1"/>
     </row>
-    <row r="237" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A237" s="1" t="s">
         <v>6</v>
       </c>
@@ -22480,7 +22487,7 @@
       </c>
       <c r="V237" s="1"/>
     </row>
-    <row r="238" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A238" s="1" t="s">
         <v>6</v>
       </c>
@@ -22538,7 +22545,7 @@
       </c>
       <c r="V238" s="1"/>
     </row>
-    <row r="239" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A239" s="1" t="s">
         <v>6</v>
       </c>
@@ -22598,7 +22605,7 @@
       </c>
       <c r="V239" s="1"/>
     </row>
-    <row r="240" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A240" s="1" t="s">
         <v>6</v>
       </c>
@@ -22656,7 +22663,7 @@
       </c>
       <c r="V240" s="1"/>
     </row>
-    <row r="241" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A241" s="1" t="s">
         <v>6</v>
       </c>
@@ -22714,7 +22721,7 @@
       </c>
       <c r="V241" s="1"/>
     </row>
-    <row r="242" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A242" s="1" t="s">
         <v>6</v>
       </c>
@@ -22774,7 +22781,7 @@
       </c>
       <c r="V242" s="1"/>
     </row>
-    <row r="243" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A243" s="1" t="s">
         <v>6</v>
       </c>
@@ -22834,7 +22841,7 @@
       </c>
       <c r="V243" s="1"/>
     </row>
-    <row r="244" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A244" s="1" t="s">
         <v>6</v>
       </c>
@@ -22896,7 +22903,7 @@
       </c>
       <c r="V244" s="1"/>
     </row>
-    <row r="245" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A245" s="1" t="s">
         <v>6</v>
       </c>
@@ -22954,7 +22961,7 @@
       </c>
       <c r="V245" s="1"/>
     </row>
-    <row r="246" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A246" s="1" t="s">
         <v>6</v>
       </c>
@@ -23012,7 +23019,7 @@
       </c>
       <c r="V246" s="1"/>
     </row>
-    <row r="247" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A247" s="1" t="s">
         <v>6</v>
       </c>
@@ -23072,7 +23079,7 @@
       </c>
       <c r="V247" s="1"/>
     </row>
-    <row r="248" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A248" s="1" t="s">
         <v>6</v>
       </c>
@@ -23132,7 +23139,7 @@
       </c>
       <c r="V248" s="1"/>
     </row>
-    <row r="249" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A249" s="1" t="s">
         <v>6</v>
       </c>
@@ -23192,7 +23199,7 @@
       </c>
       <c r="V249" s="1"/>
     </row>
-    <row r="250" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A250" s="1" t="s">
         <v>6</v>
       </c>
@@ -23250,7 +23257,7 @@
       </c>
       <c r="V250" s="1"/>
     </row>
-    <row r="251" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A251" s="1" t="s">
         <v>6</v>
       </c>
@@ -23312,7 +23319,7 @@
       </c>
       <c r="V251" s="1"/>
     </row>
-    <row r="252" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A252" s="1" t="s">
         <v>6</v>
       </c>
@@ -23374,7 +23381,7 @@
       </c>
       <c r="V252" s="1"/>
     </row>
-    <row r="253" spans="1:22" s="2" customFormat="1" ht="409.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:22" s="2" customFormat="1" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A253" s="1" t="s">
         <v>6</v>
       </c>
@@ -23436,7 +23443,7 @@
         <v>2313</v>
       </c>
     </row>
-    <row r="254" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A254" s="1" t="s">
         <v>6</v>
       </c>
@@ -23496,7 +23503,7 @@
       </c>
       <c r="V254" s="1"/>
     </row>
-    <row r="255" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A255" s="1" t="s">
         <v>6</v>
       </c>
@@ -23556,7 +23563,7 @@
       </c>
       <c r="V255" s="1"/>
     </row>
-    <row r="256" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A256" s="1" t="s">
         <v>6</v>
       </c>
@@ -23614,7 +23621,7 @@
       </c>
       <c r="V256" s="1"/>
     </row>
-    <row r="257" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A257" s="1" t="s">
         <v>6</v>
       </c>
@@ -23672,7 +23679,7 @@
       </c>
       <c r="V257" s="1"/>
     </row>
-    <row r="258" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A258" s="1" t="s">
         <v>6</v>
       </c>
@@ -23730,7 +23737,7 @@
       </c>
       <c r="V258" s="1"/>
     </row>
-    <row r="259" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A259" s="1" t="s">
         <v>6</v>
       </c>
@@ -23792,7 +23799,7 @@
       </c>
       <c r="V259" s="1"/>
     </row>
-    <row r="260" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A260" s="1" t="s">
         <v>6</v>
       </c>
@@ -23850,7 +23857,7 @@
       </c>
       <c r="V260" s="1"/>
     </row>
-    <row r="261" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A261" s="1" t="s">
         <v>6</v>
       </c>
@@ -23908,7 +23915,7 @@
       </c>
       <c r="V261" s="1"/>
     </row>
-    <row r="262" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A262" s="1" t="s">
         <v>6</v>
       </c>
@@ -23968,7 +23975,7 @@
       </c>
       <c r="V262" s="1"/>
     </row>
-    <row r="263" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A263" s="1" t="s">
         <v>6</v>
       </c>
@@ -24028,7 +24035,7 @@
       </c>
       <c r="V263" s="1"/>
     </row>
-    <row r="264" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A264" s="1" t="s">
         <v>6</v>
       </c>
@@ -24088,7 +24095,7 @@
       </c>
       <c r="V264" s="1"/>
     </row>
-    <row r="265" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A265" s="1" t="s">
         <v>6</v>
       </c>
@@ -24148,7 +24155,7 @@
       </c>
       <c r="V265" s="1"/>
     </row>
-    <row r="266" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A266" s="1" t="s">
         <v>6</v>
       </c>
@@ -24208,7 +24215,7 @@
       </c>
       <c r="V266" s="1"/>
     </row>
-    <row r="267" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A267" s="1" t="s">
         <v>6</v>
       </c>
@@ -24268,7 +24275,7 @@
       </c>
       <c r="V267" s="1"/>
     </row>
-    <row r="268" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A268" s="1" t="s">
         <v>6</v>
       </c>
@@ -24328,7 +24335,7 @@
       </c>
       <c r="V268" s="1"/>
     </row>
-    <row r="269" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A269" s="1" t="s">
         <v>6</v>
       </c>
@@ -24388,7 +24395,7 @@
       </c>
       <c r="V269" s="1"/>
     </row>
-    <row r="270" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A270" s="1" t="s">
         <v>6</v>
       </c>
@@ -24450,7 +24457,7 @@
       </c>
       <c r="V270" s="1"/>
     </row>
-    <row r="271" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A271" s="1" t="s">
         <v>6</v>
       </c>
@@ -24512,7 +24519,7 @@
       </c>
       <c r="V271" s="1"/>
     </row>
-    <row r="272" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A272" s="1" t="s">
         <v>6</v>
       </c>
@@ -24574,7 +24581,7 @@
       </c>
       <c r="V272" s="1"/>
     </row>
-    <row r="273" spans="1:22" s="2" customFormat="1" ht="377" hidden="1" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:22" s="2" customFormat="1" ht="377" x14ac:dyDescent="0.35">
       <c r="A273" s="1" t="s">
         <v>6</v>
       </c>
@@ -24638,7 +24645,7 @@
       </c>
       <c r="V273" s="1"/>
     </row>
-    <row r="274" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A274" s="1" t="s">
         <v>6</v>
       </c>
@@ -24700,7 +24707,7 @@
       </c>
       <c r="V274" s="1"/>
     </row>
-    <row r="275" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A275" s="1" t="s">
         <v>6</v>
       </c>
@@ -24762,7 +24769,7 @@
       </c>
       <c r="V275" s="1"/>
     </row>
-    <row r="276" spans="1:22" s="2" customFormat="1" ht="275.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:22" s="2" customFormat="1" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A276" s="1" t="s">
         <v>6</v>
       </c>
@@ -24826,7 +24833,7 @@
         <v>2293</v>
       </c>
     </row>
-    <row r="277" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A277" s="1" t="s">
         <v>6</v>
       </c>
@@ -24888,7 +24895,7 @@
       </c>
       <c r="V277" s="1"/>
     </row>
-    <row r="278" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A278" s="1" t="s">
         <v>6</v>
       </c>
@@ -24952,7 +24959,7 @@
       </c>
       <c r="V278" s="1"/>
     </row>
-    <row r="279" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A279" s="1" t="s">
         <v>6</v>
       </c>
@@ -25014,7 +25021,7 @@
       </c>
       <c r="V279" s="1"/>
     </row>
-    <row r="280" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A280" s="1" t="s">
         <v>6</v>
       </c>
@@ -25076,7 +25083,7 @@
       </c>
       <c r="V280" s="1"/>
     </row>
-    <row r="281" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A281" s="1" t="s">
         <v>6</v>
       </c>
@@ -25138,7 +25145,7 @@
       </c>
       <c r="V281" s="1"/>
     </row>
-    <row r="282" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A282" s="1" t="s">
         <v>6</v>
       </c>
@@ -25198,7 +25205,7 @@
       </c>
       <c r="V282" s="1"/>
     </row>
-    <row r="283" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A283" s="1" t="s">
         <v>6</v>
       </c>
@@ -25258,7 +25265,7 @@
       </c>
       <c r="V283" s="1"/>
     </row>
-    <row r="284" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A284" s="1" t="s">
         <v>6</v>
       </c>
@@ -25318,7 +25325,7 @@
       </c>
       <c r="V284" s="1"/>
     </row>
-    <row r="285" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A285" s="1" t="s">
         <v>6</v>
       </c>
@@ -25378,7 +25385,7 @@
       </c>
       <c r="V285" s="1"/>
     </row>
-    <row r="286" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A286" s="1" t="s">
         <v>6</v>
       </c>
@@ -25436,7 +25443,7 @@
       </c>
       <c r="V286" s="1"/>
     </row>
-    <row r="287" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A287" s="1" t="s">
         <v>6</v>
       </c>
@@ -25496,7 +25503,7 @@
       </c>
       <c r="V287" s="1"/>
     </row>
-    <row r="288" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A288" s="1" t="s">
         <v>6</v>
       </c>
@@ -25556,7 +25563,7 @@
       </c>
       <c r="V288" s="1"/>
     </row>
-    <row r="289" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A289" s="1" t="s">
         <v>6</v>
       </c>
@@ -25616,7 +25623,7 @@
       </c>
       <c r="V289" s="1"/>
     </row>
-    <row r="290" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A290" s="1" t="s">
         <v>6</v>
       </c>
@@ -25674,7 +25681,7 @@
       </c>
       <c r="V290" s="1"/>
     </row>
-    <row r="291" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A291" s="1" t="s">
         <v>6</v>
       </c>
@@ -25734,7 +25741,7 @@
       </c>
       <c r="V291" s="1"/>
     </row>
-    <row r="292" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A292" s="1" t="s">
         <v>6</v>
       </c>
@@ -25794,7 +25801,7 @@
       </c>
       <c r="V292" s="1"/>
     </row>
-    <row r="293" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A293" s="1" t="s">
         <v>6</v>
       </c>
@@ -25852,7 +25859,7 @@
       </c>
       <c r="V293" s="1"/>
     </row>
-    <row r="294" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A294" s="1" t="s">
         <v>6</v>
       </c>
@@ -25910,7 +25917,7 @@
       </c>
       <c r="V294" s="1"/>
     </row>
-    <row r="295" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A295" s="1" t="s">
         <v>6</v>
       </c>
@@ -25968,7 +25975,7 @@
       </c>
       <c r="V295" s="1"/>
     </row>
-    <row r="296" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A296" s="1" t="s">
         <v>6</v>
       </c>
@@ -26026,7 +26033,7 @@
       </c>
       <c r="V296" s="1"/>
     </row>
-    <row r="297" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A297" s="1" t="s">
         <v>6</v>
       </c>
@@ -26086,7 +26093,7 @@
       </c>
       <c r="V297" s="1"/>
     </row>
-    <row r="298" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A298" s="1" t="s">
         <v>6</v>
       </c>
@@ -26096,7 +26103,9 @@
       <c r="C298" s="21" t="s">
         <v>1423</v>
       </c>
-      <c r="D298" s="26"/>
+      <c r="D298" s="13" t="s">
+        <v>2360</v>
+      </c>
       <c r="E298" s="31" t="s">
         <v>1396</v>
       </c>
@@ -26131,7 +26140,7 @@
       <c r="P298" s="1"/>
       <c r="Q298" s="1"/>
       <c r="R298" s="1" t="s">
-        <v>1756</v>
+        <v>1832</v>
       </c>
       <c r="S298" s="1" t="s">
         <v>1756</v>
@@ -26144,7 +26153,7 @@
       </c>
       <c r="V298" s="1"/>
     </row>
-    <row r="299" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A299" s="1" t="s">
         <v>6</v>
       </c>
@@ -26204,7 +26213,7 @@
       </c>
       <c r="V299" s="1"/>
     </row>
-    <row r="300" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A300" s="1" t="s">
         <v>6</v>
       </c>
@@ -26262,7 +26271,7 @@
       </c>
       <c r="V300" s="1"/>
     </row>
-    <row r="301" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A301" s="1" t="s">
         <v>6</v>
       </c>
@@ -26322,7 +26331,7 @@
       </c>
       <c r="V301" s="1"/>
     </row>
-    <row r="302" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A302" s="1" t="s">
         <v>6</v>
       </c>
@@ -26380,7 +26389,7 @@
       </c>
       <c r="V302" s="1"/>
     </row>
-    <row r="303" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A303" s="1" t="s">
         <v>6</v>
       </c>
@@ -26438,7 +26447,7 @@
       </c>
       <c r="V303" s="1"/>
     </row>
-    <row r="304" spans="1:22" s="2" customFormat="1" ht="76.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:22" s="2" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A304" s="1" t="s">
         <v>6</v>
       </c>
@@ -26498,7 +26507,7 @@
       </c>
       <c r="V304" s="1"/>
     </row>
-    <row r="305" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A305" s="1" t="s">
         <v>6</v>
       </c>
@@ -26556,7 +26565,7 @@
       </c>
       <c r="V305" s="1"/>
     </row>
-    <row r="306" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A306" s="1" t="s">
         <v>6</v>
       </c>
@@ -26614,7 +26623,7 @@
       </c>
       <c r="V306" s="1"/>
     </row>
-    <row r="307" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A307" s="1" t="s">
         <v>6</v>
       </c>
@@ -26672,7 +26681,7 @@
       </c>
       <c r="V307" s="1"/>
     </row>
-    <row r="308" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A308" s="1" t="s">
         <v>6</v>
       </c>
@@ -26730,7 +26739,7 @@
       </c>
       <c r="V308" s="1"/>
     </row>
-    <row r="309" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A309" s="1" t="s">
         <v>6</v>
       </c>
@@ -26788,7 +26797,7 @@
       </c>
       <c r="V309" s="1"/>
     </row>
-    <row r="310" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A310" s="1" t="s">
         <v>6</v>
       </c>
@@ -26846,7 +26855,7 @@
       </c>
       <c r="V310" s="1"/>
     </row>
-    <row r="311" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A311" s="1" t="s">
         <v>6</v>
       </c>
@@ -26904,7 +26913,7 @@
       </c>
       <c r="V311" s="1"/>
     </row>
-    <row r="312" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A312" s="1" t="s">
         <v>6</v>
       </c>
@@ -26966,7 +26975,7 @@
       </c>
       <c r="V312" s="1"/>
     </row>
-    <row r="313" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A313" s="1" t="s">
         <v>6</v>
       </c>
@@ -27030,7 +27039,7 @@
       </c>
       <c r="V313" s="1"/>
     </row>
-    <row r="314" spans="1:22" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:22" ht="87" x14ac:dyDescent="0.35">
       <c r="A314" s="1" t="s">
         <v>6</v>
       </c>
@@ -27094,7 +27103,7 @@
       </c>
       <c r="V314" s="1"/>
     </row>
-    <row r="315" spans="1:22" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:22" ht="87" x14ac:dyDescent="0.35">
       <c r="A315" s="1" t="s">
         <v>6</v>
       </c>
@@ -27154,7 +27163,7 @@
       </c>
       <c r="V315" s="1"/>
     </row>
-    <row r="316" spans="1:22" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:22" ht="87" x14ac:dyDescent="0.35">
       <c r="A316" s="1" t="s">
         <v>6</v>
       </c>
@@ -27212,7 +27221,7 @@
       </c>
       <c r="V316" s="1"/>
     </row>
-    <row r="317" spans="1:22" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:22" ht="87" x14ac:dyDescent="0.35">
       <c r="A317" s="1" t="s">
         <v>6</v>
       </c>
@@ -27274,7 +27283,7 @@
       </c>
       <c r="V317" s="1"/>
     </row>
-    <row r="318" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A318" s="1" t="s">
         <v>6</v>
       </c>
@@ -27334,7 +27343,7 @@
       </c>
       <c r="V318" s="1"/>
     </row>
-    <row r="319" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A319" s="1" t="s">
         <v>6</v>
       </c>
@@ -27396,7 +27405,7 @@
       </c>
       <c r="V319" s="1"/>
     </row>
-    <row r="320" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A320" s="1" t="s">
         <v>6</v>
       </c>
@@ -27456,7 +27465,7 @@
       </c>
       <c r="V320" s="1"/>
     </row>
-    <row r="321" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A321" s="1" t="s">
         <v>6</v>
       </c>
@@ -27518,7 +27527,7 @@
       </c>
       <c r="V321" s="1"/>
     </row>
-    <row r="322" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A322" s="1" t="s">
         <v>6</v>
       </c>
@@ -27576,7 +27585,7 @@
       </c>
       <c r="V322" s="1"/>
     </row>
-    <row r="323" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A323" s="1" t="s">
         <v>6</v>
       </c>
@@ -27634,7 +27643,7 @@
       </c>
       <c r="V323" s="1"/>
     </row>
-    <row r="324" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A324" s="1" t="s">
         <v>6</v>
       </c>
@@ -27694,7 +27703,7 @@
       </c>
       <c r="V324" s="1"/>
     </row>
-    <row r="325" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A325" s="1" t="s">
         <v>6</v>
       </c>
@@ -27752,7 +27761,7 @@
       </c>
       <c r="V325" s="1"/>
     </row>
-    <row r="326" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A326" s="1" t="s">
         <v>6</v>
       </c>
@@ -27812,7 +27821,7 @@
       </c>
       <c r="V326" s="1"/>
     </row>
-    <row r="327" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A327" s="1" t="s">
         <v>6</v>
       </c>
@@ -27872,7 +27881,7 @@
       </c>
       <c r="V327" s="1"/>
     </row>
-    <row r="328" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A328" s="1" t="s">
         <v>6</v>
       </c>
@@ -27932,7 +27941,7 @@
       </c>
       <c r="V328" s="1"/>
     </row>
-    <row r="329" spans="1:22" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:22" ht="58" x14ac:dyDescent="0.35">
       <c r="A329" s="1" t="s">
         <v>6</v>
       </c>
@@ -27992,7 +28001,7 @@
       </c>
       <c r="V329" s="1"/>
     </row>
-    <row r="330" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A330" s="1" t="s">
         <v>6</v>
       </c>
@@ -28054,7 +28063,7 @@
       </c>
       <c r="V330" s="1"/>
     </row>
-    <row r="331" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A331" s="1" t="s">
         <v>6</v>
       </c>
@@ -28114,7 +28123,7 @@
       </c>
       <c r="V331" s="1"/>
     </row>
-    <row r="332" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A332" s="1" t="s">
         <v>6</v>
       </c>
@@ -28174,7 +28183,7 @@
       </c>
       <c r="V332" s="1"/>
     </row>
-    <row r="333" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A333" s="1" t="s">
         <v>6</v>
       </c>
@@ -28234,7 +28243,7 @@
       </c>
       <c r="V333" s="1"/>
     </row>
-    <row r="334" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A334" s="1" t="s">
         <v>6</v>
       </c>
@@ -28294,7 +28303,7 @@
       </c>
       <c r="V334" s="1"/>
     </row>
-    <row r="335" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A335" s="1" t="s">
         <v>6</v>
       </c>
@@ -28354,7 +28363,7 @@
       </c>
       <c r="V335" s="1"/>
     </row>
-    <row r="336" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A336" s="1" t="s">
         <v>6</v>
       </c>
@@ -28414,7 +28423,7 @@
       </c>
       <c r="V336" s="1"/>
     </row>
-    <row r="337" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A337" s="1" t="s">
         <v>6</v>
       </c>
@@ -28472,7 +28481,7 @@
       </c>
       <c r="V337" s="1"/>
     </row>
-    <row r="338" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A338" s="1" t="s">
         <v>6</v>
       </c>
@@ -28532,7 +28541,7 @@
       </c>
       <c r="V338" s="1"/>
     </row>
-    <row r="339" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A339" s="1" t="s">
         <v>6</v>
       </c>
@@ -28592,7 +28601,7 @@
       </c>
       <c r="V339" s="1"/>
     </row>
-    <row r="340" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A340" s="1" t="s">
         <v>6</v>
       </c>
@@ -28652,7 +28661,7 @@
       </c>
       <c r="V340" s="1"/>
     </row>
-    <row r="341" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A341" s="1" t="s">
         <v>6</v>
       </c>
@@ -28714,7 +28723,7 @@
       </c>
       <c r="V341" s="1"/>
     </row>
-    <row r="342" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A342" s="1" t="s">
         <v>6</v>
       </c>
@@ -28774,7 +28783,7 @@
       </c>
       <c r="V342" s="1"/>
     </row>
-    <row r="343" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A343" s="1" t="s">
         <v>6</v>
       </c>
@@ -28832,7 +28841,7 @@
       </c>
       <c r="V343" s="1"/>
     </row>
-    <row r="344" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A344" s="1" t="s">
         <v>6</v>
       </c>
@@ -28890,7 +28899,7 @@
       </c>
       <c r="V344" s="1"/>
     </row>
-    <row r="345" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A345" s="1" t="s">
         <v>6</v>
       </c>
@@ -28950,7 +28959,7 @@
       </c>
       <c r="V345" s="1"/>
     </row>
-    <row r="346" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A346" s="1" t="s">
         <v>6</v>
       </c>
@@ -29010,7 +29019,7 @@
       </c>
       <c r="V346" s="1"/>
     </row>
-    <row r="347" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A347" s="1" t="s">
         <v>6</v>
       </c>
@@ -29072,7 +29081,7 @@
       </c>
       <c r="V347" s="1"/>
     </row>
-    <row r="348" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A348" s="1" t="s">
         <v>6</v>
       </c>
@@ -29132,7 +29141,7 @@
       </c>
       <c r="V348" s="1"/>
     </row>
-    <row r="349" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A349" s="1" t="s">
         <v>6</v>
       </c>
@@ -29192,7 +29201,7 @@
       </c>
       <c r="V349" s="1"/>
     </row>
-    <row r="350" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A350" s="1" t="s">
         <v>6</v>
       </c>
@@ -29252,7 +29261,7 @@
       </c>
       <c r="V350" s="1"/>
     </row>
-    <row r="351" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A351" s="1" t="s">
         <v>6</v>
       </c>
@@ -29308,7 +29317,7 @@
       </c>
       <c r="V351" s="1"/>
     </row>
-    <row r="352" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A352" s="1" t="s">
         <v>6</v>
       </c>
@@ -29368,7 +29377,7 @@
       </c>
       <c r="V352" s="1"/>
     </row>
-    <row r="353" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A353" s="1" t="s">
         <v>6</v>
       </c>
@@ -29428,7 +29437,7 @@
       </c>
       <c r="V353" s="1"/>
     </row>
-    <row r="354" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A354" s="1" t="s">
         <v>6</v>
       </c>
@@ -29488,7 +29497,7 @@
       </c>
       <c r="V354" s="1"/>
     </row>
-    <row r="355" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A355" s="1" t="s">
         <v>6</v>
       </c>
@@ -29548,7 +29557,7 @@
       </c>
       <c r="V355" s="1"/>
     </row>
-    <row r="356" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A356" s="1" t="s">
         <v>6</v>
       </c>
@@ -29608,7 +29617,7 @@
       </c>
       <c r="V356" s="1"/>
     </row>
-    <row r="357" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A357" s="1" t="s">
         <v>6</v>
       </c>
@@ -29668,7 +29677,7 @@
       </c>
       <c r="V357" s="1"/>
     </row>
-    <row r="358" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A358" s="1" t="s">
         <v>6</v>
       </c>
@@ -29726,7 +29735,7 @@
       </c>
       <c r="V358" s="1"/>
     </row>
-    <row r="359" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A359" s="1" t="s">
         <v>6</v>
       </c>
@@ -29784,7 +29793,7 @@
       </c>
       <c r="V359" s="1"/>
     </row>
-    <row r="360" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A360" s="1" t="s">
         <v>6</v>
       </c>
@@ -29844,7 +29853,7 @@
       </c>
       <c r="V360" s="1"/>
     </row>
-    <row r="361" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A361" s="1" t="s">
         <v>6</v>
       </c>
@@ -29906,7 +29915,7 @@
       </c>
       <c r="V361" s="1"/>
     </row>
-    <row r="362" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A362" s="1" t="s">
         <v>6</v>
       </c>
@@ -29968,7 +29977,7 @@
       </c>
       <c r="V362" s="1"/>
     </row>
-    <row r="363" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A363" s="1" t="s">
         <v>6</v>
       </c>
@@ -30028,7 +30037,7 @@
       </c>
       <c r="V363" s="1"/>
     </row>
-    <row r="364" spans="1:22" s="2" customFormat="1" ht="409.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:22" s="2" customFormat="1" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A364" s="1" t="s">
         <v>6</v>
       </c>
@@ -30090,7 +30099,7 @@
         <v>2294</v>
       </c>
     </row>
-    <row r="365" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A365" s="1" t="s">
         <v>6</v>
       </c>
@@ -30150,7 +30159,7 @@
       </c>
       <c r="V365" s="1"/>
     </row>
-    <row r="366" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A366" s="1" t="s">
         <v>6</v>
       </c>
@@ -30208,7 +30217,7 @@
       </c>
       <c r="V366" s="1"/>
     </row>
-    <row r="367" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A367" s="1" t="s">
         <v>6</v>
       </c>
@@ -30270,7 +30279,7 @@
       </c>
       <c r="V367" s="1"/>
     </row>
-    <row r="368" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A368" s="1" t="s">
         <v>6</v>
       </c>
@@ -30332,7 +30341,7 @@
       </c>
       <c r="V368" s="1"/>
     </row>
-    <row r="369" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A369" s="1" t="s">
         <v>6</v>
       </c>
@@ -30392,7 +30401,7 @@
       </c>
       <c r="V369" s="1"/>
     </row>
-    <row r="370" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A370" s="1" t="s">
         <v>6</v>
       </c>
@@ -30452,7 +30461,7 @@
       </c>
       <c r="V370" s="1"/>
     </row>
-    <row r="371" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A371" s="1" t="s">
         <v>6</v>
       </c>
@@ -30510,7 +30519,7 @@
       </c>
       <c r="V371" s="1"/>
     </row>
-    <row r="372" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A372" s="1" t="s">
         <v>6</v>
       </c>
@@ -30570,7 +30579,7 @@
       </c>
       <c r="V372" s="1"/>
     </row>
-    <row r="373" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A373" s="1" t="s">
         <v>6</v>
       </c>
@@ -30630,7 +30639,7 @@
       </c>
       <c r="V373" s="1"/>
     </row>
-    <row r="374" spans="1:22" s="2" customFormat="1" ht="362.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:22" s="2" customFormat="1" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A374" s="1" t="s">
         <v>6</v>
       </c>
@@ -30694,7 +30703,7 @@
         <v>2292</v>
       </c>
     </row>
-    <row r="375" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A375" s="1" t="s">
         <v>6</v>
       </c>
@@ -30754,7 +30763,7 @@
       </c>
       <c r="V375" s="1"/>
     </row>
-    <row r="376" spans="1:22" s="2" customFormat="1" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:22" s="2" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A376" s="1" t="s">
         <v>6</v>
       </c>
@@ -30814,7 +30823,7 @@
       </c>
       <c r="V376" s="1"/>
     </row>
-    <row r="377" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A377" s="1" t="s">
         <v>6</v>
       </c>
@@ -30876,7 +30885,7 @@
       </c>
       <c r="V377" s="1"/>
     </row>
-    <row r="378" spans="1:22" s="2" customFormat="1" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A378" s="1" t="s">
         <v>6</v>
       </c>
@@ -30938,7 +30947,7 @@
       </c>
       <c r="V378" s="1"/>
     </row>
-    <row r="379" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A379" s="1" t="s">
         <v>6</v>
       </c>
@@ -30998,7 +31007,7 @@
       </c>
       <c r="V379" s="1"/>
     </row>
-    <row r="380" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A380" s="1" t="s">
         <v>6</v>
       </c>
@@ -31060,7 +31069,7 @@
       </c>
       <c r="V380" s="1"/>
     </row>
-    <row r="381" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A381" s="1" t="s">
         <v>6</v>
       </c>
@@ -31120,7 +31129,7 @@
       </c>
       <c r="V381" s="1"/>
     </row>
-    <row r="382" spans="1:22" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:22" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A382" s="1" t="s">
         <v>6</v>
       </c>
@@ -31178,7 +31187,7 @@
       </c>
       <c r="V382" s="1"/>
     </row>
-    <row r="383" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="383" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A383" s="1" t="s">
         <v>6</v>
       </c>
@@ -31238,7 +31247,7 @@
       </c>
       <c r="V383" s="1"/>
     </row>
-    <row r="384" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="384" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A384" s="1" t="s">
         <v>6</v>
       </c>
@@ -31300,7 +31309,7 @@
       </c>
       <c r="V384" s="1"/>
     </row>
-    <row r="385" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="385" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A385" s="1" t="s">
         <v>6</v>
       </c>
@@ -31360,7 +31369,7 @@
       </c>
       <c r="V385" s="1"/>
     </row>
-    <row r="386" spans="1:22" s="2" customFormat="1" ht="409.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="386" spans="1:22" s="2" customFormat="1" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A386" s="1" t="s">
         <v>6</v>
       </c>
@@ -31422,7 +31431,7 @@
         <v>2332</v>
       </c>
     </row>
-    <row r="387" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="387" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A387" s="1" t="s">
         <v>6</v>
       </c>
@@ -31482,7 +31491,7 @@
       </c>
       <c r="V387" s="1"/>
     </row>
-    <row r="388" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="388" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A388" s="1" t="s">
         <v>6</v>
       </c>
@@ -31542,7 +31551,7 @@
       </c>
       <c r="V388" s="1"/>
     </row>
-    <row r="389" spans="1:22" s="2" customFormat="1" ht="116" hidden="1" x14ac:dyDescent="0.35">
+    <row r="389" spans="1:22" s="2" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A389" s="1" t="s">
         <v>6</v>
       </c>
@@ -31604,7 +31613,7 @@
       </c>
       <c r="V389" s="1"/>
     </row>
-    <row r="390" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="390" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A390" s="1" t="s">
         <v>6</v>
       </c>
@@ -31664,7 +31673,7 @@
       </c>
       <c r="V390" s="1"/>
     </row>
-    <row r="391" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="391" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A391" s="1" t="s">
         <v>6</v>
       </c>
@@ -31724,7 +31733,7 @@
       </c>
       <c r="V391" s="1"/>
     </row>
-    <row r="392" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="392" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A392" s="1" t="s">
         <v>6</v>
       </c>
@@ -31784,7 +31793,7 @@
       </c>
       <c r="V392" s="1"/>
     </row>
-    <row r="393" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="393" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A393" s="1" t="s">
         <v>6</v>
       </c>
@@ -31844,7 +31853,7 @@
       </c>
       <c r="V393" s="1"/>
     </row>
-    <row r="394" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="394" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A394" s="1" t="s">
         <v>6</v>
       </c>
@@ -31906,7 +31915,7 @@
       </c>
       <c r="V394" s="1"/>
     </row>
-    <row r="395" spans="1:22" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="395" spans="1:22" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A395" s="1" t="s">
         <v>6</v>
       </c>
@@ -31968,7 +31977,7 @@
       </c>
       <c r="V395" s="1"/>
     </row>
-    <row r="396" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="396" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A396" s="1" t="s">
         <v>6</v>
       </c>
@@ -32028,7 +32037,7 @@
       </c>
       <c r="V396" s="1"/>
     </row>
-    <row r="397" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="397" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A397" s="1" t="s">
         <v>6</v>
       </c>
@@ -32088,7 +32097,7 @@
       </c>
       <c r="V397" s="1"/>
     </row>
-    <row r="398" spans="1:22" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="398" spans="1:22" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A398" s="1" t="s">
         <v>6</v>
       </c>
@@ -32150,7 +32159,7 @@
       </c>
       <c r="V398" s="1"/>
     </row>
-    <row r="399" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="399" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A399" s="1" t="s">
         <v>6</v>
       </c>
@@ -32210,7 +32219,7 @@
       </c>
       <c r="V399" s="1"/>
     </row>
-    <row r="400" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="400" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A400" s="1" t="s">
         <v>6</v>
       </c>
@@ -32270,7 +32279,7 @@
       </c>
       <c r="V400" s="1"/>
     </row>
-    <row r="401" spans="1:22" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="401" spans="1:22" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A401" s="1" t="s">
         <v>6</v>
       </c>
@@ -32330,7 +32339,7 @@
       </c>
       <c r="V401" s="1"/>
     </row>
-    <row r="402" spans="1:22" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="402" spans="1:22" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A402" s="1" t="s">
         <v>6</v>
       </c>
@@ -32390,7 +32399,7 @@
       </c>
       <c r="V402" s="1"/>
     </row>
-    <row r="403" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="403" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A403" s="1" t="s">
         <v>6</v>
       </c>
@@ -32450,7 +32459,7 @@
       </c>
       <c r="V403" s="1"/>
     </row>
-    <row r="404" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="404" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A404" s="1" t="s">
         <v>6</v>
       </c>
@@ -32510,7 +32519,7 @@
       </c>
       <c r="V404" s="1"/>
     </row>
-    <row r="405" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="405" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A405" s="1" t="s">
         <v>6</v>
       </c>
@@ -32570,7 +32579,7 @@
       </c>
       <c r="V405" s="1"/>
     </row>
-    <row r="406" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="406" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A406" s="1" t="s">
         <v>6</v>
       </c>
@@ -32630,7 +32639,7 @@
       </c>
       <c r="V406" s="1"/>
     </row>
-    <row r="407" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="407" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A407" s="1" t="s">
         <v>6</v>
       </c>
@@ -32690,7 +32699,7 @@
       </c>
       <c r="V407" s="1"/>
     </row>
-    <row r="408" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="408" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A408" s="1" t="s">
         <v>6</v>
       </c>
@@ -32750,7 +32759,7 @@
       </c>
       <c r="V408" s="1"/>
     </row>
-    <row r="409" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="409" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A409" s="1" t="s">
         <v>6</v>
       </c>
@@ -32810,7 +32819,7 @@
       </c>
       <c r="V409" s="1"/>
     </row>
-    <row r="410" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="410" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A410" s="1" t="s">
         <v>6</v>
       </c>
@@ -32870,7 +32879,7 @@
       </c>
       <c r="V410" s="1"/>
     </row>
-    <row r="411" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="411" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A411" s="1" t="s">
         <v>6</v>
       </c>
@@ -32928,7 +32937,7 @@
       </c>
       <c r="V411" s="1"/>
     </row>
-    <row r="412" spans="1:22" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="412" spans="1:22" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A412" s="1" t="s">
         <v>6</v>
       </c>
@@ -32990,7 +32999,7 @@
         <v>2297</v>
       </c>
     </row>
-    <row r="413" spans="1:22" s="2" customFormat="1" ht="377" hidden="1" x14ac:dyDescent="0.35">
+    <row r="413" spans="1:22" s="2" customFormat="1" ht="377" x14ac:dyDescent="0.35">
       <c r="A413" s="1" t="s">
         <v>6</v>
       </c>
@@ -33052,7 +33061,7 @@
         <v>2330</v>
       </c>
     </row>
-    <row r="414" spans="1:22" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="414" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A414" s="1" t="s">
         <v>6</v>
       </c>
@@ -33112,7 +33121,7 @@
       </c>
       <c r="V414" s="1"/>
     </row>
-    <row r="415" spans="1:22" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="415" spans="1:22" ht="58" x14ac:dyDescent="0.35">
       <c r="A415" s="1" t="s">
         <v>6</v>
       </c>
@@ -33172,7 +33181,7 @@
       </c>
       <c r="V415" s="1"/>
     </row>
-    <row r="416" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="416" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A416" s="1" t="s">
         <v>6</v>
       </c>
@@ -33232,7 +33241,7 @@
       </c>
       <c r="V416" s="1"/>
     </row>
-    <row r="417" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="417" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A417" s="1" t="s">
         <v>6</v>
       </c>
@@ -33293,13 +33302,7 @@
       <c r="V417" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V417" xr:uid="{00000000-0001-0000-0100-000000000000}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="Marie Arnaud"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:V417" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L227">
     <sortCondition ref="C2:C422"/>
   </sortState>
@@ -33656,8 +33659,10 @@
     <hyperlink ref="D342" r:id="rId349" xr:uid="{F9AF74BC-C5BD-4C4C-80E9-B7676EA47DD4}"/>
     <hyperlink ref="D361" r:id="rId350" xr:uid="{A24A0A03-18C8-4164-9C9C-C6D7E8079A60}"/>
     <hyperlink ref="D248" r:id="rId351" xr:uid="{3E7272D2-FD11-4455-A18D-8F4152E7C571}"/>
+    <hyperlink ref="D230" r:id="rId352" xr:uid="{8CF31450-9FF6-41B8-B89D-83C1B91BBFED}"/>
+    <hyperlink ref="D298" r:id="rId353" xr:uid="{837E84CE-D2C6-454F-9ABE-6CE8B0C7790A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId352"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId354"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
suite avec intégration de Patricia
</commit_message>
<xml_diff>
--- a/Data/FairCarboN_Datas_Contacts.xlsx
+++ b/Data/FairCarboN_Datas_Contacts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dutroncj\Documents\Outils\FairCarboN_datas\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9806927A-E200-4A93-A2F0-C49C8D885C77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F580A21E-2834-4E9D-B449-92CFBE6DA9A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6899" uniqueCount="2405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6900" uniqueCount="2406">
   <si>
     <t>Acronyme PEPR</t>
   </si>
@@ -7327,6 +7327,10 @@
   </si>
   <si>
     <t>patricia.garnier@inrae.fr</t>
+  </si>
+  <si>
+    <t>29092025 - Cà c'est un email personnalisé dis-donc ! Tu arrives à faire ça pour tout le monde ?
+Oui je confirme que je depose fidèlement sur HAL depuis un an ou 2 environ. D'accord je vais regarder et compléter bien sûr.</t>
   </si>
 </sst>
 </file>
@@ -8535,7 +8539,7 @@
       </c>
       <c r="V7" s="1"/>
     </row>
-    <row r="8" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" s="2" customFormat="1" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -8585,7 +8589,7 @@
         <v>1825</v>
       </c>
       <c r="S8" s="1" t="s">
-        <v>1749</v>
+        <v>1825</v>
       </c>
       <c r="T8" s="60" t="s">
         <v>1847</v>
@@ -8593,7 +8597,9 @@
       <c r="U8" s="60" t="s">
         <v>1842</v>
       </c>
-      <c r="V8" s="1"/>
+      <c r="V8" s="1" t="s">
+        <v>2405</v>
+      </c>
     </row>
     <row r="9" spans="1:22" s="2" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">

</xml_diff>

<commit_message>
nouvelles analyses domaines scientifiques, et tutelles
</commit_message>
<xml_diff>
--- a/Data/FairCarboN_Datas_Contacts.xlsx
+++ b/Data/FairCarboN_Datas_Contacts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dutroncj\Documents\Outils\FairCarboN_datas\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB3A9E9F-A80B-43FE-A010-44FA11C4A174}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3C7F048-FD65-4409-81EC-420225D4D72B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Liste" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10346" uniqueCount="3110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10347" uniqueCount="3110">
   <si>
     <t>Acronyme PEPR</t>
   </si>
@@ -11463,7 +11463,7 @@
       </c>
       <c r="AA17" s="17"/>
     </row>
-    <row r="18" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A18" s="17" t="s">
         <v>6</v>
       </c>
@@ -11497,7 +11497,9 @@
       <c r="K18" s="3" t="s">
         <v>2636</v>
       </c>
-      <c r="L18" s="3"/>
+      <c r="L18" s="5" t="s">
+        <v>2639</v>
+      </c>
       <c r="M18" s="17" t="s">
         <v>2637</v>
       </c>

</xml_diff>

<commit_message>
pour mes visus HAL
</commit_message>
<xml_diff>
--- a/Data/FairCarboN_Datas_Contacts.xlsx
+++ b/Data/FairCarboN_Datas_Contacts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dutroncj\Documents\Outils\FairCarboN_datas\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{917AE5E7-9C01-411A-8B20-A90F05FEE732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DAD0D5A-F939-41B6-BFCE-4C6B058C3B96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -10065,11 +10065,18 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0;[Red]0"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -10369,149 +10376,152 @@
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="23" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -10519,55 +10529,58 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -10576,10 +10589,7 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -10999,7 +11009,7 @@
       </c>
       <c r="AA2" s="17"/>
     </row>
-    <row r="3" spans="1:27" ht="87" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:27" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A3" s="17" t="s">
         <v>6</v>
       </c>
@@ -11895,7 +11905,7 @@
       </c>
       <c r="AA14" s="17"/>
     </row>
-    <row r="15" spans="1:27" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:27" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A15" s="17" t="s">
         <v>6</v>
       </c>
@@ -11968,7 +11978,7 @@
       </c>
       <c r="AA15" s="17"/>
     </row>
-    <row r="16" spans="1:27" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:27" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A16" s="17" t="s">
         <v>6</v>
       </c>
@@ -12191,7 +12201,7 @@
       </c>
       <c r="AA18" s="17"/>
     </row>
-    <row r="19" spans="1:27" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:27" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A19" s="17" t="s">
         <v>6</v>
       </c>
@@ -12722,7 +12732,7 @@
         <v>2336</v>
       </c>
     </row>
-    <row r="26" spans="1:27" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:27" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A26" s="17" t="s">
         <v>6</v>
       </c>
@@ -12795,7 +12805,7 @@
       </c>
       <c r="AA26" s="17"/>
     </row>
-    <row r="27" spans="1:27" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:27" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A27" s="17" t="s">
         <v>6</v>
       </c>
@@ -12868,7 +12878,7 @@
       </c>
       <c r="AA27" s="17"/>
     </row>
-    <row r="28" spans="1:27" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:27" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A28" s="17" t="s">
         <v>6</v>
       </c>
@@ -13316,7 +13326,7 @@
       </c>
       <c r="AA33" s="17"/>
     </row>
-    <row r="34" spans="1:27" ht="232" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:27" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A34" s="17" t="s">
         <v>6</v>
       </c>
@@ -13464,7 +13474,7 @@
       </c>
       <c r="AA35" s="17"/>
     </row>
-    <row r="36" spans="1:27" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:27" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A36" s="17" t="s">
         <v>6</v>
       </c>
@@ -14056,7 +14066,7 @@
         <v>2339</v>
       </c>
     </row>
-    <row r="44" spans="1:27" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:27" ht="87" x14ac:dyDescent="0.35">
       <c r="A44" s="17" t="s">
         <v>6</v>
       </c>
@@ -14285,7 +14295,7 @@
       </c>
       <c r="AA46" s="17"/>
     </row>
-    <row r="47" spans="1:27" ht="87" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:27" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A47" s="17" t="s">
         <v>6</v>
       </c>
@@ -14508,7 +14518,7 @@
       </c>
       <c r="AA49" s="17"/>
     </row>
-    <row r="50" spans="1:27" ht="87" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:27" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A50" s="17" t="s">
         <v>6</v>
       </c>
@@ -14731,7 +14741,7 @@
       </c>
       <c r="AA52" s="17"/>
     </row>
-    <row r="53" spans="1:27" ht="372" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:27" ht="356.5" x14ac:dyDescent="0.35">
       <c r="A53" s="17" t="s">
         <v>6</v>
       </c>
@@ -14806,7 +14816,7 @@
       </c>
       <c r="AA53" s="17"/>
     </row>
-    <row r="54" spans="1:27" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:27" ht="87" x14ac:dyDescent="0.35">
       <c r="A54" s="17" t="s">
         <v>6</v>
       </c>
@@ -14881,7 +14891,7 @@
       </c>
       <c r="AA54" s="17"/>
     </row>
-    <row r="55" spans="1:27" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:27" ht="87" x14ac:dyDescent="0.35">
       <c r="A55" s="17" t="s">
         <v>6</v>
       </c>
@@ -14956,7 +14966,7 @@
       </c>
       <c r="AA55" s="17"/>
     </row>
-    <row r="56" spans="1:27" ht="87" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:27" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A56" s="17" t="s">
         <v>6</v>
       </c>
@@ -15029,7 +15039,7 @@
       </c>
       <c r="AA56" s="17"/>
     </row>
-    <row r="57" spans="1:27" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:27" ht="87" x14ac:dyDescent="0.35">
       <c r="A57" s="17" t="s">
         <v>6</v>
       </c>
@@ -15402,7 +15412,7 @@
       </c>
       <c r="AA61" s="17"/>
     </row>
-    <row r="62" spans="1:27" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:27" ht="87" x14ac:dyDescent="0.35">
       <c r="A62" s="17" t="s">
         <v>6</v>
       </c>
@@ -15769,7 +15779,7 @@
       </c>
       <c r="AA66" s="17"/>
     </row>
-    <row r="67" spans="1:27" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:27" ht="87" x14ac:dyDescent="0.35">
       <c r="A67" s="17" t="s">
         <v>6</v>
       </c>
@@ -16073,7 +16083,7 @@
         <v>2393</v>
       </c>
     </row>
-    <row r="71" spans="1:27" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:27" ht="87" x14ac:dyDescent="0.35">
       <c r="A71" s="17" t="s">
         <v>6</v>
       </c>
@@ -16150,7 +16160,7 @@
         <v>2240</v>
       </c>
     </row>
-    <row r="72" spans="1:27" ht="87" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:27" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A72" s="17" t="s">
         <v>6</v>
       </c>
@@ -16223,7 +16233,7 @@
       </c>
       <c r="AA72" s="17"/>
     </row>
-    <row r="73" spans="1:27" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:27" ht="87" x14ac:dyDescent="0.35">
       <c r="A73" s="17" t="s">
         <v>6</v>
       </c>
@@ -16298,7 +16308,7 @@
       </c>
       <c r="AA73" s="17"/>
     </row>
-    <row r="74" spans="1:27" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:27" ht="87" x14ac:dyDescent="0.35">
       <c r="A74" s="17" t="s">
         <v>6</v>
       </c>
@@ -16373,7 +16383,7 @@
       </c>
       <c r="AA74" s="17"/>
     </row>
-    <row r="75" spans="1:27" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:27" ht="87" x14ac:dyDescent="0.35">
       <c r="A75" s="17" t="s">
         <v>6</v>
       </c>
@@ -25810,7 +25820,7 @@
       </c>
       <c r="AA197" s="17"/>
     </row>
-    <row r="198" spans="1:27" ht="387.5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:27" ht="372" x14ac:dyDescent="0.35">
       <c r="A198" s="17" t="s">
         <v>6</v>
       </c>
@@ -25887,7 +25897,7 @@
       </c>
       <c r="AA198" s="17"/>
     </row>
-    <row r="199" spans="1:27" ht="387.5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:27" ht="372" x14ac:dyDescent="0.35">
       <c r="A199" s="17" t="s">
         <v>6</v>
       </c>
@@ -26570,7 +26580,7 @@
       </c>
       <c r="AA207" s="17"/>
     </row>
-    <row r="208" spans="1:27" ht="333.5" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:27" ht="348" x14ac:dyDescent="0.35">
       <c r="A208" s="17" t="s">
         <v>6</v>
       </c>
@@ -26601,7 +26611,7 @@
       <c r="J208" s="5" t="s">
         <v>2748</v>
       </c>
-      <c r="K208" s="17" t="s">
+      <c r="K208" s="71" t="s">
         <v>2750</v>
       </c>
       <c r="L208" s="5" t="s">
@@ -29799,7 +29809,7 @@
       </c>
       <c r="AA250" s="17"/>
     </row>
-    <row r="251" spans="1:27" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:27" ht="62" x14ac:dyDescent="0.35">
       <c r="A251" s="17" t="s">
         <v>6</v>
       </c>
@@ -31619,7 +31629,7 @@
       </c>
       <c r="AA274" s="17"/>
     </row>
-    <row r="275" spans="1:27" ht="232" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:27" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A275" s="17" t="s">
         <v>6</v>
       </c>
@@ -31771,7 +31781,7 @@
         <v>2336</v>
       </c>
     </row>
-    <row r="277" spans="1:27" ht="232" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:27" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A277" s="17" t="s">
         <v>6</v>
       </c>
@@ -31996,7 +32006,7 @@
       </c>
       <c r="AA279" s="17"/>
     </row>
-    <row r="280" spans="1:27" ht="232" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:27" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A280" s="17" t="s">
         <v>6</v>
       </c>
@@ -32071,7 +32081,7 @@
       </c>
       <c r="AA280" s="17"/>
     </row>
-    <row r="281" spans="1:27" ht="232" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:27" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A281" s="17" t="s">
         <v>6</v>
       </c>
@@ -32146,7 +32156,7 @@
       </c>
       <c r="AA281" s="17"/>
     </row>
-    <row r="282" spans="1:27" ht="232" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:27" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A282" s="17" t="s">
         <v>6</v>
       </c>
@@ -32221,7 +32231,7 @@
       </c>
       <c r="AA282" s="17"/>
     </row>
-    <row r="283" spans="1:27" ht="232" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:27" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A283" s="17" t="s">
         <v>6</v>
       </c>
@@ -32296,7 +32306,7 @@
       </c>
       <c r="AA283" s="17"/>
     </row>
-    <row r="284" spans="1:27" ht="232" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:27" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A284" s="17" t="s">
         <v>6</v>
       </c>
@@ -32371,7 +32381,7 @@
       </c>
       <c r="AA284" s="17"/>
     </row>
-    <row r="285" spans="1:27" ht="232" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:27" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A285" s="17" t="s">
         <v>6</v>
       </c>
@@ -33342,7 +33352,7 @@
       </c>
       <c r="AA297" s="17"/>
     </row>
-    <row r="298" spans="1:27" ht="232" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:27" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A298" s="17" t="s">
         <v>6</v>
       </c>
@@ -33865,7 +33875,7 @@
         <v>2360</v>
       </c>
     </row>
-    <row r="305" spans="1:27" ht="319" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:27" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A305" s="17" t="s">
         <v>6</v>
       </c>
@@ -33942,7 +33952,7 @@
       </c>
       <c r="AA305" s="17"/>
     </row>
-    <row r="306" spans="1:27" ht="319" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:27" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A306" s="17" t="s">
         <v>6</v>
       </c>
@@ -34021,7 +34031,7 @@
       </c>
       <c r="AA306" s="17"/>
     </row>
-    <row r="307" spans="1:27" ht="319" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:27" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A307" s="17" t="s">
         <v>6</v>
       </c>
@@ -34100,7 +34110,7 @@
       </c>
       <c r="AA307" s="17"/>
     </row>
-    <row r="308" spans="1:27" ht="319" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:27" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A308" s="17" t="s">
         <v>6</v>
       </c>
@@ -34177,7 +34187,7 @@
       </c>
       <c r="AA308" s="17"/>
     </row>
-    <row r="309" spans="1:27" ht="319" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:27" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A309" s="17" t="s">
         <v>6</v>
       </c>
@@ -34250,7 +34260,7 @@
       </c>
       <c r="AA309" s="17"/>
     </row>
-    <row r="310" spans="1:27" ht="319" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:27" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A310" s="17" t="s">
         <v>6</v>
       </c>
@@ -34629,7 +34639,7 @@
       </c>
       <c r="AA314" s="17"/>
     </row>
-    <row r="315" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A315" s="17" t="s">
         <v>6</v>
       </c>
@@ -35154,7 +35164,7 @@
         <v>2341</v>
       </c>
     </row>
-    <row r="322" spans="1:27" ht="319" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:27" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A322" s="17" t="s">
         <v>6</v>
       </c>
@@ -35231,7 +35241,7 @@
       </c>
       <c r="AA322" s="17"/>
     </row>
-    <row r="323" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A323" s="17" t="s">
         <v>6</v>
       </c>
@@ -35308,7 +35318,7 @@
       </c>
       <c r="AA323" s="17"/>
     </row>
-    <row r="324" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A324" s="17" t="s">
         <v>6</v>
       </c>
@@ -35387,7 +35397,7 @@
         <v>2453</v>
       </c>
     </row>
-    <row r="325" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A325" s="17" t="s">
         <v>6</v>
       </c>
@@ -35462,7 +35472,7 @@
       </c>
       <c r="AA325" s="17"/>
     </row>
-    <row r="326" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A326" s="17" t="s">
         <v>6</v>
       </c>
@@ -35614,7 +35624,7 @@
         <v>2405</v>
       </c>
     </row>
-    <row r="328" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A328" s="17" t="s">
         <v>6</v>
       </c>
@@ -35691,7 +35701,7 @@
       </c>
       <c r="AA328" s="17"/>
     </row>
-    <row r="329" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A329" s="17" t="s">
         <v>6</v>
       </c>
@@ -35766,7 +35776,7 @@
       </c>
       <c r="AA329" s="17"/>
     </row>
-    <row r="330" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A330" s="17" t="s">
         <v>6</v>
       </c>
@@ -35841,7 +35851,7 @@
       </c>
       <c r="AA330" s="17"/>
     </row>
-    <row r="331" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:27" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A331" s="17" t="s">
         <v>6</v>
       </c>
@@ -35920,7 +35930,7 @@
         <v>2309</v>
       </c>
     </row>
-    <row r="332" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:27" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A332" s="17" t="s">
         <v>6</v>
       </c>
@@ -35995,7 +36005,7 @@
       </c>
       <c r="AA332" s="17"/>
     </row>
-    <row r="333" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:27" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A333" s="17" t="s">
         <v>6</v>
       </c>
@@ -36374,7 +36384,7 @@
       </c>
       <c r="AA337" s="17"/>
     </row>
-    <row r="338" spans="1:27" ht="319" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:27" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A338" s="17" t="s">
         <v>6</v>
       </c>
@@ -36451,7 +36461,7 @@
         <v>2328</v>
       </c>
     </row>
-    <row r="339" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A339" s="17" t="s">
         <v>6</v>
       </c>
@@ -36526,7 +36536,7 @@
       </c>
       <c r="AA339" s="17"/>
     </row>
-    <row r="340" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A340" s="17" t="s">
         <v>6</v>
       </c>
@@ -36753,7 +36763,7 @@
         <v>2325</v>
       </c>
     </row>
-    <row r="343" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A343" s="17" t="s">
         <v>6</v>
       </c>
@@ -36828,7 +36838,7 @@
       </c>
       <c r="AA343" s="17"/>
     </row>
-    <row r="344" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:27" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A344" s="17" t="s">
         <v>6</v>
       </c>
@@ -36903,7 +36913,7 @@
       </c>
       <c r="AA344" s="17"/>
     </row>
-    <row r="345" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A345" s="17" t="s">
         <v>6</v>
       </c>
@@ -37053,7 +37063,7 @@
       </c>
       <c r="AA346" s="17"/>
     </row>
-    <row r="347" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A347" s="17" t="s">
         <v>6</v>
       </c>
@@ -37201,7 +37211,7 @@
       </c>
       <c r="AA348" s="17"/>
     </row>
-    <row r="349" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:27" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A349" s="17" t="s">
         <v>6</v>
       </c>
@@ -37355,7 +37365,7 @@
         <v>2327</v>
       </c>
     </row>
-    <row r="351" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A351" s="17" t="s">
         <v>6</v>
       </c>
@@ -37507,7 +37517,7 @@
       </c>
       <c r="AA352" s="17"/>
     </row>
-    <row r="353" spans="1:27" ht="333.5" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:27" ht="348" x14ac:dyDescent="0.35">
       <c r="A353" s="17" t="s">
         <v>6</v>
       </c>
@@ -37584,7 +37594,7 @@
         <v>2243</v>
       </c>
     </row>
-    <row r="354" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A354" s="17" t="s">
         <v>6</v>
       </c>
@@ -37811,7 +37821,7 @@
         <v>2392</v>
       </c>
     </row>
-    <row r="357" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:27" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A357" s="17" t="s">
         <v>6</v>
       </c>
@@ -38561,7 +38571,7 @@
       </c>
       <c r="AA366" s="17"/>
     </row>
-    <row r="367" spans="1:27" ht="319" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:27" ht="333.5" x14ac:dyDescent="0.35">
       <c r="A367" s="17" t="s">
         <v>6</v>
       </c>
@@ -38792,7 +38802,7 @@
         <v>2387</v>
       </c>
     </row>
-    <row r="370" spans="1:27" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:27" ht="87" x14ac:dyDescent="0.35">
       <c r="A370" s="17" t="s">
         <v>6</v>
       </c>
@@ -40799,7 +40809,7 @@
       </c>
       <c r="AA396" s="17"/>
     </row>
-    <row r="397" spans="1:27" ht="232" x14ac:dyDescent="0.35">
+    <row r="397" spans="1:27" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A397" s="17" t="s">
         <v>6</v>
       </c>
@@ -41024,7 +41034,7 @@
         <v>2277</v>
       </c>
     </row>
-    <row r="400" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="400" spans="1:27" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A400" s="17" t="s">
         <v>6</v>
       </c>
@@ -41308,7 +41318,7 @@
       </c>
       <c r="AA403" s="17"/>
     </row>
-    <row r="404" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="404" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A404" s="17" t="s">
         <v>6</v>
       </c>
@@ -41381,7 +41391,7 @@
       <c r="Z404" s="17"/>
       <c r="AA404" s="17"/>
     </row>
-    <row r="405" spans="1:27" ht="319" x14ac:dyDescent="0.35">
+    <row r="405" spans="1:27" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A405" s="17" t="s">
         <v>6</v>
       </c>
@@ -41813,7 +41823,7 @@
       <c r="Z410" s="17"/>
       <c r="AA410" s="17"/>
     </row>
-    <row r="411" spans="1:27" ht="319" x14ac:dyDescent="0.35">
+    <row r="411" spans="1:27" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A411" s="17" t="s">
         <v>6</v>
       </c>
@@ -41886,7 +41896,7 @@
       <c r="Z411" s="17"/>
       <c r="AA411" s="17"/>
     </row>
-    <row r="412" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="412" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A412" s="17" t="s">
         <v>6</v>
       </c>
@@ -42168,7 +42178,7 @@
       <c r="Z415" s="17"/>
       <c r="AA415" s="17"/>
     </row>
-    <row r="416" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="416" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A416" s="17" t="s">
         <v>6</v>
       </c>
@@ -42379,7 +42389,7 @@
       <c r="Z418" s="17"/>
       <c r="AA418" s="17"/>
     </row>
-    <row r="419" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="419" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A419" s="17" t="s">
         <v>6</v>
       </c>
@@ -42452,7 +42462,7 @@
       <c r="Z419" s="17"/>
       <c r="AA419" s="17"/>
     </row>
-    <row r="420" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="420" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A420" s="17" t="s">
         <v>6</v>
       </c>
@@ -43081,7 +43091,7 @@
       <c r="Z428" s="17"/>
       <c r="AA428" s="17"/>
     </row>
-    <row r="429" spans="1:27" ht="87" x14ac:dyDescent="0.35">
+    <row r="429" spans="1:27" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A429" s="17" t="s">
         <v>6</v>
       </c>
@@ -43148,7 +43158,7 @@
       <c r="Z429" s="17"/>
       <c r="AA429" s="17"/>
     </row>
-    <row r="430" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="430" spans="1:27" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A430" s="17" t="s">
         <v>6</v>
       </c>
@@ -43576,7 +43586,7 @@
       <c r="Z435" s="17"/>
       <c r="AA435" s="17"/>
     </row>
-    <row r="436" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="436" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A436" s="17" t="s">
         <v>6</v>
       </c>
@@ -43643,7 +43653,7 @@
       <c r="Z436" s="17"/>
       <c r="AA436" s="17"/>
     </row>
-    <row r="437" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="437" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A437" s="17" t="s">
         <v>6</v>
       </c>
@@ -43921,7 +43931,7 @@
       <c r="Z440" s="22"/>
       <c r="AA440" s="17"/>
     </row>
-    <row r="441" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="441" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A441" s="17" t="s">
         <v>6</v>
       </c>
@@ -43992,7 +44002,7 @@
       <c r="Z441" s="17"/>
       <c r="AA441" s="17"/>
     </row>
-    <row r="442" spans="1:27" ht="319" x14ac:dyDescent="0.35">
+    <row r="442" spans="1:27" ht="348" x14ac:dyDescent="0.35">
       <c r="A442" s="17" t="s">
         <v>6</v>
       </c>
@@ -44061,7 +44071,7 @@
       <c r="Z442" s="17"/>
       <c r="AA442" s="17"/>
     </row>
-    <row r="443" spans="1:27" ht="319" x14ac:dyDescent="0.35">
+    <row r="443" spans="1:27" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A443" s="17" t="s">
         <v>6</v>
       </c>
@@ -45465,7 +45475,7 @@
       <c r="Z462" s="17"/>
       <c r="AA462" s="17"/>
     </row>
-    <row r="463" spans="1:27" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="463" spans="1:27" ht="87" x14ac:dyDescent="0.35">
       <c r="A463" s="39" t="s">
         <v>6</v>
       </c>
@@ -45536,7 +45546,7 @@
       <c r="Z463" s="17"/>
       <c r="AA463" s="17"/>
     </row>
-    <row r="464" spans="1:27" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="464" spans="1:27" ht="87" x14ac:dyDescent="0.35">
       <c r="A464" s="39" t="s">
         <v>6</v>
       </c>
@@ -46627,7 +46637,7 @@
       <c r="Z478" s="17"/>
       <c r="AA478" s="17"/>
     </row>
-    <row r="479" spans="1:27" ht="58" x14ac:dyDescent="0.35">
+    <row r="479" spans="1:27" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A479" s="42" t="s">
         <v>6</v>
       </c>
@@ -48977,7 +48987,7 @@
       <c r="Z514" s="17"/>
       <c r="AA514" s="17"/>
     </row>
-    <row r="515" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="515" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A515" s="49" t="s">
         <v>6</v>
       </c>
@@ -49119,7 +49129,7 @@
         <v>2339</v>
       </c>
     </row>
-    <row r="517" spans="1:27" ht="87" x14ac:dyDescent="0.35">
+    <row r="517" spans="1:27" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A517" s="17" t="s">
         <v>6</v>
       </c>
@@ -49600,7 +49610,7 @@
       <c r="Z523" s="17"/>
       <c r="AA523" s="17"/>
     </row>
-    <row r="524" spans="1:27" ht="217.5" x14ac:dyDescent="0.35">
+    <row r="524" spans="1:27" ht="232" x14ac:dyDescent="0.35">
       <c r="A524" s="49" t="s">
         <v>6</v>
       </c>
@@ -50034,10 +50044,10 @@
       <c r="M530" s="5" t="s">
         <v>2609</v>
       </c>
-      <c r="N530" s="5" t="s">
+      <c r="N530" s="5"/>
+      <c r="O530" s="5" t="s">
         <v>3191</v>
       </c>
-      <c r="O530" s="17"/>
       <c r="P530" s="17" t="s">
         <v>3189</v>
       </c>
@@ -50132,7 +50142,7 @@
       <c r="Z531" s="17"/>
       <c r="AA531" s="17"/>
     </row>
-    <row r="532" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="532" spans="1:27" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A532" s="49" t="s">
         <v>6</v>
       </c>
@@ -50199,7 +50209,7 @@
       <c r="Z532" s="17"/>
       <c r="AA532" s="17"/>
     </row>
-    <row r="533" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="533" spans="1:27" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A533" s="49" t="s">
         <v>6</v>
       </c>
@@ -50264,7 +50274,7 @@
       <c r="Z533" s="17"/>
       <c r="AA533" s="17"/>
     </row>
-    <row r="534" spans="1:27" ht="319" x14ac:dyDescent="0.35">
+    <row r="534" spans="1:27" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A534" s="49" t="s">
         <v>6</v>
       </c>
@@ -50329,7 +50339,7 @@
       <c r="Z534" s="17"/>
       <c r="AA534" s="17"/>
     </row>
-    <row r="535" spans="1:27" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="535" spans="1:27" ht="174" x14ac:dyDescent="0.35">
       <c r="A535" s="49" t="s">
         <v>6</v>
       </c>
@@ -50396,7 +50406,7 @@
       <c r="Z535" s="17"/>
       <c r="AA535" s="17"/>
     </row>
-    <row r="536" spans="1:27" ht="201.5" x14ac:dyDescent="0.35">
+    <row r="536" spans="1:27" ht="217" x14ac:dyDescent="0.35">
       <c r="A536" s="49" t="s">
         <v>6</v>
       </c>
@@ -50533,7 +50543,7 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Q222">
     <sortCondition ref="C2:C417"/>
   </sortState>
-  <phoneticPr fontId="13" type="noConversion"/>
+  <phoneticPr fontId="14" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{A888D081-6FD4-4DBA-B75D-11B8EF20FB9F}"/>
     <hyperlink ref="D4" r:id="rId2" xr:uid="{84186489-15CD-48F0-BE91-0362E1A8C1AB}"/>

</xml_diff>